<commit_message>
update template + timesheet
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -5,16 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Library/Mobile Documents/com~apple~CloudDocs/evidence/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7ADF8BFD-B7E4-834F-81AD-0825526168F1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CB769D9-9EBA-B34E-898E-FDFF02787269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="15960" windowHeight="18080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="36020" windowHeight="24580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="evid.PD" sheetId="1" r:id="rId1"/>
-    <sheet name="Nastaveni" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -56,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="70">
   <si>
     <t>EVIDENCE PRACOVNÍ DOBY</t>
   </si>
@@ -266,149 +265,17 @@
   </si>
   <si>
     <t xml:space="preserve">         Podpis zaměstnance </t>
-  </si>
-  <si>
-    <t>Datum</t>
-  </si>
-  <si>
-    <t>Mesic</t>
-  </si>
-  <si>
-    <t>Rok</t>
-  </si>
-  <si>
-    <t>Svatky</t>
-  </si>
-  <si>
-    <t>Nazev</t>
-  </si>
-  <si>
-    <t>Nový rok</t>
-  </si>
-  <si>
-    <t>1.1.</t>
-  </si>
-  <si>
-    <t>Velky patek</t>
-  </si>
-  <si>
-    <t>1.4.</t>
-  </si>
-  <si>
-    <t>Velikonocni pondeli</t>
-  </si>
-  <si>
-    <t>21.4.</t>
-  </si>
-  <si>
-    <t>Svatek prace</t>
-  </si>
-  <si>
-    <t>1.5.</t>
-  </si>
-  <si>
-    <t>Den vitezstvi</t>
-  </si>
-  <si>
-    <t>8.5.</t>
-  </si>
-  <si>
-    <t>Cyril, Metodej</t>
-  </si>
-  <si>
-    <t>5.7.</t>
-  </si>
-  <si>
-    <t>Jan Hus</t>
-  </si>
-  <si>
-    <t>6.7.</t>
-  </si>
-  <si>
-    <t>Ceska statnost</t>
-  </si>
-  <si>
-    <t>28.9.</t>
-  </si>
-  <si>
-    <t>Vznik ceskoslovenskeho statu</t>
-  </si>
-  <si>
-    <t>28.10.</t>
-  </si>
-  <si>
-    <t>Den boje za svobodu</t>
-  </si>
-  <si>
-    <t>17.11.</t>
-  </si>
-  <si>
-    <t>Stedry den</t>
-  </si>
-  <si>
-    <t>24.12.</t>
-  </si>
-  <si>
-    <t>Vanocni svatek</t>
-  </si>
-  <si>
-    <t>25.12.</t>
-  </si>
-  <si>
-    <t>2. Vanocni svatek</t>
-  </si>
-  <si>
-    <t>26.12.</t>
-  </si>
-  <si>
-    <t>Pracovní dny</t>
-  </si>
-  <si>
-    <t>Zacatek mesice</t>
-  </si>
-  <si>
-    <t>Konec měsíce</t>
-  </si>
-  <si>
-    <t>Pracovní dny bez svatku</t>
-  </si>
-  <si>
-    <t>Dovolená</t>
-  </si>
-  <si>
-    <t>DOVOLENA</t>
-  </si>
-  <si>
-    <t>Prepocitano</t>
-  </si>
-  <si>
-    <t>Odpracovane hodiny</t>
-  </si>
-  <si>
-    <t>Zacatek</t>
-  </si>
-  <si>
-    <t>Konec</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
-  </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color indexed="8"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -474,7 +341,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -487,20 +354,8 @@
         <bgColor auto="1"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="12"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="15"/>
-        <bgColor auto="1"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="80">
+  <borders count="81">
     <border>
       <left/>
       <right/>
@@ -1488,106 +1343,109 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="13"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="14"/>
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="13"/>
-      </left>
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="13"/>
+        <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="14"/>
+        <color indexed="8"/>
       </left>
       <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="14"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="13"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color indexed="14"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
+        <color indexed="9"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="14"/>
+        <color indexed="9"/>
       </left>
       <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="13"/>
-      </left>
-      <right style="thin">
-        <color indexed="13"/>
-      </right>
-      <top style="thin">
-        <color indexed="13"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="13"/>
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1595,55 +1453,55 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="194">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -1693,9 +1551,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1707,9 +1563,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1717,53 +1572,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1771,52 +1626,52 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
@@ -1827,11 +1682,11 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1840,7 +1695,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1855,95 +1710,108 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="67" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="67" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="73" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="75" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="76" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="74" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="77" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="76" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="77" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="74" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="20" fontId="0" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="75" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -3154,9 +3022,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="176"/>
-      <c r="C1" s="177"/>
-      <c r="D1" s="177"/>
+      <c r="B1" s="166"/>
+      <c r="C1" s="167"/>
+      <c r="D1" s="167"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3170,55 +3038,52 @@
       <c r="M1" s="2"/>
       <c r="N1" s="2"/>
       <c r="O1" s="2"/>
-      <c r="P1" s="4" cm="1">
-        <f t="array" ref="P1">12</f>
-        <v>12</v>
-      </c>
+      <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="182" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="177"/>
-      <c r="C2" s="177"/>
-      <c r="D2" s="177"/>
-      <c r="E2" s="177"/>
-      <c r="F2" s="177"/>
-      <c r="G2" s="177"/>
+      <c r="B2" s="167"/>
+      <c r="C2" s="167"/>
+      <c r="D2" s="167"/>
+      <c r="E2" s="167"/>
+      <c r="F2" s="167"/>
+      <c r="G2" s="167"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="189" t="s">
+      <c r="L2" s="181" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="177"/>
+      <c r="M2" s="167"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="178" t="s">
+      <c r="A3" s="168" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="179"/>
-      <c r="C3" s="179"/>
-      <c r="D3" s="179"/>
+      <c r="B3" s="169"/>
+      <c r="C3" s="169"/>
+      <c r="D3" s="169"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="190" t="s">
+      <c r="F3" s="183" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="179"/>
-      <c r="H3" s="179"/>
-      <c r="I3" s="179"/>
+      <c r="G3" s="169"/>
+      <c r="H3" s="169"/>
+      <c r="I3" s="169"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="179" t="str" cm="1">
+      <c r="L3" s="169" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="179"/>
-      <c r="N3" s="179"/>
+      <c r="M3" s="169"/>
+      <c r="N3" s="169"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3226,11 +3091,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="174" t="s">
+      <c r="B4" s="164" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="175"/>
-      <c r="D4" s="175"/>
+      <c r="C4" s="165"/>
+      <c r="D4" s="165"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3262,12 +3127,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="170"/>
-      <c r="C5" s="171"/>
-      <c r="D5" s="171"/>
-      <c r="E5" s="180"/>
-      <c r="F5" s="171"/>
-      <c r="G5" s="171"/>
+      <c r="B5" s="160"/>
+      <c r="C5" s="161"/>
+      <c r="D5" s="161"/>
+      <c r="E5" s="170"/>
+      <c r="F5" s="161"/>
+      <c r="G5" s="161"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3294,12 +3159,12 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="171"/>
-      <c r="C6" s="171"/>
-      <c r="D6" s="171"/>
-      <c r="E6" s="171"/>
-      <c r="F6" s="171"/>
-      <c r="G6" s="171"/>
+      <c r="B6" s="161"/>
+      <c r="C6" s="161"/>
+      <c r="D6" s="161"/>
+      <c r="E6" s="161"/>
+      <c r="F6" s="161"/>
+      <c r="G6" s="161"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
@@ -3318,11 +3183,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="30"/>
-      <c r="B7" s="172" t="s">
+      <c r="B7" s="162" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="173"/>
-      <c r="D7" s="173"/>
+      <c r="C7" s="163"/>
+      <c r="D7" s="163"/>
       <c r="E7" s="32"/>
       <c r="F7" s="31" t="s">
         <v>22</v>
@@ -3357,7 +3222,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="39"/>
-      <c r="C8" s="193" t="s">
+      <c r="C8" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="40"/>
@@ -3381,8 +3246,8 @@
       <c r="K8" s="47"/>
       <c r="L8" s="48"/>
       <c r="M8" s="49"/>
-      <c r="N8" s="181"/>
-      <c r="O8" s="182"/>
+      <c r="N8" s="171"/>
+      <c r="O8" s="172"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3390,19 +3255,23 @@
         <v>2</v>
       </c>
       <c r="B9" s="50"/>
-      <c r="C9" s="193" t="s">
+      <c r="C9" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="40"/>
-      <c r="E9" s="41"/>
+      <c r="E9" s="41" t="str" cm="1">
+        <f t="array" ref="E9">IF(ISBLANK(D9),"","12.00")</f>
+        <v/>
+      </c>
       <c r="F9" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="43"/>
+      <c r="G9" s="43" t="str" cm="1">
+        <f t="array" ref="G9">IF(ISBLANK(D9),"","12.30")</f>
+        <v/>
+      </c>
       <c r="H9" s="49"/>
-      <c r="I9" s="51">
-        <v>8</v>
-      </c>
+      <c r="I9" s="51"/>
       <c r="J9" s="5" t="str" cm="1">
         <f t="array" ref="J9">IF(AND(ISNUMBER(H9),NOT(ISERROR(H9&gt;8)),H9&gt;8),H9-8,"")</f>
         <v/>
@@ -3410,8 +3279,8 @@
       <c r="K9" s="52"/>
       <c r="L9" s="48"/>
       <c r="M9" s="49"/>
-      <c r="N9" s="181"/>
-      <c r="O9" s="182"/>
+      <c r="N9" s="171"/>
+      <c r="O9" s="172"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3419,7 +3288,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="39"/>
-      <c r="C10" s="193" t="s">
+      <c r="C10" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="40"/>
@@ -3443,8 +3312,8 @@
       <c r="K10" s="52"/>
       <c r="L10" s="48"/>
       <c r="M10" s="49"/>
-      <c r="N10" s="181"/>
-      <c r="O10" s="182"/>
+      <c r="N10" s="171"/>
+      <c r="O10" s="172"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3452,7 +3321,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="39"/>
-      <c r="C11" s="193" t="s">
+      <c r="C11" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D11" s="40"/>
@@ -3476,8 +3345,8 @@
       <c r="K11" s="52"/>
       <c r="L11" s="48"/>
       <c r="M11" s="49"/>
-      <c r="N11" s="181"/>
-      <c r="O11" s="182"/>
+      <c r="N11" s="171"/>
+      <c r="O11" s="172"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3485,7 +3354,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="39"/>
-      <c r="C12" s="193" t="s">
+      <c r="C12" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="40"/>
@@ -3508,9 +3377,9 @@
       </c>
       <c r="K12" s="52"/>
       <c r="L12" s="48"/>
-      <c r="M12" s="49"/>
-      <c r="N12" s="181"/>
-      <c r="O12" s="182"/>
+      <c r="M12" s="156"/>
+      <c r="N12" s="173"/>
+      <c r="O12" s="174"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3518,7 +3387,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="39"/>
-      <c r="C13" s="193" t="s">
+      <c r="C13" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D13" s="40"/>
@@ -3540,18 +3409,18 @@
         <v/>
       </c>
       <c r="K13" s="52"/>
-      <c r="L13" s="55"/>
-      <c r="M13" s="56"/>
-      <c r="N13" s="191"/>
-      <c r="O13" s="191"/>
-      <c r="P13" s="2"/>
+      <c r="L13" s="158"/>
+      <c r="M13" s="159"/>
+      <c r="N13" s="184"/>
+      <c r="O13" s="185"/>
+      <c r="P13" s="69"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="38">
         <v>7</v>
       </c>
       <c r="B14" s="39"/>
-      <c r="C14" s="193" t="s">
+      <c r="C14" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="40"/>
@@ -3574,9 +3443,9 @@
       </c>
       <c r="K14" s="52"/>
       <c r="L14" s="48"/>
-      <c r="M14" s="49"/>
-      <c r="N14" s="181"/>
-      <c r="O14" s="182"/>
+      <c r="M14" s="157"/>
+      <c r="N14" s="186"/>
+      <c r="O14" s="187"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3584,7 +3453,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="39"/>
-      <c r="C15" s="193" t="s">
+      <c r="C15" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D15" s="40"/>
@@ -3608,8 +3477,8 @@
       <c r="K15" s="52"/>
       <c r="L15" s="48"/>
       <c r="M15" s="49"/>
-      <c r="N15" s="181"/>
-      <c r="O15" s="182"/>
+      <c r="N15" s="171"/>
+      <c r="O15" s="172"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3617,7 +3486,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="39"/>
-      <c r="C16" s="193" t="s">
+      <c r="C16" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="40"/>
@@ -3641,8 +3510,8 @@
       <c r="K16" s="52"/>
       <c r="L16" s="48"/>
       <c r="M16" s="49"/>
-      <c r="N16" s="181"/>
-      <c r="O16" s="182"/>
+      <c r="N16" s="171"/>
+      <c r="O16" s="172"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3650,7 +3519,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="39"/>
-      <c r="C17" s="193" t="s">
+      <c r="C17" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="40"/>
@@ -3674,8 +3543,8 @@
       <c r="K17" s="52"/>
       <c r="L17" s="48"/>
       <c r="M17" s="49"/>
-      <c r="N17" s="181"/>
-      <c r="O17" s="182"/>
+      <c r="N17" s="171"/>
+      <c r="O17" s="172"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3683,7 +3552,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="39"/>
-      <c r="C18" s="193" t="s">
+      <c r="C18" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D18" s="40"/>
@@ -3707,8 +3576,8 @@
       <c r="K18" s="52"/>
       <c r="L18" s="48"/>
       <c r="M18" s="49"/>
-      <c r="N18" s="181"/>
-      <c r="O18" s="182"/>
+      <c r="N18" s="171"/>
+      <c r="O18" s="172"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3716,7 +3585,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="39"/>
-      <c r="C19" s="193" t="s">
+      <c r="C19" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="40"/>
@@ -3740,8 +3609,8 @@
       <c r="K19" s="52"/>
       <c r="L19" s="48"/>
       <c r="M19" s="49"/>
-      <c r="N19" s="181"/>
-      <c r="O19" s="182"/>
+      <c r="N19" s="171"/>
+      <c r="O19" s="172"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3749,7 +3618,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="39"/>
-      <c r="C20" s="193" t="s">
+      <c r="C20" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="40"/>
@@ -3765,7 +3634,7 @@
         <v/>
       </c>
       <c r="H20" s="49"/>
-      <c r="I20" s="57"/>
+      <c r="I20" s="55"/>
       <c r="J20" s="5" t="str" cm="1">
         <f t="array" ref="J20">IF(AND(ISNUMBER(H20),NOT(ISERROR(H20&gt;8)),H20&gt;8),H20-8,"")</f>
         <v/>
@@ -3773,8 +3642,8 @@
       <c r="K20" s="52"/>
       <c r="L20" s="48"/>
       <c r="M20" s="49"/>
-      <c r="N20" s="181"/>
-      <c r="O20" s="182"/>
+      <c r="N20" s="171"/>
+      <c r="O20" s="172"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3782,15 +3651,21 @@
         <v>14</v>
       </c>
       <c r="B21" s="39"/>
-      <c r="C21" s="193" t="s">
+      <c r="C21" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="40"/>
-      <c r="E21" s="41"/>
+      <c r="E21" s="41" t="str" cm="1">
+        <f t="array" ref="E21">IF(ISBLANK(D21),"","12.00")</f>
+        <v/>
+      </c>
       <c r="F21" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="43"/>
+      <c r="G21" s="43" t="str" cm="1">
+        <f t="array" ref="G21">IF(ISBLANK(D21),"","12.30")</f>
+        <v/>
+      </c>
       <c r="H21" s="49"/>
       <c r="I21" s="53"/>
       <c r="J21" s="5" t="str" cm="1">
@@ -3800,8 +3675,8 @@
       <c r="K21" s="52"/>
       <c r="L21" s="48"/>
       <c r="M21" s="49"/>
-      <c r="N21" s="181"/>
-      <c r="O21" s="182"/>
+      <c r="N21" s="171"/>
+      <c r="O21" s="172"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3809,7 +3684,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="39"/>
-      <c r="C22" s="193" t="s">
+      <c r="C22" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D22" s="40"/>
@@ -3833,8 +3708,8 @@
       <c r="K22" s="52"/>
       <c r="L22" s="48"/>
       <c r="M22" s="49"/>
-      <c r="N22" s="181"/>
-      <c r="O22" s="182"/>
+      <c r="N22" s="171"/>
+      <c r="O22" s="172"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3842,7 +3717,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="39"/>
-      <c r="C23" s="193" t="s">
+      <c r="C23" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D23" s="40"/>
@@ -3866,8 +3741,8 @@
       <c r="K23" s="52"/>
       <c r="L23" s="48"/>
       <c r="M23" s="49"/>
-      <c r="N23" s="181"/>
-      <c r="O23" s="182"/>
+      <c r="N23" s="171"/>
+      <c r="O23" s="172"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3875,7 +3750,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="39"/>
-      <c r="C24" s="193" t="s">
+      <c r="C24" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="40"/>
@@ -3899,8 +3774,8 @@
       <c r="K24" s="52"/>
       <c r="L24" s="48"/>
       <c r="M24" s="49"/>
-      <c r="N24" s="181"/>
-      <c r="O24" s="182"/>
+      <c r="N24" s="171"/>
+      <c r="O24" s="172"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3908,7 +3783,7 @@
         <v>18</v>
       </c>
       <c r="B25" s="39"/>
-      <c r="C25" s="193" t="s">
+      <c r="C25" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="40"/>
@@ -3932,8 +3807,8 @@
       <c r="K25" s="52"/>
       <c r="L25" s="48"/>
       <c r="M25" s="49"/>
-      <c r="N25" s="181"/>
-      <c r="O25" s="182"/>
+      <c r="N25" s="171"/>
+      <c r="O25" s="172"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3941,7 +3816,7 @@
         <v>19</v>
       </c>
       <c r="B26" s="39"/>
-      <c r="C26" s="193" t="s">
+      <c r="C26" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="40"/>
@@ -3965,8 +3840,8 @@
       <c r="K26" s="52"/>
       <c r="L26" s="48"/>
       <c r="M26" s="49"/>
-      <c r="N26" s="181"/>
-      <c r="O26" s="182"/>
+      <c r="N26" s="171"/>
+      <c r="O26" s="172"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3974,7 +3849,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="39"/>
-      <c r="C27" s="193" t="s">
+      <c r="C27" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="40"/>
@@ -3998,8 +3873,8 @@
       <c r="K27" s="52"/>
       <c r="L27" s="48"/>
       <c r="M27" s="49"/>
-      <c r="N27" s="181"/>
-      <c r="O27" s="182"/>
+      <c r="N27" s="171"/>
+      <c r="O27" s="172"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4007,15 +3882,21 @@
         <v>21</v>
       </c>
       <c r="B28" s="39"/>
-      <c r="C28" s="193" t="s">
+      <c r="C28" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D28" s="40"/>
-      <c r="E28" s="41"/>
+      <c r="E28" s="41" t="str" cm="1">
+        <f t="array" ref="E28">IF(ISBLANK(D28),"","12.00")</f>
+        <v/>
+      </c>
       <c r="F28" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="43"/>
+      <c r="G28" s="43" t="str" cm="1">
+        <f t="array" ref="G28">IF(ISBLANK(D28),"","12.30")</f>
+        <v/>
+      </c>
       <c r="H28" s="49"/>
       <c r="I28" s="53"/>
       <c r="J28" s="5" t="str" cm="1">
@@ -4025,8 +3906,8 @@
       <c r="K28" s="52"/>
       <c r="L28" s="48"/>
       <c r="M28" s="49"/>
-      <c r="N28" s="181"/>
-      <c r="O28" s="182"/>
+      <c r="N28" s="171"/>
+      <c r="O28" s="172"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4034,7 +3915,7 @@
         <v>22</v>
       </c>
       <c r="B29" s="50"/>
-      <c r="C29" s="193" t="s">
+      <c r="C29" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="40"/>
@@ -4050,9 +3931,7 @@
         <v/>
       </c>
       <c r="H29" s="49"/>
-      <c r="I29" s="51">
-        <v>8</v>
-      </c>
+      <c r="I29" s="51"/>
       <c r="J29" s="5" t="str" cm="1">
         <f t="array" ref="J29">IF(AND(ISNUMBER(H29),NOT(ISERROR(H29&gt;8)),H29&gt;8),H29-8,"")</f>
         <v/>
@@ -4060,8 +3939,8 @@
       <c r="K29" s="52"/>
       <c r="L29" s="48"/>
       <c r="M29" s="49"/>
-      <c r="N29" s="181"/>
-      <c r="O29" s="182"/>
+      <c r="N29" s="171"/>
+      <c r="O29" s="172"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4069,7 +3948,7 @@
         <v>23</v>
       </c>
       <c r="B30" s="50"/>
-      <c r="C30" s="193" t="s">
+      <c r="C30" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D30" s="40"/>
@@ -4085,9 +3964,7 @@
         <v/>
       </c>
       <c r="H30" s="49"/>
-      <c r="I30" s="51">
-        <v>8</v>
-      </c>
+      <c r="I30" s="51"/>
       <c r="J30" s="5" t="str" cm="1">
         <f t="array" ref="J30">IF(AND(ISNUMBER(H30),NOT(ISERROR(H30&gt;8)),H30&gt;8),H30-8,"")</f>
         <v/>
@@ -4095,8 +3972,8 @@
       <c r="K30" s="52"/>
       <c r="L30" s="48"/>
       <c r="M30" s="49"/>
-      <c r="N30" s="181"/>
-      <c r="O30" s="182"/>
+      <c r="N30" s="171"/>
+      <c r="O30" s="172"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4104,7 +3981,7 @@
         <v>24</v>
       </c>
       <c r="B31" s="50"/>
-      <c r="C31" s="193" t="s">
+      <c r="C31" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D31" s="40"/>
@@ -4128,8 +4005,8 @@
       <c r="K31" s="52"/>
       <c r="L31" s="48"/>
       <c r="M31" s="49"/>
-      <c r="N31" s="181"/>
-      <c r="O31" s="182"/>
+      <c r="N31" s="171"/>
+      <c r="O31" s="172"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4137,7 +4014,7 @@
         <v>25</v>
       </c>
       <c r="B32" s="50"/>
-      <c r="C32" s="193" t="s">
+      <c r="C32" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D32" s="40"/>
@@ -4161,8 +4038,8 @@
       <c r="K32" s="52"/>
       <c r="L32" s="48"/>
       <c r="M32" s="49"/>
-      <c r="N32" s="181"/>
-      <c r="O32" s="182"/>
+      <c r="N32" s="171"/>
+      <c r="O32" s="172"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4170,7 +4047,7 @@
         <v>26</v>
       </c>
       <c r="B33" s="50"/>
-      <c r="C33" s="193" t="s">
+      <c r="C33" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D33" s="40"/>
@@ -4194,8 +4071,8 @@
       <c r="K33" s="52"/>
       <c r="L33" s="48"/>
       <c r="M33" s="49"/>
-      <c r="N33" s="181"/>
-      <c r="O33" s="182"/>
+      <c r="N33" s="171"/>
+      <c r="O33" s="172"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4203,7 +4080,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="39"/>
-      <c r="C34" s="193" t="s">
+      <c r="C34" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D34" s="40"/>
@@ -4227,8 +4104,8 @@
       <c r="K34" s="52"/>
       <c r="L34" s="48"/>
       <c r="M34" s="49"/>
-      <c r="N34" s="181"/>
-      <c r="O34" s="182"/>
+      <c r="N34" s="171"/>
+      <c r="O34" s="172"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4236,7 +4113,7 @@
         <v>28</v>
       </c>
       <c r="B35" s="39"/>
-      <c r="C35" s="193" t="s">
+      <c r="C35" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="40"/>
@@ -4260,8 +4137,8 @@
       <c r="K35" s="52"/>
       <c r="L35" s="48"/>
       <c r="M35" s="49"/>
-      <c r="N35" s="181"/>
-      <c r="O35" s="182"/>
+      <c r="N35" s="171"/>
+      <c r="O35" s="172"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4269,7 +4146,7 @@
         <v>29</v>
       </c>
       <c r="B36" s="50"/>
-      <c r="C36" s="193" t="s">
+      <c r="C36" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D36" s="40"/>
@@ -4285,9 +4162,7 @@
         <v/>
       </c>
       <c r="H36" s="49"/>
-      <c r="I36" s="51">
-        <v>8</v>
-      </c>
+      <c r="I36" s="51"/>
       <c r="J36" s="5" t="str" cm="1">
         <f t="array" ref="J36">IF(AND(ISNUMBER(H36),NOT(ISERROR(H36&gt;8)),H36&gt;8),H36-8,"")</f>
         <v/>
@@ -4295,8 +4170,8 @@
       <c r="K36" s="52"/>
       <c r="L36" s="48"/>
       <c r="M36" s="49"/>
-      <c r="N36" s="181"/>
-      <c r="O36" s="182"/>
+      <c r="N36" s="171"/>
+      <c r="O36" s="172"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4304,7 +4179,7 @@
         <v>30</v>
       </c>
       <c r="B37" s="50"/>
-      <c r="C37" s="193" t="s">
+      <c r="C37" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D37" s="40"/>
@@ -4320,9 +4195,7 @@
         <v/>
       </c>
       <c r="H37" s="49"/>
-      <c r="I37" s="51">
-        <v>8</v>
-      </c>
+      <c r="I37" s="51"/>
       <c r="J37" s="5" t="str" cm="1">
         <f t="array" ref="J37">IF(AND(ISNUMBER(H37),NOT(ISERROR(H37&gt;8)),H37&gt;8),H37-8,"")</f>
         <v/>
@@ -4330,8 +4203,8 @@
       <c r="K37" s="52"/>
       <c r="L37" s="48"/>
       <c r="M37" s="49"/>
-      <c r="N37" s="181"/>
-      <c r="O37" s="182"/>
+      <c r="N37" s="171"/>
+      <c r="O37" s="172"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4339,49 +4212,53 @@
         <v>31</v>
       </c>
       <c r="B38" s="50"/>
-      <c r="C38" s="193" t="s">
+      <c r="C38" s="149" t="s">
         <v>27</v>
       </c>
       <c r="D38" s="43"/>
-      <c r="E38" s="41"/>
-      <c r="F38" s="42" t="s">
-        <v>27</v>
-      </c>
-      <c r="G38" s="43"/>
+      <c r="E38" s="41" t="str" cm="1">
+        <f t="array" ref="E38">IF(ISBLANK(D38),"","12.00")</f>
+        <v/>
+      </c>
+      <c r="F38" s="151" t="s">
+        <v>27</v>
+      </c>
+      <c r="G38" s="43" t="str" cm="1">
+        <f t="array" ref="G38">IF(ISBLANK(D38),"","12.30")</f>
+        <v/>
+      </c>
       <c r="H38" s="49"/>
-      <c r="I38" s="58">
-        <v>8</v>
-      </c>
-      <c r="J38" s="59" t="str" cm="1">
+      <c r="I38" s="56"/>
+      <c r="J38" s="57" t="str" cm="1">
         <f t="array" ref="J38">IF(AND(ISNUMBER(H38),NOT(ISERROR(H38&gt;8)),H38&gt;8),H38-8,"")</f>
         <v/>
       </c>
-      <c r="K38" s="60"/>
+      <c r="K38" s="58"/>
       <c r="L38" s="48"/>
       <c r="M38" s="49"/>
-      <c r="N38" s="181"/>
-      <c r="O38" s="182"/>
+      <c r="N38" s="171"/>
+      <c r="O38" s="172"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="61" t="s">
+      <c r="A39" s="59" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="62"/>
-      <c r="C39" s="62"/>
-      <c r="D39" s="63"/>
-      <c r="E39" s="49"/>
-      <c r="F39" s="64" t="s">
+      <c r="B39" s="60"/>
+      <c r="C39" s="60"/>
+      <c r="D39" s="60"/>
+      <c r="E39" s="153"/>
+      <c r="F39" s="154" t="s">
         <v>29</v>
       </c>
-      <c r="G39" s="49"/>
-      <c r="H39" s="44" cm="1">
+      <c r="G39" s="155"/>
+      <c r="H39" s="150" cm="1">
         <f t="array" ref="H39">SUM(H8:H38)</f>
         <v>0</v>
       </c>
       <c r="I39" s="44" cm="1">
         <f t="array" ref="I39">SUM(I8:I38)</f>
-        <v>48</v>
+        <v>0</v>
       </c>
       <c r="J39" s="44" cm="1">
         <f t="array" ref="J39">SUM(J8:J38)</f>
@@ -4395,74 +4272,74 @@
         <f t="array" ref="L39">SUM(L8:L38)</f>
         <v>0</v>
       </c>
-      <c r="M39" s="64" t="s">
+      <c r="M39" s="61" t="s">
         <v>29</v>
       </c>
-      <c r="N39" s="183" t="s">
+      <c r="N39" s="175" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="182"/>
+      <c r="O39" s="172"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="65"/>
-      <c r="B40" s="66"/>
-      <c r="C40" s="66"/>
-      <c r="D40" s="66"/>
-      <c r="E40" s="66"/>
-      <c r="F40" s="66"/>
-      <c r="G40" s="66"/>
-      <c r="H40" s="66"/>
-      <c r="I40" s="66"/>
-      <c r="J40" s="66"/>
-      <c r="K40" s="66"/>
-      <c r="L40" s="67"/>
-      <c r="M40" s="68"/>
-      <c r="N40" s="68"/>
-      <c r="O40" s="68"/>
+      <c r="A40" s="62"/>
+      <c r="B40" s="63"/>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="152"/>
+      <c r="F40" s="152"/>
+      <c r="G40" s="152"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="63"/>
+      <c r="L40" s="64"/>
+      <c r="M40" s="65"/>
+      <c r="N40" s="65"/>
+      <c r="O40" s="65"/>
       <c r="P40" s="2"/>
     </row>
     <row r="41" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="69" t="s">
+      <c r="A41" s="66" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="70"/>
-      <c r="C41" s="70"/>
-      <c r="D41" s="70"/>
-      <c r="E41" s="70"/>
-      <c r="F41" s="70"/>
-      <c r="G41" s="70"/>
-      <c r="H41" s="70"/>
-      <c r="I41" s="70"/>
-      <c r="J41" s="70"/>
-      <c r="K41" s="71" t="s">
+      <c r="B41" s="67"/>
+      <c r="C41" s="67"/>
+      <c r="D41" s="67"/>
+      <c r="E41" s="67"/>
+      <c r="F41" s="67"/>
+      <c r="G41" s="67"/>
+      <c r="H41" s="67"/>
+      <c r="I41" s="67"/>
+      <c r="J41" s="67"/>
+      <c r="K41" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="L41" s="72"/>
+      <c r="L41" s="69"/>
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
     </row>
     <row r="42" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="73" t="s">
+      <c r="A42" s="70" t="s">
         <v>31</v>
       </c>
-      <c r="B42" s="74"/>
-      <c r="C42" s="74"/>
-      <c r="D42" s="74"/>
-      <c r="E42" s="74"/>
-      <c r="F42" s="74"/>
-      <c r="G42" s="74"/>
-      <c r="H42" s="75"/>
-      <c r="I42" s="75"/>
-      <c r="J42" s="76"/>
-      <c r="K42" s="77" cm="1">
+      <c r="B42" s="71"/>
+      <c r="C42" s="71"/>
+      <c r="D42" s="71"/>
+      <c r="E42" s="71"/>
+      <c r="F42" s="71"/>
+      <c r="G42" s="71"/>
+      <c r="H42" s="72"/>
+      <c r="I42" s="72"/>
+      <c r="J42" s="73"/>
+      <c r="K42" s="74" cm="1">
         <f t="array" ref="K42">H39-J39</f>
         <v>0</v>
       </c>
-      <c r="L42" s="78"/>
-      <c r="M42" s="79" t="s">
+      <c r="L42" s="75"/>
+      <c r="M42" s="76" t="s">
         <v>32</v>
       </c>
       <c r="N42" s="2"/>
@@ -4470,24 +4347,24 @@
       <c r="P42" s="2"/>
     </row>
     <row r="43" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="80" t="s">
+      <c r="A43" s="77" t="s">
         <v>33</v>
       </c>
-      <c r="B43" s="81"/>
-      <c r="C43" s="81"/>
-      <c r="D43" s="81"/>
-      <c r="E43" s="81"/>
-      <c r="F43" s="81"/>
-      <c r="G43" s="81"/>
-      <c r="H43" s="82"/>
-      <c r="I43" s="82"/>
-      <c r="J43" s="83"/>
-      <c r="K43" s="84" cm="1">
+      <c r="B43" s="78"/>
+      <c r="C43" s="78"/>
+      <c r="D43" s="78"/>
+      <c r="E43" s="78"/>
+      <c r="F43" s="78"/>
+      <c r="G43" s="78"/>
+      <c r="H43" s="79"/>
+      <c r="I43" s="79"/>
+      <c r="J43" s="80"/>
+      <c r="K43" s="81" cm="1">
         <f t="array" ref="K43">J39</f>
         <v>0</v>
       </c>
-      <c r="L43" s="78"/>
-      <c r="M43" s="79" t="s">
+      <c r="L43" s="75"/>
+      <c r="M43" s="76" t="s">
         <v>34</v>
       </c>
       <c r="N43" s="2"/>
@@ -4495,24 +4372,24 @@
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="85" t="s">
+      <c r="A44" s="82" t="s">
         <v>35</v>
       </c>
-      <c r="B44" s="86"/>
-      <c r="C44" s="86"/>
-      <c r="D44" s="86"/>
-      <c r="E44" s="86"/>
-      <c r="F44" s="86"/>
-      <c r="G44" s="86"/>
-      <c r="H44" s="87"/>
-      <c r="I44" s="87"/>
-      <c r="J44" s="88"/>
-      <c r="K44" s="89" cm="1">
+      <c r="B44" s="83"/>
+      <c r="C44" s="83"/>
+      <c r="D44" s="83"/>
+      <c r="E44" s="83"/>
+      <c r="F44" s="83"/>
+      <c r="G44" s="83"/>
+      <c r="H44" s="84"/>
+      <c r="I44" s="84"/>
+      <c r="J44" s="85"/>
+      <c r="K44" s="86" cm="1">
         <f t="array" ref="K44">K39</f>
         <v>0</v>
       </c>
-      <c r="L44" s="78"/>
-      <c r="M44" s="79" t="s">
+      <c r="L44" s="75"/>
+      <c r="M44" s="76" t="s">
         <v>36</v>
       </c>
       <c r="N44" s="2"/>
@@ -4520,24 +4397,24 @@
       <c r="P44" s="2"/>
     </row>
     <row r="45" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="90" t="s">
+      <c r="A45" s="87" t="s">
         <v>37</v>
       </c>
-      <c r="B45" s="91"/>
-      <c r="C45" s="91"/>
-      <c r="D45" s="91"/>
-      <c r="E45" s="91"/>
-      <c r="F45" s="91"/>
-      <c r="G45" s="91"/>
-      <c r="H45" s="92"/>
-      <c r="I45" s="92"/>
-      <c r="J45" s="93"/>
-      <c r="K45" s="94" cm="1">
+      <c r="B45" s="88"/>
+      <c r="C45" s="88"/>
+      <c r="D45" s="88"/>
+      <c r="E45" s="88"/>
+      <c r="F45" s="88"/>
+      <c r="G45" s="88"/>
+      <c r="H45" s="89"/>
+      <c r="I45" s="89"/>
+      <c r="J45" s="90"/>
+      <c r="K45" s="91" cm="1">
         <f t="array" ref="K45">H39</f>
         <v>0</v>
       </c>
-      <c r="L45" s="78"/>
-      <c r="M45" s="79" t="s">
+      <c r="L45" s="75"/>
+      <c r="M45" s="76" t="s">
         <v>38</v>
       </c>
       <c r="N45" s="2"/>
@@ -4545,19 +4422,19 @@
       <c r="P45" s="2"/>
     </row>
     <row r="46" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="95"/>
-      <c r="B46" s="96"/>
-      <c r="C46" s="96"/>
-      <c r="D46" s="96"/>
-      <c r="E46" s="96"/>
-      <c r="F46" s="96"/>
-      <c r="G46" s="96"/>
-      <c r="H46" s="96"/>
-      <c r="I46" s="96"/>
-      <c r="J46" s="96"/>
-      <c r="K46" s="96"/>
-      <c r="L46" s="72"/>
-      <c r="M46" s="79" t="s">
+      <c r="A46" s="92"/>
+      <c r="B46" s="93"/>
+      <c r="C46" s="93"/>
+      <c r="D46" s="93"/>
+      <c r="E46" s="93"/>
+      <c r="F46" s="93"/>
+      <c r="G46" s="93"/>
+      <c r="H46" s="93"/>
+      <c r="I46" s="93"/>
+      <c r="J46" s="93"/>
+      <c r="K46" s="93"/>
+      <c r="L46" s="69"/>
+      <c r="M46" s="76" t="s">
         <v>39</v>
       </c>
       <c r="N46" s="2"/>
@@ -4565,27 +4442,27 @@
       <c r="P46" s="2"/>
     </row>
     <row r="47" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="97" t="s">
+      <c r="A47" s="94" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="98"/>
-      <c r="C47" s="98"/>
-      <c r="D47" s="98"/>
-      <c r="E47" s="98"/>
-      <c r="F47" s="98"/>
-      <c r="G47" s="98"/>
-      <c r="H47" s="70"/>
-      <c r="I47" s="71" t="s">
+      <c r="B47" s="95"/>
+      <c r="C47" s="95"/>
+      <c r="D47" s="95"/>
+      <c r="E47" s="95"/>
+      <c r="F47" s="95"/>
+      <c r="G47" s="95"/>
+      <c r="H47" s="67"/>
+      <c r="I47" s="68" t="s">
         <v>41</v>
       </c>
-      <c r="J47" s="71" t="s">
+      <c r="J47" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="K47" s="71" t="s">
+      <c r="K47" s="68" t="s">
         <v>17</v>
       </c>
-      <c r="L47" s="72"/>
-      <c r="M47" s="79" t="s">
+      <c r="L47" s="69"/>
+      <c r="M47" s="76" t="s">
         <v>43</v>
       </c>
       <c r="N47" s="2"/>
@@ -4593,29 +4470,29 @@
       <c r="P47" s="2"/>
     </row>
     <row r="48" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="73" t="s">
+      <c r="A48" s="70" t="s">
         <v>44</v>
       </c>
-      <c r="B48" s="74"/>
-      <c r="C48" s="74"/>
-      <c r="D48" s="74"/>
-      <c r="E48" s="99"/>
-      <c r="F48" s="99"/>
-      <c r="G48" s="99"/>
-      <c r="H48" s="99"/>
-      <c r="I48" s="100" t="s">
+      <c r="B48" s="71"/>
+      <c r="C48" s="71"/>
+      <c r="D48" s="71"/>
+      <c r="E48" s="96"/>
+      <c r="F48" s="96"/>
+      <c r="G48" s="96"/>
+      <c r="H48" s="96"/>
+      <c r="I48" s="97" t="s">
         <v>29</v>
       </c>
-      <c r="J48" s="101" cm="1">
+      <c r="J48" s="98" cm="1">
         <f t="array" ref="J48">COUNTIF(H8:H38,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="K48" s="102" cm="1">
+      <c r="K48" s="99" cm="1">
         <f t="array" ref="K48">K42</f>
         <v>0</v>
       </c>
-      <c r="L48" s="78"/>
-      <c r="M48" s="79" t="s">
+      <c r="L48" s="75"/>
+      <c r="M48" s="76" t="s">
         <v>45</v>
       </c>
       <c r="N48" s="2"/>
@@ -4623,26 +4500,26 @@
       <c r="P48" s="2"/>
     </row>
     <row r="49" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="80" t="s">
+      <c r="A49" s="77" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="81"/>
-      <c r="C49" s="81"/>
-      <c r="D49" s="81"/>
-      <c r="E49" s="103"/>
-      <c r="F49" s="103"/>
-      <c r="G49" s="103"/>
-      <c r="H49" s="103"/>
-      <c r="I49" s="104" t="s">
+      <c r="B49" s="78"/>
+      <c r="C49" s="78"/>
+      <c r="D49" s="78"/>
+      <c r="E49" s="100"/>
+      <c r="F49" s="100"/>
+      <c r="G49" s="100"/>
+      <c r="H49" s="100"/>
+      <c r="I49" s="101" t="s">
         <v>29</v>
       </c>
-      <c r="J49" s="105"/>
-      <c r="K49" s="106" cm="1">
+      <c r="J49" s="102"/>
+      <c r="K49" s="103" cm="1">
         <f t="array" ref="K49">I39</f>
-        <v>48</v>
-      </c>
-      <c r="L49" s="78"/>
-      <c r="M49" s="79" t="s">
+        <v>0</v>
+      </c>
+      <c r="L49" s="75"/>
+      <c r="M49" s="76" t="s">
         <v>47</v>
       </c>
       <c r="N49" s="2"/>
@@ -4650,28 +4527,28 @@
       <c r="P49" s="2"/>
     </row>
     <row r="50" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="85" t="s">
+      <c r="A50" s="82" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="86"/>
-      <c r="C50" s="86"/>
-      <c r="D50" s="86"/>
-      <c r="E50" s="107"/>
-      <c r="F50" s="107"/>
-      <c r="G50" s="107"/>
-      <c r="H50" s="107"/>
-      <c r="I50" s="108" t="s">
+      <c r="B50" s="83"/>
+      <c r="C50" s="83"/>
+      <c r="D50" s="83"/>
+      <c r="E50" s="104"/>
+      <c r="F50" s="104"/>
+      <c r="G50" s="104"/>
+      <c r="H50" s="104"/>
+      <c r="I50" s="105" t="s">
         <v>29</v>
       </c>
-      <c r="J50" s="109" t="s">
+      <c r="J50" s="106" t="s">
         <v>29</v>
       </c>
-      <c r="K50" s="110" cm="1">
+      <c r="K50" s="107" cm="1">
         <f t="array" ref="K50">K39</f>
         <v>0</v>
       </c>
-      <c r="L50" s="78"/>
-      <c r="M50" s="79" t="s">
+      <c r="L50" s="75"/>
+      <c r="M50" s="76" t="s">
         <v>49</v>
       </c>
       <c r="N50" s="2"/>
@@ -4679,29 +4556,29 @@
       <c r="P50" s="2"/>
     </row>
     <row r="51" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="111" t="s">
+      <c r="A51" s="108" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="91"/>
-      <c r="C51" s="91"/>
-      <c r="D51" s="91"/>
-      <c r="E51" s="112"/>
-      <c r="F51" s="112"/>
-      <c r="G51" s="112"/>
-      <c r="H51" s="112"/>
-      <c r="I51" s="113" t="s">
+      <c r="B51" s="88"/>
+      <c r="C51" s="88"/>
+      <c r="D51" s="88"/>
+      <c r="E51" s="109"/>
+      <c r="F51" s="109"/>
+      <c r="G51" s="109"/>
+      <c r="H51" s="109"/>
+      <c r="I51" s="110" t="s">
         <v>29</v>
       </c>
-      <c r="J51" s="114" cm="1">
+      <c r="J51" s="111" cm="1">
         <f t="array" ref="J51">J48+J49</f>
         <v>0</v>
       </c>
-      <c r="K51" s="115" cm="1">
+      <c r="K51" s="112" cm="1">
         <f t="array" ref="K51">SUM(K48:K50)</f>
-        <v>48</v>
-      </c>
-      <c r="L51" s="78"/>
-      <c r="M51" s="79" t="s">
+        <v>0</v>
+      </c>
+      <c r="L51" s="75"/>
+      <c r="M51" s="76" t="s">
         <v>51</v>
       </c>
       <c r="N51" s="2"/>
@@ -4709,211 +4586,211 @@
       <c r="P51" s="2"/>
     </row>
     <row r="52" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="73" t="s">
+      <c r="A52" s="70" t="s">
         <v>52</v>
       </c>
-      <c r="B52" s="74"/>
-      <c r="C52" s="74"/>
-      <c r="D52" s="74"/>
-      <c r="E52" s="99"/>
-      <c r="F52" s="99"/>
-      <c r="G52" s="99"/>
-      <c r="H52" s="99"/>
-      <c r="I52" s="100" t="s">
+      <c r="B52" s="71"/>
+      <c r="C52" s="71"/>
+      <c r="D52" s="71"/>
+      <c r="E52" s="96"/>
+      <c r="F52" s="96"/>
+      <c r="G52" s="96"/>
+      <c r="H52" s="96"/>
+      <c r="I52" s="97" t="s">
         <v>29</v>
       </c>
-      <c r="J52" s="101">
+      <c r="J52" s="98">
         <v>0</v>
       </c>
-      <c r="K52" s="102">
+      <c r="K52" s="99">
         <v>0</v>
       </c>
-      <c r="L52" s="78"/>
+      <c r="L52" s="75"/>
       <c r="M52" s="7"/>
       <c r="N52" s="7"/>
       <c r="O52" s="7"/>
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="184" t="s">
+      <c r="A53" s="176" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="185"/>
-      <c r="C53" s="182"/>
-      <c r="D53" s="182"/>
-      <c r="E53" s="182"/>
-      <c r="F53" s="182"/>
-      <c r="G53" s="117"/>
-      <c r="H53" s="188"/>
-      <c r="I53" s="185"/>
-      <c r="J53" s="118" cm="1">
+      <c r="B53" s="177"/>
+      <c r="C53" s="172"/>
+      <c r="D53" s="172"/>
+      <c r="E53" s="172"/>
+      <c r="F53" s="172"/>
+      <c r="G53" s="114"/>
+      <c r="H53" s="178"/>
+      <c r="I53" s="177"/>
+      <c r="J53" s="115" cm="1">
         <f t="array" ref="J53">COUNTIF(B8:B38,"=D")</f>
         <v>0</v>
       </c>
-      <c r="K53" s="106" cm="1">
+      <c r="K53" s="103" cm="1">
         <f t="array" ref="K53">J53*8</f>
         <v>0</v>
       </c>
-      <c r="L53" s="119"/>
-      <c r="M53" s="120" t="s">
+      <c r="L53" s="116"/>
+      <c r="M53" s="117" t="s">
         <v>54</v>
       </c>
-      <c r="N53" s="121" t="s">
+      <c r="N53" s="118" t="s">
         <v>55</v>
       </c>
-      <c r="O53" s="122" t="s">
+      <c r="O53" s="119" t="s">
         <v>56</v>
       </c>
       <c r="P53" s="17"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="184" t="s">
+      <c r="A54" s="176" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="185"/>
-      <c r="C54" s="182"/>
-      <c r="D54" s="182"/>
-      <c r="E54" s="182"/>
-      <c r="F54" s="182"/>
-      <c r="G54" s="117"/>
-      <c r="H54" s="123"/>
-      <c r="I54" s="124"/>
-      <c r="J54" s="125">
-        <v>3</v>
-      </c>
-      <c r="K54" s="106" cm="1">
+      <c r="B54" s="177"/>
+      <c r="C54" s="172"/>
+      <c r="D54" s="172"/>
+      <c r="E54" s="172"/>
+      <c r="F54" s="172"/>
+      <c r="G54" s="114"/>
+      <c r="H54" s="120"/>
+      <c r="I54" s="121"/>
+      <c r="J54" s="122">
+        <v>0</v>
+      </c>
+      <c r="K54" s="103" cm="1">
         <f t="array" ref="K54">J54*8</f>
-        <v>24</v>
-      </c>
-      <c r="L54" s="119"/>
-      <c r="M54" s="120" t="s">
+        <v>0</v>
+      </c>
+      <c r="L54" s="116"/>
+      <c r="M54" s="117" t="s">
         <v>58</v>
       </c>
-      <c r="N54" s="126">
-        <v>20</v>
-      </c>
-      <c r="O54" s="127" cm="1">
+      <c r="N54" s="123">
+        <v>0</v>
+      </c>
+      <c r="O54" s="124" cm="1">
         <f t="array" ref="O54">N54*8</f>
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="P54" s="17"/>
     </row>
     <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="184" t="s">
+      <c r="A55" s="176" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="185"/>
-      <c r="C55" s="182"/>
-      <c r="D55" s="182"/>
-      <c r="E55" s="182"/>
-      <c r="F55" s="182"/>
-      <c r="G55" s="117"/>
-      <c r="H55" s="123"/>
-      <c r="I55" s="124"/>
-      <c r="J55" s="105"/>
-      <c r="K55" s="128"/>
-      <c r="L55" s="119"/>
-      <c r="M55" s="120" t="s">
+      <c r="B55" s="177"/>
+      <c r="C55" s="172"/>
+      <c r="D55" s="172"/>
+      <c r="E55" s="172"/>
+      <c r="F55" s="172"/>
+      <c r="G55" s="114"/>
+      <c r="H55" s="120"/>
+      <c r="I55" s="121"/>
+      <c r="J55" s="102"/>
+      <c r="K55" s="125"/>
+      <c r="L55" s="116"/>
+      <c r="M55" s="117" t="s">
         <v>60</v>
       </c>
-      <c r="N55" s="129" cm="1">
+      <c r="N55" s="126" cm="1">
         <f t="array" ref="N55">J54</f>
-        <v>3</v>
-      </c>
-      <c r="O55" s="130" cm="1">
+        <v>0</v>
+      </c>
+      <c r="O55" s="127" cm="1">
         <f t="array" ref="O55">K54</f>
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="P55" s="17"/>
     </row>
     <row r="56" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="184" t="s">
+      <c r="A56" s="176" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="185"/>
-      <c r="C56" s="182"/>
-      <c r="D56" s="182"/>
-      <c r="E56" s="182"/>
-      <c r="F56" s="182"/>
-      <c r="G56" s="117"/>
-      <c r="H56" s="123"/>
-      <c r="I56" s="124"/>
-      <c r="J56" s="105"/>
-      <c r="K56" s="128"/>
-      <c r="L56" s="119"/>
-      <c r="M56" s="120" t="s">
+      <c r="B56" s="177"/>
+      <c r="C56" s="172"/>
+      <c r="D56" s="172"/>
+      <c r="E56" s="172"/>
+      <c r="F56" s="172"/>
+      <c r="G56" s="114"/>
+      <c r="H56" s="120"/>
+      <c r="I56" s="121"/>
+      <c r="J56" s="102"/>
+      <c r="K56" s="125"/>
+      <c r="L56" s="116"/>
+      <c r="M56" s="117" t="s">
         <v>8</v>
       </c>
-      <c r="N56" s="131" cm="1">
+      <c r="N56" s="128" cm="1">
         <f t="array" ref="N56">SUM(N54:N55)</f>
-        <v>23</v>
-      </c>
-      <c r="O56" s="132" cm="1">
+        <v>0</v>
+      </c>
+      <c r="O56" s="129" cm="1">
         <f t="array" ref="O56">SUM(O54:O55)</f>
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="P56" s="17"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="184" t="s">
+      <c r="A57" s="176" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="185"/>
-      <c r="C57" s="182"/>
-      <c r="D57" s="182"/>
-      <c r="E57" s="182"/>
-      <c r="F57" s="182"/>
-      <c r="G57" s="117"/>
-      <c r="H57" s="123"/>
-      <c r="I57" s="124"/>
-      <c r="J57" s="105"/>
-      <c r="K57" s="128"/>
-      <c r="L57" s="78"/>
-      <c r="M57" s="68"/>
-      <c r="N57" s="68"/>
-      <c r="O57" s="68"/>
+      <c r="B57" s="177"/>
+      <c r="C57" s="172"/>
+      <c r="D57" s="172"/>
+      <c r="E57" s="172"/>
+      <c r="F57" s="172"/>
+      <c r="G57" s="114"/>
+      <c r="H57" s="120"/>
+      <c r="I57" s="121"/>
+      <c r="J57" s="102"/>
+      <c r="K57" s="125"/>
+      <c r="L57" s="75"/>
+      <c r="M57" s="65"/>
+      <c r="N57" s="65"/>
+      <c r="O57" s="65"/>
       <c r="P57" s="2"/>
     </row>
     <row r="58" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="186" t="s">
+      <c r="A58" s="179" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="187"/>
-      <c r="C58" s="187"/>
-      <c r="D58" s="187"/>
-      <c r="E58" s="187"/>
-      <c r="F58" s="187"/>
-      <c r="G58" s="134"/>
-      <c r="H58" s="134"/>
-      <c r="I58" s="135" t="s">
+      <c r="B58" s="180"/>
+      <c r="C58" s="180"/>
+      <c r="D58" s="180"/>
+      <c r="E58" s="180"/>
+      <c r="F58" s="180"/>
+      <c r="G58" s="131"/>
+      <c r="H58" s="131"/>
+      <c r="I58" s="132" t="s">
         <v>29</v>
       </c>
-      <c r="J58" s="136" cm="1">
+      <c r="J58" s="133" cm="1">
         <f t="array" ref="J58">SUM(J51:J57)</f>
-        <v>3</v>
-      </c>
-      <c r="K58" s="110" cm="1">
+        <v>0</v>
+      </c>
+      <c r="K58" s="107" cm="1">
         <f t="array" ref="K58">SUM(K51:K57)</f>
-        <v>72</v>
-      </c>
-      <c r="L58" s="78"/>
+        <v>0</v>
+      </c>
+      <c r="L58" s="75"/>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
     <row r="59" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="137"/>
-      <c r="B59" s="137"/>
-      <c r="C59" s="137"/>
-      <c r="D59" s="137"/>
-      <c r="E59" s="137"/>
-      <c r="F59" s="137"/>
-      <c r="G59" s="137"/>
-      <c r="H59" s="137"/>
-      <c r="I59" s="137"/>
-      <c r="J59" s="138"/>
-      <c r="K59" s="138"/>
+      <c r="A59" s="134"/>
+      <c r="B59" s="134"/>
+      <c r="C59" s="134"/>
+      <c r="D59" s="134"/>
+      <c r="E59" s="134"/>
+      <c r="F59" s="134"/>
+      <c r="G59" s="134"/>
+      <c r="H59" s="134"/>
+      <c r="I59" s="134"/>
+      <c r="J59" s="135"/>
+      <c r="K59" s="135"/>
       <c r="L59" s="2"/>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
@@ -4921,19 +4798,19 @@
       <c r="P59" s="2"/>
     </row>
     <row r="60" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="139" t="s">
+      <c r="A60" s="136" t="s">
         <v>63</v>
       </c>
-      <c r="B60" s="140"/>
-      <c r="C60" s="140"/>
-      <c r="D60" s="140"/>
-      <c r="E60" s="140"/>
-      <c r="F60" s="140"/>
-      <c r="G60" s="140"/>
-      <c r="H60" s="140"/>
-      <c r="I60" s="140"/>
-      <c r="J60" s="141"/>
-      <c r="K60" s="142" t="s">
+      <c r="B60" s="137"/>
+      <c r="C60" s="137"/>
+      <c r="D60" s="137"/>
+      <c r="E60" s="137"/>
+      <c r="F60" s="137"/>
+      <c r="G60" s="137"/>
+      <c r="H60" s="137"/>
+      <c r="I60" s="137"/>
+      <c r="J60" s="138"/>
+      <c r="K60" s="139" t="s">
         <v>17</v>
       </c>
       <c r="L60" s="2"/>
@@ -4943,117 +4820,117 @@
       <c r="P60" s="2"/>
     </row>
     <row r="61" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="143" t="s">
+      <c r="A61" s="140" t="s">
         <v>64</v>
       </c>
-      <c r="B61" s="144"/>
-      <c r="C61" s="144"/>
-      <c r="D61" s="144"/>
-      <c r="E61" s="145"/>
-      <c r="F61" s="145"/>
-      <c r="G61" s="145"/>
-      <c r="H61" s="145"/>
-      <c r="I61" s="145"/>
-      <c r="J61" s="146"/>
-      <c r="K61" s="102">
-        <v>39</v>
-      </c>
-      <c r="L61" s="78"/>
+      <c r="B61" s="141"/>
+      <c r="C61" s="141"/>
+      <c r="D61" s="141"/>
+      <c r="E61" s="142"/>
+      <c r="F61" s="142"/>
+      <c r="G61" s="142"/>
+      <c r="H61" s="142"/>
+      <c r="I61" s="142"/>
+      <c r="J61" s="143"/>
+      <c r="K61" s="99">
+        <v>0</v>
+      </c>
+      <c r="L61" s="75"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
     <row r="62" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="116" t="s">
+      <c r="A62" s="113" t="s">
         <v>65</v>
       </c>
-      <c r="B62" s="147"/>
-      <c r="C62" s="147"/>
-      <c r="D62" s="147"/>
-      <c r="E62" s="123"/>
-      <c r="F62" s="123"/>
-      <c r="G62" s="123"/>
-      <c r="H62" s="123"/>
-      <c r="I62" s="123"/>
-      <c r="J62" s="124"/>
-      <c r="K62" s="106" cm="1">
+      <c r="B62" s="144"/>
+      <c r="C62" s="144"/>
+      <c r="D62" s="144"/>
+      <c r="E62" s="120"/>
+      <c r="F62" s="120"/>
+      <c r="G62" s="120"/>
+      <c r="H62" s="120"/>
+      <c r="I62" s="120"/>
+      <c r="J62" s="121"/>
+      <c r="K62" s="103" cm="1">
         <f t="array" ref="K62">K49</f>
-        <v>48</v>
-      </c>
-      <c r="L62" s="78"/>
+        <v>0</v>
+      </c>
+      <c r="L62" s="75"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
     </row>
     <row r="63" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="116" t="s">
+      <c r="A63" s="113" t="s">
         <v>66</v>
       </c>
-      <c r="B63" s="147"/>
-      <c r="C63" s="147"/>
-      <c r="D63" s="147"/>
-      <c r="E63" s="123"/>
-      <c r="F63" s="123"/>
-      <c r="G63" s="123"/>
-      <c r="H63" s="123"/>
-      <c r="I63" s="123"/>
-      <c r="J63" s="124"/>
-      <c r="K63" s="106" cm="1">
+      <c r="B63" s="144"/>
+      <c r="C63" s="144"/>
+      <c r="D63" s="144"/>
+      <c r="E63" s="120"/>
+      <c r="F63" s="120"/>
+      <c r="G63" s="120"/>
+      <c r="H63" s="120"/>
+      <c r="I63" s="120"/>
+      <c r="J63" s="121"/>
+      <c r="K63" s="103" cm="1">
         <f t="array" ref="K63">K43</f>
         <v>0</v>
       </c>
-      <c r="L63" s="78"/>
-      <c r="M63" s="79" t="s">
+      <c r="L63" s="75"/>
+      <c r="M63" s="76" t="s">
         <v>67</v>
       </c>
-      <c r="N63" s="148"/>
-      <c r="O63" s="148"/>
+      <c r="N63" s="145"/>
+      <c r="O63" s="145"/>
       <c r="P63" s="2"/>
     </row>
     <row r="64" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="133" t="s">
+      <c r="A64" s="130" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="149"/>
-      <c r="C64" s="149"/>
-      <c r="D64" s="149"/>
-      <c r="E64" s="134"/>
-      <c r="F64" s="134"/>
-      <c r="G64" s="134"/>
-      <c r="H64" s="134"/>
-      <c r="I64" s="134"/>
-      <c r="J64" s="150"/>
-      <c r="K64" s="110" cm="1">
+      <c r="B64" s="146"/>
+      <c r="C64" s="146"/>
+      <c r="D64" s="146"/>
+      <c r="E64" s="131"/>
+      <c r="F64" s="131"/>
+      <c r="G64" s="131"/>
+      <c r="H64" s="131"/>
+      <c r="I64" s="131"/>
+      <c r="J64" s="147"/>
+      <c r="K64" s="107" cm="1">
         <f t="array" ref="K64">K61+K63-K62</f>
-        <v>-9</v>
-      </c>
-      <c r="L64" s="78"/>
-      <c r="M64" s="79" t="s">
+        <v>0</v>
+      </c>
+      <c r="L64" s="75"/>
+      <c r="M64" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="N64" s="148"/>
-      <c r="O64" s="148"/>
+      <c r="N64" s="145"/>
+      <c r="O64" s="145"/>
       <c r="P64" s="2"/>
     </row>
     <row r="65" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="137"/>
-      <c r="B65" s="137"/>
-      <c r="C65" s="137"/>
-      <c r="D65" s="137"/>
-      <c r="E65" s="137"/>
-      <c r="F65" s="137"/>
-      <c r="G65" s="137"/>
-      <c r="H65" s="137"/>
-      <c r="I65" s="151"/>
-      <c r="J65" s="151"/>
-      <c r="K65" s="151"/>
-      <c r="L65" s="148"/>
+      <c r="A65" s="134"/>
+      <c r="B65" s="134"/>
+      <c r="C65" s="134"/>
+      <c r="D65" s="134"/>
+      <c r="E65" s="134"/>
+      <c r="F65" s="134"/>
+      <c r="G65" s="134"/>
+      <c r="H65" s="134"/>
+      <c r="I65" s="148"/>
+      <c r="J65" s="148"/>
+      <c r="K65" s="148"/>
+      <c r="L65" s="145"/>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
-      <c r="P65" s="148"/>
+      <c r="P65" s="145"/>
     </row>
   </sheetData>
   <mergeCells count="49">
@@ -5070,19 +4947,19 @@
     <mergeCell ref="N17:O17"/>
     <mergeCell ref="N16:O16"/>
     <mergeCell ref="N15:O15"/>
+    <mergeCell ref="N35:O35"/>
+    <mergeCell ref="N30:O30"/>
+    <mergeCell ref="N31:O31"/>
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="A56:F56"/>
     <mergeCell ref="A57:F57"/>
     <mergeCell ref="A58:F58"/>
-    <mergeCell ref="N35:O35"/>
     <mergeCell ref="N37:O37"/>
     <mergeCell ref="N38:O38"/>
     <mergeCell ref="N39:O39"/>
     <mergeCell ref="A53:F53"/>
     <mergeCell ref="H53:I53"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="N31:O31"/>
     <mergeCell ref="N32:O32"/>
     <mergeCell ref="N33:O33"/>
     <mergeCell ref="N34:O34"/>
@@ -5111,494 +4988,4 @@
   <pageSetup scale="85" orientation="portrait"/>
   <drawing r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:K62"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="16.33203125" defaultRowHeight="15.5" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="3" width="16.33203125" style="1" customWidth="1"/>
-    <col min="4" max="4" width="6.1640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="19.1640625" style="1" customWidth="1"/>
-    <col min="7" max="8" width="16.33203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="17.83203125" style="1" customWidth="1"/>
-    <col min="10" max="10" width="17.6640625" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.83203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="16.33203125" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="16.33203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="192" t="s">
-        <v>70</v>
-      </c>
-      <c r="B1" s="192"/>
-    </row>
-    <row r="2" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="152" t="s">
-        <v>71</v>
-      </c>
-      <c r="B2" s="152" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="153" cm="1">
-        <f t="array" aca="1" ref="A3" ca="1">MONTH(TODAY())-1</f>
-        <v>0</v>
-      </c>
-      <c r="B3" s="153" cm="1">
-        <f t="array" aca="1" ref="B3" ca="1">YEAR(TODAY())</f>
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C5" s="192" t="s">
-        <v>73</v>
-      </c>
-      <c r="D5" s="192"/>
-      <c r="E5" s="192"/>
-    </row>
-    <row r="6" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C6" s="152" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="152" t="s">
-        <v>70</v>
-      </c>
-      <c r="E6" s="154"/>
-    </row>
-    <row r="7" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C7" s="155" t="s">
-        <v>75</v>
-      </c>
-      <c r="D7" s="156" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="157" t="e" cm="1">
-        <f t="array" aca="1" ref="E7" ca="1">DATEVALUE(_xlfn.CONCAT(D7,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C8" s="158" t="s">
-        <v>77</v>
-      </c>
-      <c r="D8" s="159" t="s">
-        <v>78</v>
-      </c>
-      <c r="E8" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E8" ca="1">DATEVALUE(_xlfn.CONCAT(D8,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C9" s="158" t="s">
-        <v>79</v>
-      </c>
-      <c r="D9" s="159" t="s">
-        <v>80</v>
-      </c>
-      <c r="E9" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E9" ca="1">DATEVALUE(_xlfn.CONCAT(D9,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C10" s="158" t="s">
-        <v>81</v>
-      </c>
-      <c r="D10" s="159" t="s">
-        <v>82</v>
-      </c>
-      <c r="E10" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E10" ca="1">DATEVALUE(_xlfn.CONCAT(D10,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C11" s="158" t="s">
-        <v>83</v>
-      </c>
-      <c r="D11" s="159" t="s">
-        <v>84</v>
-      </c>
-      <c r="E11" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E11" ca="1">DATEVALUE(_xlfn.CONCAT(D11,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C12" s="158" t="s">
-        <v>85</v>
-      </c>
-      <c r="D12" s="159" t="s">
-        <v>86</v>
-      </c>
-      <c r="E12" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E12" ca="1">DATEVALUE(_xlfn.CONCAT(D12,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C13" s="158" t="s">
-        <v>87</v>
-      </c>
-      <c r="D13" s="159" t="s">
-        <v>88</v>
-      </c>
-      <c r="E13" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E13" ca="1">DATEVALUE(_xlfn.CONCAT(D13,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C14" s="158" t="s">
-        <v>89</v>
-      </c>
-      <c r="D14" s="159" t="s">
-        <v>90</v>
-      </c>
-      <c r="E14" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E14" ca="1">DATEVALUE(_xlfn.CONCAT(D14,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C15" s="158" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15" s="159" t="s">
-        <v>92</v>
-      </c>
-      <c r="E15" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E15" ca="1">DATEVALUE(_xlfn.CONCAT(D15,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C16" s="158" t="s">
-        <v>93</v>
-      </c>
-      <c r="D16" s="159" t="s">
-        <v>94</v>
-      </c>
-      <c r="E16" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E16" ca="1">DATEVALUE(_xlfn.CONCAT(D16,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="17" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C17" s="158" t="s">
-        <v>95</v>
-      </c>
-      <c r="D17" s="159" t="s">
-        <v>96</v>
-      </c>
-      <c r="E17" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E17" ca="1">DATEVALUE(_xlfn.CONCAT(D17,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="18" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C18" s="158" t="s">
-        <v>97</v>
-      </c>
-      <c r="D18" s="159" t="s">
-        <v>98</v>
-      </c>
-      <c r="E18" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E18" ca="1">DATEVALUE(_xlfn.CONCAT(D18,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="19" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="C19" s="158" t="s">
-        <v>99</v>
-      </c>
-      <c r="D19" s="159" t="s">
-        <v>100</v>
-      </c>
-      <c r="E19" s="160" t="e" cm="1">
-        <f t="array" aca="1" ref="E19" ca="1">DATEVALUE(_xlfn.CONCAT(D19,$B$3))</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="21" spans="3:7" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F21" s="192" t="s">
-        <v>101</v>
-      </c>
-      <c r="G21" s="192"/>
-    </row>
-    <row r="22" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F22" s="154"/>
-      <c r="G22" s="154"/>
-    </row>
-    <row r="23" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F23" s="155" t="s">
-        <v>102</v>
-      </c>
-      <c r="G23" s="161" cm="1">
-        <f t="array" aca="1" ref="G23" ca="1">DATE($B$3,$A$3,1)</f>
-        <v>45992</v>
-      </c>
-    </row>
-    <row r="24" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F24" s="158" t="s">
-        <v>103</v>
-      </c>
-      <c r="G24" s="162" cm="1">
-        <f t="array" aca="1" ref="G24" ca="1">EOMONTH(DATE(B3,A3,1),0)</f>
-        <v>46022</v>
-      </c>
-    </row>
-    <row r="25" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F25" s="158" t="s">
-        <v>101</v>
-      </c>
-      <c r="G25" s="163" cm="1">
-        <f t="array" aca="1" ref="G25" ca="1">NETWORKDAYS($G$23,$G$24)</f>
-        <v>23</v>
-      </c>
-    </row>
-    <row r="26" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F26" s="158" t="s">
-        <v>73</v>
-      </c>
-      <c r="G26" s="163" t="e" cm="1">
-        <f t="array" aca="1" ref="G26" ca="1">G25-NETWORKDAYS($G$23,$G$24,E7:E19)</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="27" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F27" s="158" t="s">
-        <v>104</v>
-      </c>
-      <c r="G27" s="163" t="e" cm="1">
-        <f t="array" aca="1" ref="G27" ca="1">G25-G26</f>
-        <v>#VALUE!</v>
-      </c>
-    </row>
-    <row r="28" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F28" s="158" t="s">
-        <v>105</v>
-      </c>
-      <c r="G28" s="164" cm="1">
-        <f t="array" ref="G28">COUNT(H37:H50)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F29" s="165"/>
-      <c r="G29" s="163"/>
-    </row>
-    <row r="30" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F30" s="165"/>
-      <c r="G30" s="163"/>
-    </row>
-    <row r="31" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F31" s="165"/>
-      <c r="G31" s="163"/>
-    </row>
-    <row r="32" spans="3:7" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F32" s="165"/>
-      <c r="G32" s="163"/>
-    </row>
-    <row r="33" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F33" s="165"/>
-      <c r="G33" s="163"/>
-    </row>
-    <row r="35" spans="6:9" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H35" s="192" t="s">
-        <v>106</v>
-      </c>
-      <c r="I35" s="192"/>
-    </row>
-    <row r="36" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H36" s="152" t="s">
-        <v>5</v>
-      </c>
-      <c r="I36" s="152" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="37" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H37" s="166"/>
-      <c r="I37" s="166" t="str" cm="1">
-        <f t="array" ref="I37">IF(ISBLANK(H37),"",DATE(B3,A3,H37))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H38" s="167"/>
-      <c r="I38" s="167" t="str" cm="1">
-        <f t="array" ref="I38">IF(ISBLANK(H38),"",DATE(B4,A4,H38))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H39" s="167"/>
-      <c r="I39" s="167" t="str" cm="1">
-        <f t="array" ref="I39">IF(ISBLANK(H39),"",DATE(B5,A5,H39))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H40" s="167"/>
-      <c r="I40" s="167" t="str" cm="1">
-        <f t="array" ref="I40">IF(ISBLANK(H40),"",DATE(B6,A6,H40))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H41" s="167"/>
-      <c r="I41" s="167" t="str" cm="1">
-        <f t="array" ref="I41">IF(ISBLANK(H41),"",DATE(B7,A7,H41))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H42" s="167"/>
-      <c r="I42" s="167" t="str" cm="1">
-        <f t="array" ref="I42">IF(ISBLANK(H42),"",DATE(B8,A8,H42))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H43" s="167"/>
-      <c r="I43" s="167" t="str" cm="1">
-        <f t="array" ref="I43">IF(ISBLANK(H43),"",DATE(B9,A9,H43))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H44" s="167"/>
-      <c r="I44" s="167" t="str" cm="1">
-        <f t="array" ref="I44">IF(ISBLANK(H44),"",DATE(B10,A10,H44))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H45" s="167"/>
-      <c r="I45" s="167" t="str" cm="1">
-        <f t="array" ref="I45">IF(ISBLANK(H45),"",DATE(B11,A11,H45))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H46" s="167"/>
-      <c r="I46" s="167" t="str" cm="1">
-        <f t="array" ref="I46">IF(ISBLANK(H46),"",DATE(B12,A12,H46))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H47" s="167"/>
-      <c r="I47" s="167" t="str" cm="1">
-        <f t="array" ref="I47">IF(ISBLANK(H47),"",DATE(B13,A13,H47))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="6:9" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H48" s="167"/>
-      <c r="I48" s="167" t="str" cm="1">
-        <f t="array" ref="I48">IF(ISBLANK(H48),"",DATE(B14,A14,H48))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H49" s="167"/>
-      <c r="I49" s="167" t="str" cm="1">
-        <f t="array" ref="I49">IF(ISBLANK(H49),"",DATE(B15,A15,H49))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="H50" s="167"/>
-      <c r="I50" s="167" t="str" cm="1">
-        <f t="array" ref="I50">IF(ISBLANK(H50),"",DATE(B16,A16,H50))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="8:11" ht="15.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J52" s="192" t="s">
-        <v>108</v>
-      </c>
-      <c r="K52" s="192"/>
-    </row>
-    <row r="53" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J53" s="152" t="s">
-        <v>109</v>
-      </c>
-      <c r="K53" s="152" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="54" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J54" s="168">
-        <v>45690.291666666664</v>
-      </c>
-      <c r="K54" s="168">
-        <v>45690.666666666664</v>
-      </c>
-    </row>
-    <row r="55" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J55" s="169">
-        <v>45690.333333333336</v>
-      </c>
-      <c r="K55" s="169">
-        <v>45690.645833333336</v>
-      </c>
-    </row>
-    <row r="56" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J56" s="169">
-        <v>45690.3125</v>
-      </c>
-      <c r="K56" s="169">
-        <v>45690.6875</v>
-      </c>
-    </row>
-    <row r="57" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J57" s="167"/>
-      <c r="K57" s="167"/>
-    </row>
-    <row r="58" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J58" s="167"/>
-      <c r="K58" s="167"/>
-    </row>
-    <row r="59" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J59" s="167"/>
-      <c r="K59" s="167"/>
-    </row>
-    <row r="60" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J60" s="167"/>
-      <c r="K60" s="167"/>
-    </row>
-    <row r="61" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J61" s="167"/>
-      <c r="K61" s="167"/>
-    </row>
-    <row r="62" spans="8:11" ht="13" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J62" s="167"/>
-      <c r="K62" s="167"/>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="C5:E5"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="J52:K52"/>
-  </mergeCells>
-  <pageMargins left="1" right="1" top="1" bottom="1" header="0.25" footer="0.25"/>
-  <pageSetup orientation="portrait"/>
-  <headerFooter>
-    <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
-  </headerFooter>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
add FPD and NV input values to XLSX export, improve table input sizing
- Export working days count to N54 and previous months NV to K61
- Update template.xlsx with formulas for summary sections
- Make table inputs fill their cells with w-full styling

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C25D03B-EF7D-304D-8986-48329C408942}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BE7CED-067A-034F-9547-F2041C5BD629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="36020" windowHeight="24580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20" yWindow="680" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="evid.PD" sheetId="1" r:id="rId1"/>
@@ -271,7 +271,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -340,6 +340,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -355,7 +361,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="82">
+  <borders count="93">
     <border>
       <left/>
       <right/>
@@ -1160,68 +1166,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="8"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="8"/>
       </left>
@@ -1461,6 +1405,239 @@
       </top>
       <bottom style="thin">
         <color indexed="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color indexed="9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top style="medium">
+        <color indexed="8"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="9"/>
+      </left>
+      <right style="thin">
+        <color indexed="9"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="9"/>
+      </left>
+      <right style="thin">
+        <color indexed="9"/>
+      </right>
+      <top style="thin">
+        <color indexed="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="9"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="medium">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="medium">
+        <color theme="1"/>
+      </right>
+      <top style="thin">
+        <color theme="1"/>
+      </top>
+      <bottom style="medium">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="8"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="9"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1468,7 +1645,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="200">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1596,9 +1773,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1609,9 +1783,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1620,18 +1791,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
@@ -1642,9 +1807,6 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1652,20 +1814,8 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1673,84 +1823,40 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="67" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="70" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="71" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="72" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="67" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1761,24 +1867,99 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="75" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="75" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="81" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="82" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="83" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="84" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="85" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="86" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="88" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="77" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="89" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1802,10 +1983,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1814,19 +1995,37 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="65" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="79" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="81" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -3037,9 +3236,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="164"/>
-      <c r="C1" s="165"/>
-      <c r="D1" s="165"/>
+      <c r="B1" s="170"/>
+      <c r="C1" s="171"/>
+      <c r="D1" s="171"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3056,49 +3255,49 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="180" t="s">
+      <c r="A2" s="186" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="165"/>
-      <c r="C2" s="165"/>
-      <c r="D2" s="165"/>
-      <c r="E2" s="165"/>
-      <c r="F2" s="165"/>
-      <c r="G2" s="165"/>
+      <c r="B2" s="171"/>
+      <c r="C2" s="171"/>
+      <c r="D2" s="171"/>
+      <c r="E2" s="171"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="171"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="179" t="s">
+      <c r="L2" s="185" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="165"/>
+      <c r="M2" s="171"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="166" t="s">
+      <c r="A3" s="172" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="167"/>
-      <c r="C3" s="167"/>
-      <c r="D3" s="167"/>
+      <c r="B3" s="173"/>
+      <c r="C3" s="173"/>
+      <c r="D3" s="173"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="181" t="s">
+      <c r="F3" s="187" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="167"/>
-      <c r="H3" s="167"/>
-      <c r="I3" s="167"/>
+      <c r="G3" s="173"/>
+      <c r="H3" s="173"/>
+      <c r="I3" s="173"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="167" t="str" cm="1">
+      <c r="L3" s="173" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="167"/>
-      <c r="N3" s="167"/>
+      <c r="M3" s="173"/>
+      <c r="N3" s="173"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3106,11 +3305,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="162" t="s">
+      <c r="B4" s="168" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="163"/>
-      <c r="D4" s="163"/>
+      <c r="C4" s="169"/>
+      <c r="D4" s="169"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3142,12 +3341,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="158"/>
-      <c r="C5" s="159"/>
-      <c r="D5" s="159"/>
-      <c r="E5" s="168"/>
-      <c r="F5" s="159"/>
-      <c r="G5" s="159"/>
+      <c r="B5" s="164"/>
+      <c r="C5" s="165"/>
+      <c r="D5" s="165"/>
+      <c r="E5" s="174"/>
+      <c r="F5" s="165"/>
+      <c r="G5" s="165"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3174,22 +3373,22 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="159"/>
-      <c r="C6" s="159"/>
-      <c r="D6" s="159"/>
-      <c r="E6" s="159"/>
-      <c r="F6" s="159"/>
-      <c r="G6" s="159"/>
+      <c r="B6" s="165"/>
+      <c r="C6" s="165"/>
+      <c r="D6" s="165"/>
+      <c r="E6" s="165"/>
+      <c r="F6" s="165"/>
+      <c r="G6" s="165"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
       <c r="I6" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="186" t="s">
+      <c r="J6" s="133" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="187"/>
+      <c r="K6" s="134"/>
       <c r="L6" s="26"/>
       <c r="M6" s="18"/>
       <c r="N6" s="27"/>
@@ -3198,11 +3397,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="28"/>
-      <c r="B7" s="160" t="s">
+      <c r="B7" s="166" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="161"/>
-      <c r="D7" s="161"/>
+      <c r="C7" s="167"/>
+      <c r="D7" s="167"/>
       <c r="E7" s="30"/>
       <c r="F7" s="29" t="s">
         <v>22</v>
@@ -3237,7 +3436,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="37"/>
-      <c r="C8" s="146" t="s">
+      <c r="C8" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="38"/>
@@ -3261,16 +3460,16 @@
       <c r="K8" s="45"/>
       <c r="L8" s="46"/>
       <c r="M8" s="47"/>
-      <c r="N8" s="169"/>
-      <c r="O8" s="170"/>
+      <c r="N8" s="175"/>
+      <c r="O8" s="176"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="36">
         <v>2</v>
       </c>
-      <c r="B9" s="157"/>
-      <c r="C9" s="146" t="s">
+      <c r="B9" s="132"/>
+      <c r="C9" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="38"/>
@@ -3294,8 +3493,8 @@
       <c r="K9" s="49"/>
       <c r="L9" s="46"/>
       <c r="M9" s="47"/>
-      <c r="N9" s="169"/>
-      <c r="O9" s="170"/>
+      <c r="N9" s="175"/>
+      <c r="O9" s="176"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3303,7 +3502,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="37"/>
-      <c r="C10" s="146" t="s">
+      <c r="C10" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="38"/>
@@ -3327,8 +3526,8 @@
       <c r="K10" s="49"/>
       <c r="L10" s="46"/>
       <c r="M10" s="47"/>
-      <c r="N10" s="169"/>
-      <c r="O10" s="170"/>
+      <c r="N10" s="175"/>
+      <c r="O10" s="176"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3336,7 +3535,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="37"/>
-      <c r="C11" s="146" t="s">
+      <c r="C11" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D11" s="38"/>
@@ -3360,8 +3559,8 @@
       <c r="K11" s="49"/>
       <c r="L11" s="46"/>
       <c r="M11" s="47"/>
-      <c r="N11" s="169"/>
-      <c r="O11" s="170"/>
+      <c r="N11" s="175"/>
+      <c r="O11" s="176"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3369,7 +3568,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="37"/>
-      <c r="C12" s="146" t="s">
+      <c r="C12" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="38"/>
@@ -3392,9 +3591,9 @@
       </c>
       <c r="K12" s="49"/>
       <c r="L12" s="46"/>
-      <c r="M12" s="153"/>
-      <c r="N12" s="171"/>
-      <c r="O12" s="172"/>
+      <c r="M12" s="128"/>
+      <c r="N12" s="177"/>
+      <c r="O12" s="178"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3402,7 +3601,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="37"/>
-      <c r="C13" s="146" t="s">
+      <c r="C13" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D13" s="38"/>
@@ -3424,10 +3623,10 @@
         <v/>
       </c>
       <c r="K13" s="49"/>
-      <c r="L13" s="155"/>
-      <c r="M13" s="156"/>
-      <c r="N13" s="182"/>
-      <c r="O13" s="183"/>
+      <c r="L13" s="130"/>
+      <c r="M13" s="131"/>
+      <c r="N13" s="188"/>
+      <c r="O13" s="189"/>
       <c r="P13" s="66"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3435,7 +3634,7 @@
         <v>7</v>
       </c>
       <c r="B14" s="37"/>
-      <c r="C14" s="146" t="s">
+      <c r="C14" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="38"/>
@@ -3458,9 +3657,9 @@
       </c>
       <c r="K14" s="49"/>
       <c r="L14" s="46"/>
-      <c r="M14" s="154"/>
-      <c r="N14" s="184"/>
-      <c r="O14" s="185"/>
+      <c r="M14" s="129"/>
+      <c r="N14" s="190"/>
+      <c r="O14" s="191"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3468,7 +3667,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="37"/>
-      <c r="C15" s="146" t="s">
+      <c r="C15" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D15" s="38"/>
@@ -3492,8 +3691,8 @@
       <c r="K15" s="49"/>
       <c r="L15" s="46"/>
       <c r="M15" s="47"/>
-      <c r="N15" s="169"/>
-      <c r="O15" s="170"/>
+      <c r="N15" s="175"/>
+      <c r="O15" s="176"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3501,7 +3700,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="37"/>
-      <c r="C16" s="146" t="s">
+      <c r="C16" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="38"/>
@@ -3525,8 +3724,8 @@
       <c r="K16" s="49"/>
       <c r="L16" s="46"/>
       <c r="M16" s="47"/>
-      <c r="N16" s="169"/>
-      <c r="O16" s="170"/>
+      <c r="N16" s="175"/>
+      <c r="O16" s="176"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3534,7 +3733,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="37"/>
-      <c r="C17" s="146" t="s">
+      <c r="C17" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="38"/>
@@ -3558,8 +3757,8 @@
       <c r="K17" s="49"/>
       <c r="L17" s="46"/>
       <c r="M17" s="47"/>
-      <c r="N17" s="169"/>
-      <c r="O17" s="170"/>
+      <c r="N17" s="175"/>
+      <c r="O17" s="176"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3567,7 +3766,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="37"/>
-      <c r="C18" s="146" t="s">
+      <c r="C18" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D18" s="38"/>
@@ -3591,8 +3790,8 @@
       <c r="K18" s="49"/>
       <c r="L18" s="46"/>
       <c r="M18" s="47"/>
-      <c r="N18" s="169"/>
-      <c r="O18" s="170"/>
+      <c r="N18" s="175"/>
+      <c r="O18" s="176"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3600,7 +3799,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="37"/>
-      <c r="C19" s="146" t="s">
+      <c r="C19" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="38"/>
@@ -3624,8 +3823,8 @@
       <c r="K19" s="49"/>
       <c r="L19" s="46"/>
       <c r="M19" s="47"/>
-      <c r="N19" s="169"/>
-      <c r="O19" s="170"/>
+      <c r="N19" s="175"/>
+      <c r="O19" s="176"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3633,7 +3832,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="37"/>
-      <c r="C20" s="146" t="s">
+      <c r="C20" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="38"/>
@@ -3657,8 +3856,8 @@
       <c r="K20" s="49"/>
       <c r="L20" s="46"/>
       <c r="M20" s="47"/>
-      <c r="N20" s="169"/>
-      <c r="O20" s="170"/>
+      <c r="N20" s="175"/>
+      <c r="O20" s="176"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3666,7 +3865,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="37"/>
-      <c r="C21" s="146" t="s">
+      <c r="C21" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="38"/>
@@ -3690,8 +3889,8 @@
       <c r="K21" s="49"/>
       <c r="L21" s="46"/>
       <c r="M21" s="47"/>
-      <c r="N21" s="169"/>
-      <c r="O21" s="170"/>
+      <c r="N21" s="175"/>
+      <c r="O21" s="176"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3699,7 +3898,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="37"/>
-      <c r="C22" s="146" t="s">
+      <c r="C22" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D22" s="38"/>
@@ -3723,8 +3922,8 @@
       <c r="K22" s="49"/>
       <c r="L22" s="46"/>
       <c r="M22" s="47"/>
-      <c r="N22" s="169"/>
-      <c r="O22" s="170"/>
+      <c r="N22" s="175"/>
+      <c r="O22" s="176"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3732,7 +3931,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="37"/>
-      <c r="C23" s="146" t="s">
+      <c r="C23" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D23" s="38"/>
@@ -3756,8 +3955,8 @@
       <c r="K23" s="49"/>
       <c r="L23" s="46"/>
       <c r="M23" s="47"/>
-      <c r="N23" s="169"/>
-      <c r="O23" s="170"/>
+      <c r="N23" s="175"/>
+      <c r="O23" s="176"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3765,7 +3964,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="37"/>
-      <c r="C24" s="146" t="s">
+      <c r="C24" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="38"/>
@@ -3789,8 +3988,8 @@
       <c r="K24" s="49"/>
       <c r="L24" s="46"/>
       <c r="M24" s="47"/>
-      <c r="N24" s="169"/>
-      <c r="O24" s="170"/>
+      <c r="N24" s="175"/>
+      <c r="O24" s="176"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3798,7 +3997,7 @@
         <v>18</v>
       </c>
       <c r="B25" s="37"/>
-      <c r="C25" s="146" t="s">
+      <c r="C25" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="38"/>
@@ -3822,8 +4021,8 @@
       <c r="K25" s="49"/>
       <c r="L25" s="46"/>
       <c r="M25" s="47"/>
-      <c r="N25" s="169"/>
-      <c r="O25" s="170"/>
+      <c r="N25" s="175"/>
+      <c r="O25" s="176"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3831,7 +4030,7 @@
         <v>19</v>
       </c>
       <c r="B26" s="37"/>
-      <c r="C26" s="146" t="s">
+      <c r="C26" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="38"/>
@@ -3855,8 +4054,8 @@
       <c r="K26" s="49"/>
       <c r="L26" s="46"/>
       <c r="M26" s="47"/>
-      <c r="N26" s="169"/>
-      <c r="O26" s="170"/>
+      <c r="N26" s="175"/>
+      <c r="O26" s="176"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3864,7 +4063,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="37"/>
-      <c r="C27" s="146" t="s">
+      <c r="C27" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="38"/>
@@ -3888,8 +4087,8 @@
       <c r="K27" s="49"/>
       <c r="L27" s="46"/>
       <c r="M27" s="47"/>
-      <c r="N27" s="169"/>
-      <c r="O27" s="170"/>
+      <c r="N27" s="175"/>
+      <c r="O27" s="176"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3897,7 +4096,7 @@
         <v>21</v>
       </c>
       <c r="B28" s="37"/>
-      <c r="C28" s="146" t="s">
+      <c r="C28" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D28" s="38"/>
@@ -3921,16 +4120,16 @@
       <c r="K28" s="49"/>
       <c r="L28" s="46"/>
       <c r="M28" s="47"/>
-      <c r="N28" s="169"/>
-      <c r="O28" s="170"/>
+      <c r="N28" s="175"/>
+      <c r="O28" s="176"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="36">
         <v>22</v>
       </c>
-      <c r="B29" s="157"/>
-      <c r="C29" s="146" t="s">
+      <c r="B29" s="132"/>
+      <c r="C29" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="38"/>
@@ -3954,16 +4153,16 @@
       <c r="K29" s="49"/>
       <c r="L29" s="46"/>
       <c r="M29" s="47"/>
-      <c r="N29" s="169"/>
-      <c r="O29" s="170"/>
+      <c r="N29" s="175"/>
+      <c r="O29" s="176"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="36">
         <v>23</v>
       </c>
-      <c r="B30" s="157"/>
-      <c r="C30" s="146" t="s">
+      <c r="B30" s="132"/>
+      <c r="C30" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D30" s="38"/>
@@ -3987,16 +4186,16 @@
       <c r="K30" s="49"/>
       <c r="L30" s="46"/>
       <c r="M30" s="47"/>
-      <c r="N30" s="169"/>
-      <c r="O30" s="170"/>
+      <c r="N30" s="175"/>
+      <c r="O30" s="176"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="36">
         <v>24</v>
       </c>
-      <c r="B31" s="157"/>
-      <c r="C31" s="146" t="s">
+      <c r="B31" s="163"/>
+      <c r="C31" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D31" s="38"/>
@@ -4020,16 +4219,16 @@
       <c r="K31" s="49"/>
       <c r="L31" s="46"/>
       <c r="M31" s="47"/>
-      <c r="N31" s="169"/>
-      <c r="O31" s="170"/>
+      <c r="N31" s="175"/>
+      <c r="O31" s="176"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="36">
         <v>25</v>
       </c>
-      <c r="B32" s="157"/>
-      <c r="C32" s="146" t="s">
+      <c r="B32" s="132"/>
+      <c r="C32" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D32" s="38"/>
@@ -4053,16 +4252,16 @@
       <c r="K32" s="49"/>
       <c r="L32" s="46"/>
       <c r="M32" s="47"/>
-      <c r="N32" s="169"/>
-      <c r="O32" s="170"/>
+      <c r="N32" s="175"/>
+      <c r="O32" s="176"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="36">
         <v>26</v>
       </c>
-      <c r="B33" s="157"/>
-      <c r="C33" s="146" t="s">
+      <c r="B33" s="132"/>
+      <c r="C33" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D33" s="38"/>
@@ -4086,8 +4285,8 @@
       <c r="K33" s="49"/>
       <c r="L33" s="46"/>
       <c r="M33" s="47"/>
-      <c r="N33" s="169"/>
-      <c r="O33" s="170"/>
+      <c r="N33" s="175"/>
+      <c r="O33" s="176"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4095,7 +4294,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="37"/>
-      <c r="C34" s="146" t="s">
+      <c r="C34" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D34" s="38"/>
@@ -4119,8 +4318,8 @@
       <c r="K34" s="49"/>
       <c r="L34" s="46"/>
       <c r="M34" s="47"/>
-      <c r="N34" s="169"/>
-      <c r="O34" s="170"/>
+      <c r="N34" s="175"/>
+      <c r="O34" s="176"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4128,7 +4327,7 @@
         <v>28</v>
       </c>
       <c r="B35" s="37"/>
-      <c r="C35" s="146" t="s">
+      <c r="C35" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="38"/>
@@ -4152,16 +4351,16 @@
       <c r="K35" s="49"/>
       <c r="L35" s="46"/>
       <c r="M35" s="47"/>
-      <c r="N35" s="169"/>
-      <c r="O35" s="170"/>
+      <c r="N35" s="175"/>
+      <c r="O35" s="176"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="36">
         <v>29</v>
       </c>
-      <c r="B36" s="157"/>
-      <c r="C36" s="146" t="s">
+      <c r="B36" s="132"/>
+      <c r="C36" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D36" s="38"/>
@@ -4185,16 +4384,16 @@
       <c r="K36" s="49"/>
       <c r="L36" s="46"/>
       <c r="M36" s="47"/>
-      <c r="N36" s="169"/>
-      <c r="O36" s="170"/>
+      <c r="N36" s="175"/>
+      <c r="O36" s="176"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="36">
         <v>30</v>
       </c>
-      <c r="B37" s="157"/>
-      <c r="C37" s="146" t="s">
+      <c r="B37" s="132"/>
+      <c r="C37" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D37" s="38"/>
@@ -4218,16 +4417,16 @@
       <c r="K37" s="49"/>
       <c r="L37" s="46"/>
       <c r="M37" s="47"/>
-      <c r="N37" s="169"/>
-      <c r="O37" s="170"/>
+      <c r="N37" s="175"/>
+      <c r="O37" s="176"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="36">
         <v>31</v>
       </c>
-      <c r="B38" s="157"/>
-      <c r="C38" s="146" t="s">
+      <c r="B38" s="132"/>
+      <c r="C38" s="121" t="s">
         <v>27</v>
       </c>
       <c r="D38" s="41"/>
@@ -4235,7 +4434,7 @@
         <f t="array" ref="E38">IF(ISBLANK(D38),"","12.00")</f>
         <v/>
       </c>
-      <c r="F38" s="148" t="s">
+      <c r="F38" s="123" t="s">
         <v>27</v>
       </c>
       <c r="G38" s="41" t="str" cm="1">
@@ -4251,8 +4450,8 @@
       <c r="K38" s="55"/>
       <c r="L38" s="46"/>
       <c r="M38" s="47"/>
-      <c r="N38" s="169"/>
-      <c r="O38" s="170"/>
+      <c r="N38" s="175"/>
+      <c r="O38" s="176"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4262,12 +4461,12 @@
       <c r="B39" s="57"/>
       <c r="C39" s="57"/>
       <c r="D39" s="57"/>
-      <c r="E39" s="150"/>
-      <c r="F39" s="151" t="s">
+      <c r="E39" s="125"/>
+      <c r="F39" s="126" t="s">
         <v>29</v>
       </c>
-      <c r="G39" s="152"/>
-      <c r="H39" s="147" cm="1">
+      <c r="G39" s="127"/>
+      <c r="H39" s="122" cm="1">
         <f t="array" ref="H39">SUM(H8:H38)</f>
         <v>0</v>
       </c>
@@ -4279,21 +4478,21 @@
         <f t="array" ref="J39">SUM(J8:J38)</f>
         <v>0</v>
       </c>
-      <c r="K39" s="42" cm="1">
+      <c r="K39" s="198" cm="1">
         <f t="array" ref="K39">SUM(K8:K38)</f>
         <v>0</v>
       </c>
-      <c r="L39" s="42" cm="1">
+      <c r="L39" s="199" cm="1">
         <f t="array" ref="L39">SUM(L8:L38)</f>
         <v>0</v>
       </c>
       <c r="M39" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="N39" s="173" t="s">
+      <c r="N39" s="179" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="170"/>
+      <c r="O39" s="176"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4301,9 +4500,9 @@
       <c r="B40" s="60"/>
       <c r="C40" s="60"/>
       <c r="D40" s="60"/>
-      <c r="E40" s="149"/>
-      <c r="F40" s="149"/>
-      <c r="G40" s="149"/>
+      <c r="E40" s="124"/>
+      <c r="F40" s="124"/>
+      <c r="G40" s="124"/>
       <c r="H40" s="60"/>
       <c r="I40" s="60"/>
       <c r="J40" s="60"/>
@@ -4349,12 +4548,12 @@
       <c r="H42" s="69"/>
       <c r="I42" s="69"/>
       <c r="J42" s="70"/>
-      <c r="K42" s="71" cm="1">
-        <f t="array" ref="K42">H39-J39</f>
+      <c r="K42" s="144">
+        <f>H39-J39-K39</f>
         <v>0</v>
       </c>
-      <c r="L42" s="72"/>
-      <c r="M42" s="73" t="s">
+      <c r="L42" s="71"/>
+      <c r="M42" s="72" t="s">
         <v>32</v>
       </c>
       <c r="N42" s="2"/>
@@ -4362,24 +4561,24 @@
       <c r="P42" s="2"/>
     </row>
     <row r="43" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="74" t="s">
+      <c r="A43" s="73" t="s">
         <v>33</v>
       </c>
-      <c r="B43" s="75"/>
-      <c r="C43" s="75"/>
-      <c r="D43" s="75"/>
-      <c r="E43" s="75"/>
-      <c r="F43" s="75"/>
-      <c r="G43" s="75"/>
-      <c r="H43" s="76"/>
-      <c r="I43" s="76"/>
-      <c r="J43" s="77"/>
-      <c r="K43" s="78" cm="1">
-        <f t="array" ref="K43">J39</f>
+      <c r="B43" s="74"/>
+      <c r="C43" s="74"/>
+      <c r="D43" s="74"/>
+      <c r="E43" s="74"/>
+      <c r="F43" s="74"/>
+      <c r="G43" s="74"/>
+      <c r="H43" s="75"/>
+      <c r="I43" s="75"/>
+      <c r="J43" s="76"/>
+      <c r="K43" s="145">
+        <f>J39</f>
         <v>0</v>
       </c>
-      <c r="L43" s="72"/>
-      <c r="M43" s="73" t="s">
+      <c r="L43" s="197"/>
+      <c r="M43" s="196" t="s">
         <v>34</v>
       </c>
       <c r="N43" s="2"/>
@@ -4387,24 +4586,24 @@
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="79" t="s">
+      <c r="A44" s="77" t="s">
         <v>35</v>
       </c>
-      <c r="B44" s="80"/>
-      <c r="C44" s="80"/>
-      <c r="D44" s="80"/>
-      <c r="E44" s="80"/>
-      <c r="F44" s="80"/>
-      <c r="G44" s="80"/>
-      <c r="H44" s="81"/>
-      <c r="I44" s="81"/>
-      <c r="J44" s="82"/>
-      <c r="K44" s="83" cm="1">
-        <f t="array" ref="K44">K39</f>
+      <c r="B44" s="78"/>
+      <c r="C44" s="78"/>
+      <c r="D44" s="78"/>
+      <c r="E44" s="78"/>
+      <c r="F44" s="78"/>
+      <c r="G44" s="78"/>
+      <c r="H44" s="79"/>
+      <c r="I44" s="79"/>
+      <c r="J44" s="80"/>
+      <c r="K44" s="146">
+        <f>K39</f>
         <v>0</v>
       </c>
-      <c r="L44" s="72"/>
-      <c r="M44" s="73" t="s">
+      <c r="L44" s="135"/>
+      <c r="M44" s="72" t="s">
         <v>36</v>
       </c>
       <c r="N44" s="2"/>
@@ -4412,24 +4611,24 @@
       <c r="P44" s="2"/>
     </row>
     <row r="45" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="84" t="s">
+      <c r="A45" s="81" t="s">
         <v>37</v>
       </c>
-      <c r="B45" s="85"/>
-      <c r="C45" s="85"/>
-      <c r="D45" s="85"/>
-      <c r="E45" s="85"/>
-      <c r="F45" s="85"/>
-      <c r="G45" s="85"/>
-      <c r="H45" s="86"/>
-      <c r="I45" s="86"/>
-      <c r="J45" s="87"/>
-      <c r="K45" s="88" cm="1">
-        <f t="array" ref="K45">H39</f>
+      <c r="B45" s="82"/>
+      <c r="C45" s="82"/>
+      <c r="D45" s="82"/>
+      <c r="E45" s="82"/>
+      <c r="F45" s="82"/>
+      <c r="G45" s="82"/>
+      <c r="H45" s="83"/>
+      <c r="I45" s="83"/>
+      <c r="J45" s="84"/>
+      <c r="K45" s="159">
+        <f>H39</f>
         <v>0</v>
       </c>
-      <c r="L45" s="72"/>
-      <c r="M45" s="73" t="s">
+      <c r="L45" s="71"/>
+      <c r="M45" s="72" t="s">
         <v>38</v>
       </c>
       <c r="N45" s="2"/>
@@ -4437,35 +4636,35 @@
       <c r="P45" s="2"/>
     </row>
     <row r="46" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="89"/>
-      <c r="B46" s="90"/>
-      <c r="C46" s="90"/>
-      <c r="D46" s="90"/>
-      <c r="E46" s="90"/>
-      <c r="F46" s="90"/>
-      <c r="G46" s="90"/>
-      <c r="H46" s="90"/>
-      <c r="I46" s="90"/>
-      <c r="J46" s="90"/>
-      <c r="K46" s="90"/>
+      <c r="A46" s="85"/>
+      <c r="B46" s="86"/>
+      <c r="C46" s="86"/>
+      <c r="D46" s="86"/>
+      <c r="E46" s="86"/>
+      <c r="F46" s="86"/>
+      <c r="G46" s="86"/>
+      <c r="H46" s="86"/>
+      <c r="I46" s="86"/>
+      <c r="J46" s="86"/>
+      <c r="K46" s="86"/>
       <c r="L46" s="66"/>
-      <c r="M46" s="73" t="s">
+      <c r="M46" s="72" t="s">
         <v>39</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
     </row>
-    <row r="47" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="91" t="s">
+    <row r="47" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="87" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="92"/>
-      <c r="C47" s="92"/>
-      <c r="D47" s="92"/>
-      <c r="E47" s="92"/>
-      <c r="F47" s="92"/>
-      <c r="G47" s="92"/>
+      <c r="B47" s="88"/>
+      <c r="C47" s="88"/>
+      <c r="D47" s="88"/>
+      <c r="E47" s="88"/>
+      <c r="F47" s="88"/>
+      <c r="G47" s="88"/>
       <c r="H47" s="64"/>
       <c r="I47" s="65" t="s">
         <v>41</v>
@@ -4477,7 +4676,7 @@
         <v>17</v>
       </c>
       <c r="L47" s="66"/>
-      <c r="M47" s="73" t="s">
+      <c r="M47" s="72" t="s">
         <v>43</v>
       </c>
       <c r="N47" s="2"/>
@@ -4491,23 +4690,23 @@
       <c r="B48" s="68"/>
       <c r="C48" s="68"/>
       <c r="D48" s="68"/>
-      <c r="E48" s="93"/>
-      <c r="F48" s="93"/>
-      <c r="G48" s="93"/>
-      <c r="H48" s="93"/>
-      <c r="I48" s="94" t="s">
+      <c r="E48" s="89"/>
+      <c r="F48" s="89"/>
+      <c r="G48" s="89"/>
+      <c r="H48" s="89"/>
+      <c r="I48" s="90" t="s">
         <v>29</v>
       </c>
-      <c r="J48" s="95" cm="1">
-        <f t="array" ref="J48">COUNTIF(H8:H38,"&gt;0")</f>
+      <c r="J48" s="147">
+        <f>K48/8</f>
         <v>0</v>
       </c>
-      <c r="K48" s="96" cm="1">
-        <f t="array" ref="K48">K42</f>
+      <c r="K48" s="154">
+        <f>K42</f>
         <v>0</v>
       </c>
-      <c r="L48" s="72"/>
-      <c r="M48" s="73" t="s">
+      <c r="L48" s="71"/>
+      <c r="M48" s="72" t="s">
         <v>45</v>
       </c>
       <c r="N48" s="2"/>
@@ -4515,297 +4714,318 @@
       <c r="P48" s="2"/>
     </row>
     <row r="49" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="74" t="s">
+      <c r="A49" s="73" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="75"/>
-      <c r="C49" s="75"/>
-      <c r="D49" s="75"/>
-      <c r="E49" s="97"/>
-      <c r="F49" s="97"/>
-      <c r="G49" s="97"/>
-      <c r="H49" s="97"/>
-      <c r="I49" s="98" t="s">
+      <c r="B49" s="74"/>
+      <c r="C49" s="74"/>
+      <c r="D49" s="74"/>
+      <c r="E49" s="92"/>
+      <c r="F49" s="92"/>
+      <c r="G49" s="92"/>
+      <c r="H49" s="92"/>
+      <c r="I49" s="93" t="s">
         <v>29</v>
       </c>
-      <c r="J49" s="99"/>
-      <c r="K49" s="100" cm="1">
-        <f t="array" ref="K49">I39</f>
+      <c r="J49" s="148">
+        <f>K49/8</f>
         <v>0</v>
       </c>
-      <c r="L49" s="72"/>
-      <c r="M49" s="73" t="s">
+      <c r="K49" s="155">
+        <f>I39</f>
+        <v>0</v>
+      </c>
+      <c r="L49" s="71"/>
+      <c r="M49" s="72" t="s">
         <v>47</v>
       </c>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
     </row>
-    <row r="50" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="79" t="s">
+    <row r="50" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="77" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="80"/>
-      <c r="C50" s="80"/>
-      <c r="D50" s="80"/>
-      <c r="E50" s="101"/>
-      <c r="F50" s="101"/>
-      <c r="G50" s="101"/>
-      <c r="H50" s="101"/>
-      <c r="I50" s="102" t="s">
+      <c r="B50" s="78"/>
+      <c r="C50" s="78"/>
+      <c r="D50" s="78"/>
+      <c r="E50" s="94"/>
+      <c r="F50" s="94"/>
+      <c r="G50" s="94"/>
+      <c r="H50" s="94"/>
+      <c r="I50" s="95" t="s">
         <v>29</v>
       </c>
-      <c r="J50" s="103" t="s">
+      <c r="J50" s="149" t="s">
         <v>29</v>
       </c>
-      <c r="K50" s="104" cm="1">
-        <f t="array" ref="K50">K39</f>
+      <c r="K50" s="156">
+        <f>K39</f>
         <v>0</v>
       </c>
-      <c r="L50" s="72"/>
-      <c r="M50" s="73" t="s">
+      <c r="L50" s="71"/>
+      <c r="M50" s="72" t="s">
         <v>49</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
     </row>
-    <row r="51" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="105" t="s">
+    <row r="51" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="96" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="85"/>
-      <c r="C51" s="85"/>
-      <c r="D51" s="85"/>
-      <c r="E51" s="106"/>
-      <c r="F51" s="106"/>
-      <c r="G51" s="106"/>
-      <c r="H51" s="106"/>
-      <c r="I51" s="107" t="s">
+      <c r="B51" s="82"/>
+      <c r="C51" s="82"/>
+      <c r="D51" s="82"/>
+      <c r="E51" s="97"/>
+      <c r="F51" s="97"/>
+      <c r="G51" s="97"/>
+      <c r="H51" s="97"/>
+      <c r="I51" s="98" t="s">
         <v>29</v>
       </c>
-      <c r="J51" s="108" cm="1">
-        <f t="array" ref="J51">J48+J49</f>
+      <c r="J51" s="150">
+        <f>SUM(J48:J49)</f>
         <v>0</v>
       </c>
-      <c r="K51" s="109" cm="1">
-        <f t="array" ref="K51">SUM(K48:K50)</f>
+      <c r="K51" s="157">
+        <f>SUM(K48:K50)</f>
         <v>0</v>
       </c>
-      <c r="L51" s="72"/>
-      <c r="M51" s="73" t="s">
+      <c r="L51" s="71"/>
+      <c r="M51" s="72" t="s">
         <v>51</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" s="2"/>
     </row>
-    <row r="52" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A52" s="67" t="s">
         <v>52</v>
       </c>
       <c r="B52" s="68"/>
       <c r="C52" s="68"/>
       <c r="D52" s="68"/>
-      <c r="E52" s="93"/>
-      <c r="F52" s="93"/>
-      <c r="G52" s="93"/>
-      <c r="H52" s="93"/>
-      <c r="I52" s="94" t="s">
+      <c r="E52" s="89"/>
+      <c r="F52" s="89"/>
+      <c r="G52" s="89"/>
+      <c r="H52" s="89"/>
+      <c r="I52" s="90" t="s">
         <v>29</v>
       </c>
-      <c r="J52" s="95">
+      <c r="J52" s="147">
+        <f>COUNTIF(L8:L38,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="K52" s="96">
+      <c r="K52" s="158">
+        <f>L39</f>
         <v>0</v>
       </c>
-      <c r="L52" s="72"/>
-      <c r="M52" s="7"/>
-      <c r="N52" s="7"/>
-      <c r="O52" s="7"/>
+      <c r="L52" s="71"/>
+      <c r="M52" s="137"/>
+      <c r="N52" s="137"/>
+      <c r="O52" s="137"/>
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="174" t="s">
+      <c r="A53" s="180" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="175"/>
-      <c r="C53" s="170"/>
-      <c r="D53" s="170"/>
-      <c r="E53" s="170"/>
-      <c r="F53" s="170"/>
-      <c r="G53" s="111"/>
-      <c r="H53" s="176"/>
-      <c r="I53" s="175"/>
-      <c r="J53" s="112" cm="1">
-        <f t="array" ref="J53">COUNTIF(B8:B38,"=D")</f>
+      <c r="B53" s="181"/>
+      <c r="C53" s="176"/>
+      <c r="D53" s="176"/>
+      <c r="E53" s="176"/>
+      <c r="F53" s="176"/>
+      <c r="G53" s="100"/>
+      <c r="H53" s="182"/>
+      <c r="I53" s="181"/>
+      <c r="J53" s="151">
+        <f>COUNTIF(C8:C38,"=D")</f>
         <v>0</v>
       </c>
-      <c r="K53" s="100" cm="1">
-        <f t="array" ref="K53">J53*8</f>
+      <c r="K53" s="155">
+        <f>J53*8</f>
         <v>0</v>
       </c>
-      <c r="L53" s="113"/>
-      <c r="M53" s="114" t="s">
+      <c r="L53" s="138"/>
+      <c r="M53" s="139" t="s">
         <v>54</v>
       </c>
-      <c r="N53" s="115" t="s">
+      <c r="N53" s="140" t="s">
         <v>55</v>
       </c>
-      <c r="O53" s="116" t="s">
+      <c r="O53" s="141" t="s">
         <v>56</v>
       </c>
-      <c r="P53" s="17"/>
+      <c r="P53" s="66"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="174" t="s">
+      <c r="A54" s="180" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="175"/>
-      <c r="C54" s="170"/>
-      <c r="D54" s="170"/>
-      <c r="E54" s="170"/>
-      <c r="F54" s="170"/>
-      <c r="G54" s="111"/>
-      <c r="H54" s="117"/>
-      <c r="I54" s="118"/>
-      <c r="J54" s="119">
+      <c r="B54" s="181"/>
+      <c r="C54" s="176"/>
+      <c r="D54" s="176"/>
+      <c r="E54" s="176"/>
+      <c r="F54" s="176"/>
+      <c r="G54" s="100"/>
+      <c r="H54" s="101"/>
+      <c r="I54" s="102"/>
+      <c r="J54" s="152">
+        <f>COUNTIF(C8:C38,"=Sv")</f>
         <v>0</v>
       </c>
-      <c r="K54" s="100" cm="1">
-        <f t="array" ref="K54">J54*8</f>
+      <c r="K54" s="155">
+        <f t="shared" ref="K54:K57" si="0">J54*8</f>
         <v>0</v>
       </c>
-      <c r="L54" s="113"/>
-      <c r="M54" s="114" t="s">
+      <c r="L54" s="138"/>
+      <c r="M54" s="142" t="s">
         <v>58</v>
       </c>
-      <c r="N54" s="120">
+      <c r="N54" s="161"/>
+      <c r="O54" s="194">
+        <f>N54*8</f>
         <v>0</v>
       </c>
-      <c r="O54" s="121" cm="1">
-        <f t="array" ref="O54">N54*8</f>
+      <c r="P54" s="66"/>
+    </row>
+    <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="180" t="s">
+        <v>59</v>
+      </c>
+      <c r="B55" s="181"/>
+      <c r="C55" s="176"/>
+      <c r="D55" s="176"/>
+      <c r="E55" s="176"/>
+      <c r="F55" s="176"/>
+      <c r="G55" s="100"/>
+      <c r="H55" s="101"/>
+      <c r="I55" s="102"/>
+      <c r="J55" s="148">
+        <f>COUNTIF(C8:C38,"=N")</f>
         <v>0</v>
       </c>
-      <c r="P54" s="17"/>
-    </row>
-    <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="174" t="s">
-        <v>59</v>
-      </c>
-      <c r="B55" s="175"/>
-      <c r="C55" s="170"/>
-      <c r="D55" s="170"/>
-      <c r="E55" s="170"/>
-      <c r="F55" s="170"/>
-      <c r="G55" s="111"/>
-      <c r="H55" s="117"/>
-      <c r="I55" s="118"/>
-      <c r="J55" s="99"/>
-      <c r="K55" s="122"/>
-      <c r="L55" s="113"/>
-      <c r="M55" s="114" t="s">
+      <c r="K55" s="155">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L55" s="138"/>
+      <c r="M55" s="142" t="s">
         <v>60</v>
       </c>
-      <c r="N55" s="123" cm="1">
-        <f t="array" ref="N55">J54</f>
+      <c r="N55" s="162">
+        <f>J54</f>
         <v>0</v>
       </c>
-      <c r="O55" s="124" cm="1">
-        <f t="array" ref="O55">K54</f>
+      <c r="O55" s="194">
+        <f>N55*8</f>
         <v>0</v>
       </c>
-      <c r="P55" s="17"/>
-    </row>
-    <row r="56" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="174" t="s">
+      <c r="P55" s="66"/>
+    </row>
+    <row r="56" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="180" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="175"/>
-      <c r="C56" s="170"/>
-      <c r="D56" s="170"/>
-      <c r="E56" s="170"/>
-      <c r="F56" s="170"/>
-      <c r="G56" s="111"/>
-      <c r="H56" s="117"/>
-      <c r="I56" s="118"/>
-      <c r="J56" s="99"/>
-      <c r="K56" s="122"/>
-      <c r="L56" s="113"/>
-      <c r="M56" s="114" t="s">
+      <c r="B56" s="181"/>
+      <c r="C56" s="176"/>
+      <c r="D56" s="176"/>
+      <c r="E56" s="176"/>
+      <c r="F56" s="176"/>
+      <c r="G56" s="100"/>
+      <c r="H56" s="101"/>
+      <c r="I56" s="102"/>
+      <c r="J56" s="148">
+        <f>COUNTIF(C8:C38,"=Oš")</f>
+        <v>0</v>
+      </c>
+      <c r="K56" s="155">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L56" s="138"/>
+      <c r="M56" s="143" t="s">
         <v>8</v>
       </c>
-      <c r="N56" s="125" cm="1">
-        <f t="array" ref="N56">SUM(N54:N55)</f>
+      <c r="N56" s="160">
+        <f>SUM(N54:N55)</f>
         <v>0</v>
       </c>
-      <c r="O56" s="126" cm="1">
-        <f t="array" ref="O56">SUM(O54:O55)</f>
+      <c r="O56" s="195">
+        <f>SUM(O54:O55)</f>
         <v>0</v>
       </c>
-      <c r="P56" s="17"/>
+      <c r="P56" s="66"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="174" t="s">
+      <c r="A57" s="180" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="175"/>
-      <c r="C57" s="170"/>
-      <c r="D57" s="170"/>
-      <c r="E57" s="170"/>
-      <c r="F57" s="170"/>
-      <c r="G57" s="111"/>
-      <c r="H57" s="117"/>
-      <c r="I57" s="118"/>
-      <c r="J57" s="99"/>
-      <c r="K57" s="122"/>
-      <c r="L57" s="72"/>
-      <c r="M57" s="62"/>
-      <c r="N57" s="62"/>
-      <c r="O57" s="62"/>
+      <c r="B57" s="181"/>
+      <c r="C57" s="176"/>
+      <c r="D57" s="176"/>
+      <c r="E57" s="176"/>
+      <c r="F57" s="176"/>
+      <c r="G57" s="100"/>
+      <c r="H57" s="101"/>
+      <c r="I57" s="102"/>
+      <c r="J57" s="148">
+        <f>COUNTIF(C8:C38,"=NP")</f>
+        <v>0</v>
+      </c>
+      <c r="K57" s="155">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="L57" s="71"/>
+      <c r="M57" s="136"/>
+      <c r="O57" s="136"/>
       <c r="P57" s="2"/>
     </row>
-    <row r="58" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="177" t="s">
+    <row r="58" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="183" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="178"/>
-      <c r="C58" s="178"/>
-      <c r="D58" s="178"/>
-      <c r="E58" s="178"/>
-      <c r="F58" s="178"/>
-      <c r="G58" s="128"/>
-      <c r="H58" s="128"/>
-      <c r="I58" s="129" t="s">
+      <c r="B58" s="184"/>
+      <c r="C58" s="184"/>
+      <c r="D58" s="184"/>
+      <c r="E58" s="184"/>
+      <c r="F58" s="184"/>
+      <c r="G58" s="104"/>
+      <c r="H58" s="104"/>
+      <c r="I58" s="105" t="s">
         <v>29</v>
       </c>
-      <c r="J58" s="130" cm="1">
-        <f t="array" ref="J58">SUM(J51:J57)</f>
+      <c r="J58" s="153">
+        <f>SUM(J48:J57)</f>
         <v>0</v>
       </c>
-      <c r="K58" s="104" cm="1">
-        <f t="array" ref="K58">SUM(K51:K57)</f>
+      <c r="K58" s="156">
+        <f>SUM(K48:K57)</f>
         <v>0</v>
       </c>
-      <c r="L58" s="72"/>
+      <c r="L58" s="71"/>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
     <row r="59" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="131"/>
-      <c r="B59" s="131"/>
-      <c r="C59" s="131"/>
-      <c r="D59" s="131"/>
-      <c r="E59" s="131"/>
-      <c r="F59" s="131"/>
-      <c r="G59" s="131"/>
-      <c r="H59" s="131"/>
-      <c r="I59" s="131"/>
-      <c r="J59" s="132"/>
-      <c r="K59" s="132"/>
+      <c r="A59" s="106"/>
+      <c r="B59" s="106"/>
+      <c r="C59" s="106"/>
+      <c r="D59" s="106"/>
+      <c r="E59" s="106"/>
+      <c r="F59" s="106"/>
+      <c r="G59" s="106"/>
+      <c r="H59" s="106"/>
+      <c r="I59" s="106"/>
+      <c r="J59" s="107"/>
+      <c r="K59" s="107"/>
       <c r="L59" s="2"/>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
@@ -4813,19 +5033,19 @@
       <c r="P59" s="2"/>
     </row>
     <row r="60" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="133" t="s">
+      <c r="A60" s="108" t="s">
         <v>63</v>
       </c>
-      <c r="B60" s="134"/>
-      <c r="C60" s="134"/>
-      <c r="D60" s="134"/>
-      <c r="E60" s="134"/>
-      <c r="F60" s="134"/>
-      <c r="G60" s="134"/>
-      <c r="H60" s="134"/>
-      <c r="I60" s="134"/>
-      <c r="J60" s="135"/>
-      <c r="K60" s="136" t="s">
+      <c r="B60" s="109"/>
+      <c r="C60" s="109"/>
+      <c r="D60" s="109"/>
+      <c r="E60" s="109"/>
+      <c r="F60" s="109"/>
+      <c r="G60" s="109"/>
+      <c r="H60" s="109"/>
+      <c r="I60" s="109"/>
+      <c r="J60" s="110"/>
+      <c r="K60" s="111" t="s">
         <v>17</v>
       </c>
       <c r="L60" s="2"/>
@@ -4835,117 +5055,115 @@
       <c r="P60" s="2"/>
     </row>
     <row r="61" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="137" t="s">
+      <c r="A61" s="112" t="s">
         <v>64</v>
       </c>
-      <c r="B61" s="138"/>
-      <c r="C61" s="138"/>
-      <c r="D61" s="138"/>
-      <c r="E61" s="139"/>
-      <c r="F61" s="139"/>
-      <c r="G61" s="139"/>
-      <c r="H61" s="139"/>
-      <c r="I61" s="139"/>
-      <c r="J61" s="140"/>
-      <c r="K61" s="96">
-        <v>0</v>
-      </c>
-      <c r="L61" s="72"/>
+      <c r="B61" s="113"/>
+      <c r="C61" s="113"/>
+      <c r="D61" s="113"/>
+      <c r="E61" s="114"/>
+      <c r="F61" s="114"/>
+      <c r="G61" s="114"/>
+      <c r="H61" s="114"/>
+      <c r="I61" s="114"/>
+      <c r="J61" s="115"/>
+      <c r="K61" s="91"/>
+      <c r="L61" s="71"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
     <row r="62" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="110" t="s">
+      <c r="A62" s="99" t="s">
         <v>65</v>
       </c>
-      <c r="B62" s="141"/>
-      <c r="C62" s="141"/>
-      <c r="D62" s="141"/>
-      <c r="E62" s="117"/>
-      <c r="F62" s="117"/>
-      <c r="G62" s="117"/>
-      <c r="H62" s="117"/>
-      <c r="I62" s="117"/>
-      <c r="J62" s="118"/>
-      <c r="K62" s="100" cm="1">
-        <f t="array" ref="K62">K49</f>
+      <c r="B62" s="116"/>
+      <c r="C62" s="116"/>
+      <c r="D62" s="116"/>
+      <c r="E62" s="101"/>
+      <c r="F62" s="101"/>
+      <c r="G62" s="101"/>
+      <c r="H62" s="101"/>
+      <c r="I62" s="101"/>
+      <c r="J62" s="102"/>
+      <c r="K62" s="192">
+        <f>I39</f>
         <v>0</v>
       </c>
-      <c r="L62" s="72"/>
+      <c r="L62" s="71"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
     </row>
     <row r="63" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="110" t="s">
+      <c r="A63" s="99" t="s">
         <v>66</v>
       </c>
-      <c r="B63" s="141"/>
-      <c r="C63" s="141"/>
-      <c r="D63" s="141"/>
-      <c r="E63" s="117"/>
-      <c r="F63" s="117"/>
-      <c r="G63" s="117"/>
-      <c r="H63" s="117"/>
-      <c r="I63" s="117"/>
-      <c r="J63" s="118"/>
-      <c r="K63" s="100" cm="1">
-        <f t="array" ref="K63">K43</f>
+      <c r="B63" s="116"/>
+      <c r="C63" s="116"/>
+      <c r="D63" s="116"/>
+      <c r="E63" s="101"/>
+      <c r="F63" s="101"/>
+      <c r="G63" s="101"/>
+      <c r="H63" s="101"/>
+      <c r="I63" s="101"/>
+      <c r="J63" s="102"/>
+      <c r="K63" s="192">
+        <f>J39</f>
         <v>0</v>
       </c>
-      <c r="L63" s="72"/>
-      <c r="M63" s="73" t="s">
+      <c r="L63" s="71"/>
+      <c r="M63" s="72" t="s">
         <v>67</v>
       </c>
-      <c r="N63" s="142"/>
-      <c r="O63" s="142"/>
+      <c r="N63" s="117"/>
+      <c r="O63" s="117"/>
       <c r="P63" s="2"/>
     </row>
     <row r="64" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="127" t="s">
+      <c r="A64" s="103" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="143"/>
-      <c r="C64" s="143"/>
-      <c r="D64" s="143"/>
-      <c r="E64" s="128"/>
-      <c r="F64" s="128"/>
-      <c r="G64" s="128"/>
-      <c r="H64" s="128"/>
-      <c r="I64" s="128"/>
-      <c r="J64" s="144"/>
-      <c r="K64" s="104" cm="1">
-        <f t="array" ref="K64">K61+K63-K62</f>
+      <c r="B64" s="118"/>
+      <c r="C64" s="118"/>
+      <c r="D64" s="118"/>
+      <c r="E64" s="104"/>
+      <c r="F64" s="104"/>
+      <c r="G64" s="104"/>
+      <c r="H64" s="104"/>
+      <c r="I64" s="104"/>
+      <c r="J64" s="119"/>
+      <c r="K64" s="193">
+        <f>K61+K63-K62</f>
         <v>0</v>
       </c>
-      <c r="L64" s="72"/>
-      <c r="M64" s="73" t="s">
+      <c r="L64" s="71"/>
+      <c r="M64" s="72" t="s">
         <v>69</v>
       </c>
-      <c r="N64" s="142"/>
-      <c r="O64" s="142"/>
+      <c r="N64" s="117"/>
+      <c r="O64" s="117"/>
       <c r="P64" s="2"/>
     </row>
     <row r="65" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="131"/>
-      <c r="B65" s="131"/>
-      <c r="C65" s="131"/>
-      <c r="D65" s="131"/>
-      <c r="E65" s="131"/>
-      <c r="F65" s="131"/>
-      <c r="G65" s="131"/>
-      <c r="H65" s="131"/>
-      <c r="I65" s="145"/>
-      <c r="J65" s="145"/>
-      <c r="K65" s="145"/>
-      <c r="L65" s="142"/>
+      <c r="A65" s="106"/>
+      <c r="B65" s="106"/>
+      <c r="C65" s="106"/>
+      <c r="D65" s="106"/>
+      <c r="E65" s="106"/>
+      <c r="F65" s="106"/>
+      <c r="G65" s="106"/>
+      <c r="H65" s="106"/>
+      <c r="I65" s="120"/>
+      <c r="J65" s="120"/>
+      <c r="K65" s="120"/>
+      <c r="L65" s="117"/>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
-      <c r="P65" s="142"/>
+      <c r="P65" s="117"/>
     </row>
   </sheetData>
   <mergeCells count="49">

</xml_diff>

<commit_message>
add time input component, NV modal dialog, and UI improvements
- Add TimeInput component with hour/minute selection and 30min step arrows
- Replace inline NV prompt with modal dialog
- Add beforeunload confirmation when modal is open
- Update signature position in XLSX export
- Use TimeInput for all time fields in timesheet and schedule

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3BE7CED-067A-034F-9547-F2041C5BD629}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{066C8D5C-E076-8D43-82E0-0746E3C760D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="680" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="evid.PD" sheetId="1" r:id="rId1"/>
@@ -1962,70 +1962,70 @@
     <xf numFmtId="49" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -2109,61 +2109,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>12</xdr:col>
-      <xdr:colOff>1356</xdr:colOff>
-      <xdr:row>57</xdr:row>
-      <xdr:rowOff>149225</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>5677</xdr:colOff>
-      <xdr:row>62</xdr:row>
-      <xdr:rowOff>57190</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Rukopis 124" descr="Rukopis 124">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4954356" y="9378950"/>
-          <a:ext cx="1388622" cy="717591"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="12700" cap="flat">
-          <a:noFill/>
-          <a:miter lim="400000"/>
-        </a:ln>
-        <a:effectLst/>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3236,9 +3181,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="170"/>
-      <c r="C1" s="171"/>
-      <c r="D1" s="171"/>
+      <c r="B1" s="198"/>
+      <c r="C1" s="174"/>
+      <c r="D1" s="174"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3255,49 +3200,49 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="186" t="s">
+      <c r="A2" s="175" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="171"/>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
+      <c r="B2" s="174"/>
+      <c r="C2" s="174"/>
+      <c r="D2" s="174"/>
+      <c r="E2" s="174"/>
+      <c r="F2" s="174"/>
+      <c r="G2" s="174"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="185" t="s">
+      <c r="L2" s="173" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="171"/>
+      <c r="M2" s="174"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="172" t="s">
+      <c r="A3" s="199" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="173"/>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
+      <c r="B3" s="172"/>
+      <c r="C3" s="172"/>
+      <c r="D3" s="172"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="187" t="s">
+      <c r="F3" s="176" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="173"/>
-      <c r="H3" s="173"/>
-      <c r="I3" s="173"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="173" t="str" cm="1">
+      <c r="L3" s="172" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="173"/>
-      <c r="N3" s="173"/>
+      <c r="M3" s="172"/>
+      <c r="N3" s="172"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3305,11 +3250,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="168" t="s">
+      <c r="B4" s="196" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="169"/>
-      <c r="D4" s="169"/>
+      <c r="C4" s="197"/>
+      <c r="D4" s="197"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3341,12 +3286,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="164"/>
-      <c r="C5" s="165"/>
-      <c r="D5" s="165"/>
-      <c r="E5" s="174"/>
-      <c r="F5" s="165"/>
-      <c r="G5" s="165"/>
+      <c r="B5" s="193"/>
+      <c r="C5" s="190"/>
+      <c r="D5" s="190"/>
+      <c r="E5" s="189"/>
+      <c r="F5" s="190"/>
+      <c r="G5" s="190"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3373,12 +3318,12 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="165"/>
-      <c r="C6" s="165"/>
-      <c r="D6" s="165"/>
-      <c r="E6" s="165"/>
-      <c r="F6" s="165"/>
-      <c r="G6" s="165"/>
+      <c r="B6" s="190"/>
+      <c r="C6" s="190"/>
+      <c r="D6" s="190"/>
+      <c r="E6" s="190"/>
+      <c r="F6" s="190"/>
+      <c r="G6" s="190"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
@@ -3397,11 +3342,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="28"/>
-      <c r="B7" s="166" t="s">
+      <c r="B7" s="194" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="167"/>
-      <c r="D7" s="167"/>
+      <c r="C7" s="195"/>
+      <c r="D7" s="195"/>
       <c r="E7" s="30"/>
       <c r="F7" s="29" t="s">
         <v>22</v>
@@ -3460,8 +3405,8 @@
       <c r="K8" s="45"/>
       <c r="L8" s="46"/>
       <c r="M8" s="47"/>
-      <c r="N8" s="175"/>
-      <c r="O8" s="176"/>
+      <c r="N8" s="177"/>
+      <c r="O8" s="178"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3493,8 +3438,8 @@
       <c r="K9" s="49"/>
       <c r="L9" s="46"/>
       <c r="M9" s="47"/>
-      <c r="N9" s="175"/>
-      <c r="O9" s="176"/>
+      <c r="N9" s="177"/>
+      <c r="O9" s="178"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3526,8 +3471,8 @@
       <c r="K10" s="49"/>
       <c r="L10" s="46"/>
       <c r="M10" s="47"/>
-      <c r="N10" s="175"/>
-      <c r="O10" s="176"/>
+      <c r="N10" s="177"/>
+      <c r="O10" s="178"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3559,8 +3504,8 @@
       <c r="K11" s="49"/>
       <c r="L11" s="46"/>
       <c r="M11" s="47"/>
-      <c r="N11" s="175"/>
-      <c r="O11" s="176"/>
+      <c r="N11" s="177"/>
+      <c r="O11" s="178"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3592,8 +3537,8 @@
       <c r="K12" s="49"/>
       <c r="L12" s="46"/>
       <c r="M12" s="128"/>
-      <c r="N12" s="177"/>
-      <c r="O12" s="178"/>
+      <c r="N12" s="191"/>
+      <c r="O12" s="192"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3625,8 +3570,8 @@
       <c r="K13" s="49"/>
       <c r="L13" s="130"/>
       <c r="M13" s="131"/>
-      <c r="N13" s="188"/>
-      <c r="O13" s="189"/>
+      <c r="N13" s="179"/>
+      <c r="O13" s="180"/>
       <c r="P13" s="66"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3658,8 +3603,8 @@
       <c r="K14" s="49"/>
       <c r="L14" s="46"/>
       <c r="M14" s="129"/>
-      <c r="N14" s="190"/>
-      <c r="O14" s="191"/>
+      <c r="N14" s="181"/>
+      <c r="O14" s="182"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3691,8 +3636,8 @@
       <c r="K15" s="49"/>
       <c r="L15" s="46"/>
       <c r="M15" s="47"/>
-      <c r="N15" s="175"/>
-      <c r="O15" s="176"/>
+      <c r="N15" s="177"/>
+      <c r="O15" s="178"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3724,8 +3669,8 @@
       <c r="K16" s="49"/>
       <c r="L16" s="46"/>
       <c r="M16" s="47"/>
-      <c r="N16" s="175"/>
-      <c r="O16" s="176"/>
+      <c r="N16" s="177"/>
+      <c r="O16" s="178"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3757,8 +3702,8 @@
       <c r="K17" s="49"/>
       <c r="L17" s="46"/>
       <c r="M17" s="47"/>
-      <c r="N17" s="175"/>
-      <c r="O17" s="176"/>
+      <c r="N17" s="177"/>
+      <c r="O17" s="178"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3790,8 +3735,8 @@
       <c r="K18" s="49"/>
       <c r="L18" s="46"/>
       <c r="M18" s="47"/>
-      <c r="N18" s="175"/>
-      <c r="O18" s="176"/>
+      <c r="N18" s="177"/>
+      <c r="O18" s="178"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3823,8 +3768,8 @@
       <c r="K19" s="49"/>
       <c r="L19" s="46"/>
       <c r="M19" s="47"/>
-      <c r="N19" s="175"/>
-      <c r="O19" s="176"/>
+      <c r="N19" s="177"/>
+      <c r="O19" s="178"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3856,8 +3801,8 @@
       <c r="K20" s="49"/>
       <c r="L20" s="46"/>
       <c r="M20" s="47"/>
-      <c r="N20" s="175"/>
-      <c r="O20" s="176"/>
+      <c r="N20" s="177"/>
+      <c r="O20" s="178"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3889,8 +3834,8 @@
       <c r="K21" s="49"/>
       <c r="L21" s="46"/>
       <c r="M21" s="47"/>
-      <c r="N21" s="175"/>
-      <c r="O21" s="176"/>
+      <c r="N21" s="177"/>
+      <c r="O21" s="178"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3922,8 +3867,8 @@
       <c r="K22" s="49"/>
       <c r="L22" s="46"/>
       <c r="M22" s="47"/>
-      <c r="N22" s="175"/>
-      <c r="O22" s="176"/>
+      <c r="N22" s="177"/>
+      <c r="O22" s="178"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3955,8 +3900,8 @@
       <c r="K23" s="49"/>
       <c r="L23" s="46"/>
       <c r="M23" s="47"/>
-      <c r="N23" s="175"/>
-      <c r="O23" s="176"/>
+      <c r="N23" s="177"/>
+      <c r="O23" s="178"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3988,8 +3933,8 @@
       <c r="K24" s="49"/>
       <c r="L24" s="46"/>
       <c r="M24" s="47"/>
-      <c r="N24" s="175"/>
-      <c r="O24" s="176"/>
+      <c r="N24" s="177"/>
+      <c r="O24" s="178"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4021,8 +3966,8 @@
       <c r="K25" s="49"/>
       <c r="L25" s="46"/>
       <c r="M25" s="47"/>
-      <c r="N25" s="175"/>
-      <c r="O25" s="176"/>
+      <c r="N25" s="177"/>
+      <c r="O25" s="178"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4054,8 +3999,8 @@
       <c r="K26" s="49"/>
       <c r="L26" s="46"/>
       <c r="M26" s="47"/>
-      <c r="N26" s="175"/>
-      <c r="O26" s="176"/>
+      <c r="N26" s="177"/>
+      <c r="O26" s="178"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4087,8 +4032,8 @@
       <c r="K27" s="49"/>
       <c r="L27" s="46"/>
       <c r="M27" s="47"/>
-      <c r="N27" s="175"/>
-      <c r="O27" s="176"/>
+      <c r="N27" s="177"/>
+      <c r="O27" s="178"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4120,8 +4065,8 @@
       <c r="K28" s="49"/>
       <c r="L28" s="46"/>
       <c r="M28" s="47"/>
-      <c r="N28" s="175"/>
-      <c r="O28" s="176"/>
+      <c r="N28" s="177"/>
+      <c r="O28" s="178"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4153,8 +4098,8 @@
       <c r="K29" s="49"/>
       <c r="L29" s="46"/>
       <c r="M29" s="47"/>
-      <c r="N29" s="175"/>
-      <c r="O29" s="176"/>
+      <c r="N29" s="177"/>
+      <c r="O29" s="178"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4186,8 +4131,8 @@
       <c r="K30" s="49"/>
       <c r="L30" s="46"/>
       <c r="M30" s="47"/>
-      <c r="N30" s="175"/>
-      <c r="O30" s="176"/>
+      <c r="N30" s="177"/>
+      <c r="O30" s="178"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4219,8 +4164,8 @@
       <c r="K31" s="49"/>
       <c r="L31" s="46"/>
       <c r="M31" s="47"/>
-      <c r="N31" s="175"/>
-      <c r="O31" s="176"/>
+      <c r="N31" s="177"/>
+      <c r="O31" s="178"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4252,8 +4197,8 @@
       <c r="K32" s="49"/>
       <c r="L32" s="46"/>
       <c r="M32" s="47"/>
-      <c r="N32" s="175"/>
-      <c r="O32" s="176"/>
+      <c r="N32" s="177"/>
+      <c r="O32" s="178"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4285,8 +4230,8 @@
       <c r="K33" s="49"/>
       <c r="L33" s="46"/>
       <c r="M33" s="47"/>
-      <c r="N33" s="175"/>
-      <c r="O33" s="176"/>
+      <c r="N33" s="177"/>
+      <c r="O33" s="178"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4318,8 +4263,8 @@
       <c r="K34" s="49"/>
       <c r="L34" s="46"/>
       <c r="M34" s="47"/>
-      <c r="N34" s="175"/>
-      <c r="O34" s="176"/>
+      <c r="N34" s="177"/>
+      <c r="O34" s="178"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4351,8 +4296,8 @@
       <c r="K35" s="49"/>
       <c r="L35" s="46"/>
       <c r="M35" s="47"/>
-      <c r="N35" s="175"/>
-      <c r="O35" s="176"/>
+      <c r="N35" s="177"/>
+      <c r="O35" s="178"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4384,8 +4329,8 @@
       <c r="K36" s="49"/>
       <c r="L36" s="46"/>
       <c r="M36" s="47"/>
-      <c r="N36" s="175"/>
-      <c r="O36" s="176"/>
+      <c r="N36" s="177"/>
+      <c r="O36" s="178"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4417,8 +4362,8 @@
       <c r="K37" s="49"/>
       <c r="L37" s="46"/>
       <c r="M37" s="47"/>
-      <c r="N37" s="175"/>
-      <c r="O37" s="176"/>
+      <c r="N37" s="177"/>
+      <c r="O37" s="178"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4450,8 +4395,8 @@
       <c r="K38" s="55"/>
       <c r="L38" s="46"/>
       <c r="M38" s="47"/>
-      <c r="N38" s="175"/>
-      <c r="O38" s="176"/>
+      <c r="N38" s="177"/>
+      <c r="O38" s="178"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4478,21 +4423,21 @@
         <f t="array" ref="J39">SUM(J8:J38)</f>
         <v>0</v>
       </c>
-      <c r="K39" s="198" cm="1">
+      <c r="K39" s="170" cm="1">
         <f t="array" ref="K39">SUM(K8:K38)</f>
         <v>0</v>
       </c>
-      <c r="L39" s="199" cm="1">
+      <c r="L39" s="171" cm="1">
         <f t="array" ref="L39">SUM(L8:L38)</f>
         <v>0</v>
       </c>
       <c r="M39" s="58" t="s">
         <v>29</v>
       </c>
-      <c r="N39" s="179" t="s">
+      <c r="N39" s="187" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="176"/>
+      <c r="O39" s="178"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4577,8 +4522,8 @@
         <f>J39</f>
         <v>0</v>
       </c>
-      <c r="L43" s="197"/>
-      <c r="M43" s="196" t="s">
+      <c r="L43" s="169"/>
+      <c r="M43" s="168" t="s">
         <v>34</v>
       </c>
       <c r="N43" s="2"/>
@@ -4831,17 +4776,17 @@
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="180" t="s">
+      <c r="A53" s="183" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="181"/>
-      <c r="C53" s="176"/>
-      <c r="D53" s="176"/>
-      <c r="E53" s="176"/>
-      <c r="F53" s="176"/>
+      <c r="B53" s="184"/>
+      <c r="C53" s="178"/>
+      <c r="D53" s="178"/>
+      <c r="E53" s="178"/>
+      <c r="F53" s="178"/>
       <c r="G53" s="100"/>
-      <c r="H53" s="182"/>
-      <c r="I53" s="181"/>
+      <c r="H53" s="188"/>
+      <c r="I53" s="184"/>
       <c r="J53" s="151">
         <f>COUNTIF(C8:C38,"=D")</f>
         <v>0</v>
@@ -4863,14 +4808,14 @@
       <c r="P53" s="66"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="180" t="s">
+      <c r="A54" s="183" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="181"/>
-      <c r="C54" s="176"/>
-      <c r="D54" s="176"/>
-      <c r="E54" s="176"/>
-      <c r="F54" s="176"/>
+      <c r="B54" s="184"/>
+      <c r="C54" s="178"/>
+      <c r="D54" s="178"/>
+      <c r="E54" s="178"/>
+      <c r="F54" s="178"/>
       <c r="G54" s="100"/>
       <c r="H54" s="101"/>
       <c r="I54" s="102"/>
@@ -4887,21 +4832,21 @@
         <v>58</v>
       </c>
       <c r="N54" s="161"/>
-      <c r="O54" s="194">
+      <c r="O54" s="166">
         <f>N54*8</f>
         <v>0</v>
       </c>
       <c r="P54" s="66"/>
     </row>
     <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="180" t="s">
+      <c r="A55" s="183" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="181"/>
-      <c r="C55" s="176"/>
-      <c r="D55" s="176"/>
-      <c r="E55" s="176"/>
-      <c r="F55" s="176"/>
+      <c r="B55" s="184"/>
+      <c r="C55" s="178"/>
+      <c r="D55" s="178"/>
+      <c r="E55" s="178"/>
+      <c r="F55" s="178"/>
       <c r="G55" s="100"/>
       <c r="H55" s="101"/>
       <c r="I55" s="102"/>
@@ -4921,21 +4866,21 @@
         <f>J54</f>
         <v>0</v>
       </c>
-      <c r="O55" s="194">
+      <c r="O55" s="166">
         <f>N55*8</f>
         <v>0</v>
       </c>
       <c r="P55" s="66"/>
     </row>
     <row r="56" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="180" t="s">
+      <c r="A56" s="183" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="181"/>
-      <c r="C56" s="176"/>
-      <c r="D56" s="176"/>
-      <c r="E56" s="176"/>
-      <c r="F56" s="176"/>
+      <c r="B56" s="184"/>
+      <c r="C56" s="178"/>
+      <c r="D56" s="178"/>
+      <c r="E56" s="178"/>
+      <c r="F56" s="178"/>
       <c r="G56" s="100"/>
       <c r="H56" s="101"/>
       <c r="I56" s="102"/>
@@ -4955,21 +4900,21 @@
         <f>SUM(N54:N55)</f>
         <v>0</v>
       </c>
-      <c r="O56" s="195">
+      <c r="O56" s="167">
         <f>SUM(O54:O55)</f>
         <v>0</v>
       </c>
       <c r="P56" s="66"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="180" t="s">
+      <c r="A57" s="183" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="181"/>
-      <c r="C57" s="176"/>
-      <c r="D57" s="176"/>
-      <c r="E57" s="176"/>
-      <c r="F57" s="176"/>
+      <c r="B57" s="184"/>
+      <c r="C57" s="178"/>
+      <c r="D57" s="178"/>
+      <c r="E57" s="178"/>
+      <c r="F57" s="178"/>
       <c r="G57" s="100"/>
       <c r="H57" s="101"/>
       <c r="I57" s="102"/>
@@ -4987,14 +4932,14 @@
       <c r="P57" s="2"/>
     </row>
     <row r="58" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="183" t="s">
+      <c r="A58" s="185" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="184"/>
-      <c r="C58" s="184"/>
-      <c r="D58" s="184"/>
-      <c r="E58" s="184"/>
-      <c r="F58" s="184"/>
+      <c r="B58" s="186"/>
+      <c r="C58" s="186"/>
+      <c r="D58" s="186"/>
+      <c r="E58" s="186"/>
+      <c r="F58" s="186"/>
       <c r="G58" s="104"/>
       <c r="H58" s="104"/>
       <c r="I58" s="105" t="s">
@@ -5087,7 +5032,7 @@
       <c r="H62" s="101"/>
       <c r="I62" s="101"/>
       <c r="J62" s="102"/>
-      <c r="K62" s="192">
+      <c r="K62" s="164">
         <f>I39</f>
         <v>0</v>
       </c>
@@ -5110,7 +5055,7 @@
       <c r="H63" s="101"/>
       <c r="I63" s="101"/>
       <c r="J63" s="102"/>
-      <c r="K63" s="192">
+      <c r="K63" s="164">
         <f>J39</f>
         <v>0</v>
       </c>
@@ -5135,7 +5080,7 @@
       <c r="H64" s="104"/>
       <c r="I64" s="104"/>
       <c r="J64" s="119"/>
-      <c r="K64" s="193">
+      <c r="K64" s="165">
         <f>K61+K63-K62</f>
         <v>0</v>
       </c>
@@ -5167,6 +5112,39 @@
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="B5:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="L3:N3"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="A2:G2"/>
@@ -5183,42 +5161,8 @@
     <mergeCell ref="N35:O35"/>
     <mergeCell ref="N30:O30"/>
     <mergeCell ref="N31:O31"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="E5:G6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="B5:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.59055100000000005" right="0.19685" top="0.59055100000000005" bottom="0" header="0.11811000000000001" footer="0.11811000000000001"/>
   <pageSetup scale="85" orientation="portrait"/>
-  <drawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
simplify pass time entry with auto-calculated end time
- Add "Od" column for specifying pass start time
- Auto-calculate passTo from passFrom + passHours
- Remove redundant Od-Do display column
- Reset pass times when hours are cleared

Co-Authored-By: Claude Opus 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{066C8D5C-E076-8D43-82E0-0746E3C760D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6046DEDE-F0C3-0B47-BA7B-4805B4142480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1982,50 +1982,50 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -3181,9 +3181,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="198"/>
-      <c r="C1" s="174"/>
-      <c r="D1" s="174"/>
+      <c r="B1" s="178"/>
+      <c r="C1" s="179"/>
+      <c r="D1" s="179"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3200,49 +3200,49 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="175" t="s">
+      <c r="A2" s="194" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="174"/>
-      <c r="C2" s="174"/>
-      <c r="D2" s="174"/>
-      <c r="E2" s="174"/>
-      <c r="F2" s="174"/>
-      <c r="G2" s="174"/>
+      <c r="B2" s="179"/>
+      <c r="C2" s="179"/>
+      <c r="D2" s="179"/>
+      <c r="E2" s="179"/>
+      <c r="F2" s="179"/>
+      <c r="G2" s="179"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="173" t="s">
+      <c r="L2" s="193" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="174"/>
+      <c r="M2" s="179"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="199" t="s">
+      <c r="A3" s="180" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="172"/>
-      <c r="C3" s="172"/>
-      <c r="D3" s="172"/>
+      <c r="B3" s="181"/>
+      <c r="C3" s="181"/>
+      <c r="D3" s="181"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="176" t="s">
+      <c r="F3" s="195" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
+      <c r="G3" s="181"/>
+      <c r="H3" s="181"/>
+      <c r="I3" s="181"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="172" t="str" cm="1">
+      <c r="L3" s="181" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="172"/>
-      <c r="N3" s="172"/>
+      <c r="M3" s="181"/>
+      <c r="N3" s="181"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3250,11 +3250,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="196" t="s">
+      <c r="B4" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="197"/>
-      <c r="D4" s="197"/>
+      <c r="C4" s="177"/>
+      <c r="D4" s="177"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3286,12 +3286,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="193"/>
-      <c r="C5" s="190"/>
-      <c r="D5" s="190"/>
-      <c r="E5" s="189"/>
-      <c r="F5" s="190"/>
-      <c r="G5" s="190"/>
+      <c r="B5" s="172"/>
+      <c r="C5" s="173"/>
+      <c r="D5" s="173"/>
+      <c r="E5" s="182"/>
+      <c r="F5" s="173"/>
+      <c r="G5" s="173"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3318,12 +3318,12 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="190"/>
-      <c r="C6" s="190"/>
-      <c r="D6" s="190"/>
-      <c r="E6" s="190"/>
-      <c r="F6" s="190"/>
-      <c r="G6" s="190"/>
+      <c r="B6" s="173"/>
+      <c r="C6" s="173"/>
+      <c r="D6" s="173"/>
+      <c r="E6" s="173"/>
+      <c r="F6" s="173"/>
+      <c r="G6" s="173"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
@@ -3342,11 +3342,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="28"/>
-      <c r="B7" s="194" t="s">
+      <c r="B7" s="174" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="195"/>
-      <c r="D7" s="195"/>
+      <c r="C7" s="175"/>
+      <c r="D7" s="175"/>
       <c r="E7" s="30"/>
       <c r="F7" s="29" t="s">
         <v>22</v>
@@ -3398,15 +3398,15 @@
       </c>
       <c r="H8" s="42"/>
       <c r="I8" s="43"/>
-      <c r="J8" s="44" t="str" cm="1">
-        <f t="array" ref="J8">IF(AND(ISNUMBER(H8),NOT(ISERROR(H8&gt;8)),H8&gt;8),H8-8,"")</f>
+      <c r="J8" s="44" t="str">
+        <f>IF(AND(ISNUMBER(H8),NOT(ISERROR(H8&gt;8)),H8&gt;8),H8-8,"")</f>
         <v/>
       </c>
       <c r="K8" s="45"/>
       <c r="L8" s="46"/>
       <c r="M8" s="47"/>
-      <c r="N8" s="177"/>
-      <c r="O8" s="178"/>
+      <c r="N8" s="183"/>
+      <c r="O8" s="184"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3438,8 +3438,8 @@
       <c r="K9" s="49"/>
       <c r="L9" s="46"/>
       <c r="M9" s="47"/>
-      <c r="N9" s="177"/>
-      <c r="O9" s="178"/>
+      <c r="N9" s="183"/>
+      <c r="O9" s="184"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3471,8 +3471,8 @@
       <c r="K10" s="49"/>
       <c r="L10" s="46"/>
       <c r="M10" s="47"/>
-      <c r="N10" s="177"/>
-      <c r="O10" s="178"/>
+      <c r="N10" s="183"/>
+      <c r="O10" s="184"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3504,8 +3504,8 @@
       <c r="K11" s="49"/>
       <c r="L11" s="46"/>
       <c r="M11" s="47"/>
-      <c r="N11" s="177"/>
-      <c r="O11" s="178"/>
+      <c r="N11" s="183"/>
+      <c r="O11" s="184"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3537,8 +3537,8 @@
       <c r="K12" s="49"/>
       <c r="L12" s="46"/>
       <c r="M12" s="128"/>
-      <c r="N12" s="191"/>
-      <c r="O12" s="192"/>
+      <c r="N12" s="185"/>
+      <c r="O12" s="186"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3570,8 +3570,8 @@
       <c r="K13" s="49"/>
       <c r="L13" s="130"/>
       <c r="M13" s="131"/>
-      <c r="N13" s="179"/>
-      <c r="O13" s="180"/>
+      <c r="N13" s="196"/>
+      <c r="O13" s="197"/>
       <c r="P13" s="66"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3603,8 +3603,8 @@
       <c r="K14" s="49"/>
       <c r="L14" s="46"/>
       <c r="M14" s="129"/>
-      <c r="N14" s="181"/>
-      <c r="O14" s="182"/>
+      <c r="N14" s="198"/>
+      <c r="O14" s="199"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3636,8 +3636,8 @@
       <c r="K15" s="49"/>
       <c r="L15" s="46"/>
       <c r="M15" s="47"/>
-      <c r="N15" s="177"/>
-      <c r="O15" s="178"/>
+      <c r="N15" s="183"/>
+      <c r="O15" s="184"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3669,8 +3669,8 @@
       <c r="K16" s="49"/>
       <c r="L16" s="46"/>
       <c r="M16" s="47"/>
-      <c r="N16" s="177"/>
-      <c r="O16" s="178"/>
+      <c r="N16" s="183"/>
+      <c r="O16" s="184"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3702,8 +3702,8 @@
       <c r="K17" s="49"/>
       <c r="L17" s="46"/>
       <c r="M17" s="47"/>
-      <c r="N17" s="177"/>
-      <c r="O17" s="178"/>
+      <c r="N17" s="183"/>
+      <c r="O17" s="184"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3735,8 +3735,8 @@
       <c r="K18" s="49"/>
       <c r="L18" s="46"/>
       <c r="M18" s="47"/>
-      <c r="N18" s="177"/>
-      <c r="O18" s="178"/>
+      <c r="N18" s="183"/>
+      <c r="O18" s="184"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3768,8 +3768,8 @@
       <c r="K19" s="49"/>
       <c r="L19" s="46"/>
       <c r="M19" s="47"/>
-      <c r="N19" s="177"/>
-      <c r="O19" s="178"/>
+      <c r="N19" s="183"/>
+      <c r="O19" s="184"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3801,8 +3801,8 @@
       <c r="K20" s="49"/>
       <c r="L20" s="46"/>
       <c r="M20" s="47"/>
-      <c r="N20" s="177"/>
-      <c r="O20" s="178"/>
+      <c r="N20" s="183"/>
+      <c r="O20" s="184"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3834,8 +3834,8 @@
       <c r="K21" s="49"/>
       <c r="L21" s="46"/>
       <c r="M21" s="47"/>
-      <c r="N21" s="177"/>
-      <c r="O21" s="178"/>
+      <c r="N21" s="183"/>
+      <c r="O21" s="184"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3867,8 +3867,8 @@
       <c r="K22" s="49"/>
       <c r="L22" s="46"/>
       <c r="M22" s="47"/>
-      <c r="N22" s="177"/>
-      <c r="O22" s="178"/>
+      <c r="N22" s="183"/>
+      <c r="O22" s="184"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3900,8 +3900,8 @@
       <c r="K23" s="49"/>
       <c r="L23" s="46"/>
       <c r="M23" s="47"/>
-      <c r="N23" s="177"/>
-      <c r="O23" s="178"/>
+      <c r="N23" s="183"/>
+      <c r="O23" s="184"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3933,8 +3933,8 @@
       <c r="K24" s="49"/>
       <c r="L24" s="46"/>
       <c r="M24" s="47"/>
-      <c r="N24" s="177"/>
-      <c r="O24" s="178"/>
+      <c r="N24" s="183"/>
+      <c r="O24" s="184"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3966,8 +3966,8 @@
       <c r="K25" s="49"/>
       <c r="L25" s="46"/>
       <c r="M25" s="47"/>
-      <c r="N25" s="177"/>
-      <c r="O25" s="178"/>
+      <c r="N25" s="183"/>
+      <c r="O25" s="184"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3999,8 +3999,8 @@
       <c r="K26" s="49"/>
       <c r="L26" s="46"/>
       <c r="M26" s="47"/>
-      <c r="N26" s="177"/>
-      <c r="O26" s="178"/>
+      <c r="N26" s="183"/>
+      <c r="O26" s="184"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4032,8 +4032,8 @@
       <c r="K27" s="49"/>
       <c r="L27" s="46"/>
       <c r="M27" s="47"/>
-      <c r="N27" s="177"/>
-      <c r="O27" s="178"/>
+      <c r="N27" s="183"/>
+      <c r="O27" s="184"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4065,8 +4065,8 @@
       <c r="K28" s="49"/>
       <c r="L28" s="46"/>
       <c r="M28" s="47"/>
-      <c r="N28" s="177"/>
-      <c r="O28" s="178"/>
+      <c r="N28" s="183"/>
+      <c r="O28" s="184"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4098,8 +4098,8 @@
       <c r="K29" s="49"/>
       <c r="L29" s="46"/>
       <c r="M29" s="47"/>
-      <c r="N29" s="177"/>
-      <c r="O29" s="178"/>
+      <c r="N29" s="183"/>
+      <c r="O29" s="184"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4131,8 +4131,8 @@
       <c r="K30" s="49"/>
       <c r="L30" s="46"/>
       <c r="M30" s="47"/>
-      <c r="N30" s="177"/>
-      <c r="O30" s="178"/>
+      <c r="N30" s="183"/>
+      <c r="O30" s="184"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4164,8 +4164,8 @@
       <c r="K31" s="49"/>
       <c r="L31" s="46"/>
       <c r="M31" s="47"/>
-      <c r="N31" s="177"/>
-      <c r="O31" s="178"/>
+      <c r="N31" s="183"/>
+      <c r="O31" s="184"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4197,8 +4197,8 @@
       <c r="K32" s="49"/>
       <c r="L32" s="46"/>
       <c r="M32" s="47"/>
-      <c r="N32" s="177"/>
-      <c r="O32" s="178"/>
+      <c r="N32" s="183"/>
+      <c r="O32" s="184"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4230,8 +4230,8 @@
       <c r="K33" s="49"/>
       <c r="L33" s="46"/>
       <c r="M33" s="47"/>
-      <c r="N33" s="177"/>
-      <c r="O33" s="178"/>
+      <c r="N33" s="183"/>
+      <c r="O33" s="184"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4263,8 +4263,8 @@
       <c r="K34" s="49"/>
       <c r="L34" s="46"/>
       <c r="M34" s="47"/>
-      <c r="N34" s="177"/>
-      <c r="O34" s="178"/>
+      <c r="N34" s="183"/>
+      <c r="O34" s="184"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4296,8 +4296,8 @@
       <c r="K35" s="49"/>
       <c r="L35" s="46"/>
       <c r="M35" s="47"/>
-      <c r="N35" s="177"/>
-      <c r="O35" s="178"/>
+      <c r="N35" s="183"/>
+      <c r="O35" s="184"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4329,8 +4329,8 @@
       <c r="K36" s="49"/>
       <c r="L36" s="46"/>
       <c r="M36" s="47"/>
-      <c r="N36" s="177"/>
-      <c r="O36" s="178"/>
+      <c r="N36" s="183"/>
+      <c r="O36" s="184"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4362,8 +4362,8 @@
       <c r="K37" s="49"/>
       <c r="L37" s="46"/>
       <c r="M37" s="47"/>
-      <c r="N37" s="177"/>
-      <c r="O37" s="178"/>
+      <c r="N37" s="183"/>
+      <c r="O37" s="184"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4395,8 +4395,8 @@
       <c r="K38" s="55"/>
       <c r="L38" s="46"/>
       <c r="M38" s="47"/>
-      <c r="N38" s="177"/>
-      <c r="O38" s="178"/>
+      <c r="N38" s="183"/>
+      <c r="O38" s="184"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4437,7 +4437,7 @@
       <c r="N39" s="187" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="178"/>
+      <c r="O39" s="184"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4776,17 +4776,17 @@
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="183" t="s">
+      <c r="A53" s="188" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="184"/>
-      <c r="C53" s="178"/>
-      <c r="D53" s="178"/>
-      <c r="E53" s="178"/>
-      <c r="F53" s="178"/>
+      <c r="B53" s="189"/>
+      <c r="C53" s="184"/>
+      <c r="D53" s="184"/>
+      <c r="E53" s="184"/>
+      <c r="F53" s="184"/>
       <c r="G53" s="100"/>
-      <c r="H53" s="188"/>
-      <c r="I53" s="184"/>
+      <c r="H53" s="190"/>
+      <c r="I53" s="189"/>
       <c r="J53" s="151">
         <f>COUNTIF(C8:C38,"=D")</f>
         <v>0</v>
@@ -4808,14 +4808,14 @@
       <c r="P53" s="66"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="183" t="s">
+      <c r="A54" s="188" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="184"/>
-      <c r="C54" s="178"/>
-      <c r="D54" s="178"/>
-      <c r="E54" s="178"/>
-      <c r="F54" s="178"/>
+      <c r="B54" s="189"/>
+      <c r="C54" s="184"/>
+      <c r="D54" s="184"/>
+      <c r="E54" s="184"/>
+      <c r="F54" s="184"/>
       <c r="G54" s="100"/>
       <c r="H54" s="101"/>
       <c r="I54" s="102"/>
@@ -4839,14 +4839,14 @@
       <c r="P54" s="66"/>
     </row>
     <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="183" t="s">
+      <c r="A55" s="188" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="184"/>
-      <c r="C55" s="178"/>
-      <c r="D55" s="178"/>
-      <c r="E55" s="178"/>
-      <c r="F55" s="178"/>
+      <c r="B55" s="189"/>
+      <c r="C55" s="184"/>
+      <c r="D55" s="184"/>
+      <c r="E55" s="184"/>
+      <c r="F55" s="184"/>
       <c r="G55" s="100"/>
       <c r="H55" s="101"/>
       <c r="I55" s="102"/>
@@ -4873,14 +4873,14 @@
       <c r="P55" s="66"/>
     </row>
     <row r="56" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="183" t="s">
+      <c r="A56" s="188" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="184"/>
-      <c r="C56" s="178"/>
-      <c r="D56" s="178"/>
-      <c r="E56" s="178"/>
-      <c r="F56" s="178"/>
+      <c r="B56" s="189"/>
+      <c r="C56" s="184"/>
+      <c r="D56" s="184"/>
+      <c r="E56" s="184"/>
+      <c r="F56" s="184"/>
       <c r="G56" s="100"/>
       <c r="H56" s="101"/>
       <c r="I56" s="102"/>
@@ -4907,14 +4907,14 @@
       <c r="P56" s="66"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="183" t="s">
+      <c r="A57" s="188" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="184"/>
-      <c r="C57" s="178"/>
-      <c r="D57" s="178"/>
-      <c r="E57" s="178"/>
-      <c r="F57" s="178"/>
+      <c r="B57" s="189"/>
+      <c r="C57" s="184"/>
+      <c r="D57" s="184"/>
+      <c r="E57" s="184"/>
+      <c r="F57" s="184"/>
       <c r="G57" s="100"/>
       <c r="H57" s="101"/>
       <c r="I57" s="102"/>
@@ -4932,25 +4932,25 @@
       <c r="P57" s="2"/>
     </row>
     <row r="58" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="185" t="s">
+      <c r="A58" s="191" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="186"/>
-      <c r="C58" s="186"/>
-      <c r="D58" s="186"/>
-      <c r="E58" s="186"/>
-      <c r="F58" s="186"/>
+      <c r="B58" s="192"/>
+      <c r="C58" s="192"/>
+      <c r="D58" s="192"/>
+      <c r="E58" s="192"/>
+      <c r="F58" s="192"/>
       <c r="G58" s="104"/>
       <c r="H58" s="104"/>
       <c r="I58" s="105" t="s">
         <v>29</v>
       </c>
       <c r="J58" s="153">
-        <f>SUM(J48:J57)</f>
+        <f>SUM(J51:J57)</f>
         <v>0</v>
       </c>
       <c r="K58" s="156">
-        <f>SUM(K48:K57)</f>
+        <f>SUM(K51:K57)</f>
         <v>0</v>
       </c>
       <c r="L58" s="71"/>
@@ -5112,39 +5112,6 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B5:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E5:G6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A58:F58"/>
     <mergeCell ref="L3:N3"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="A2:G2"/>
@@ -5161,6 +5128,39 @@
     <mergeCell ref="N35:O35"/>
     <mergeCell ref="N30:O30"/>
     <mergeCell ref="N31:O31"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="B5:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.59055100000000005" right="0.19685" top="0.59055100000000005" bottom="0" header="0.11811000000000001" footer="0.11811000000000001"/>
   <pageSetup scale="85" orientation="portrait"/>

</xml_diff>

<commit_message>
Implement PDF conversion using Python UNO script and enhance Excel export functionality
- Added a Python script to convert Excel files to PDF using LibreOffice with formula recalculation.
- Updated the PDF conversion method to include a fallback for different LibreOffice paths.
- Enhanced Excel export to force formula recalculation on load.
- Adjusted TimesheetTable component to disable input based on interruption type.
- Modified timesheet store logic to handle new interruption types and reset hours accordingly.
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6046DEDE-F0C3-0B47-BA7B-4805B4142480}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0C7D16-FC37-4948-ADC5-B8EA08727873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -361,7 +361,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="93">
+  <borders count="97">
     <border>
       <left/>
       <right/>
@@ -532,21 +532,6 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right style="medium">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
         <color indexed="8"/>
       </left>
       <right style="thin">
@@ -644,40 +629,10 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="9"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right style="thin">
-        <color indexed="9"/>
-      </right>
-      <top style="thin">
-        <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="9"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right style="medium">
-        <color indexed="8"/>
+        <color indexed="9"/>
+      </left>
+      <right style="thin">
+        <color indexed="9"/>
       </right>
       <top style="thin">
         <color indexed="8"/>
@@ -726,36 +681,6 @@
       </right>
       <top style="thin">
         <color indexed="8"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="8"/>
-      </left>
-      <right style="thin">
-        <color indexed="9"/>
-      </right>
-      <top style="thin">
-        <color indexed="9"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="8"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="9"/>
-      </left>
-      <right style="medium">
-        <color indexed="8"/>
-      </right>
-      <top style="thin">
-        <color indexed="9"/>
       </top>
       <bottom style="thin">
         <color indexed="8"/>
@@ -1641,11 +1566,146 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color indexed="8"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color theme="3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="8"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="thin">
+        <color theme="3"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="3"/>
+      </left>
+      <right style="medium">
+        <color indexed="8"/>
+      </right>
+      <top style="thin">
+        <color theme="3"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="8"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="200">
+  <cellXfs count="201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1680,352 +1740,355 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="41" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="2" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="52" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="58" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="55" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="63" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="65" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="44" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="39" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="2" borderId="48" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="57" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="61" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="62" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="9" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="63" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="64" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="65" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="61" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="62" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="69" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="70" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="75" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="80" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="81" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="82" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="80" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="81" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="83" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="84" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="85" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="86" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="88" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="56" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="3" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="55" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="40" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="77" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="72" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="78" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="73" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="51" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="89" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="46" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="84" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="1" fontId="11" fillId="0" borderId="79" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="1" fontId="11" fillId="0" borderId="74" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="87" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="82" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="90" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="36" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="86" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="71" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="73" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="74" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="72" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normální" xfId="0" builtinId="0"/>
@@ -3181,9 +3244,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="178"/>
-      <c r="C1" s="179"/>
-      <c r="D1" s="179"/>
+      <c r="B1" s="187"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3200,49 +3263,49 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="194" t="s">
+      <c r="A2" s="164" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="179"/>
-      <c r="C2" s="179"/>
-      <c r="D2" s="179"/>
-      <c r="E2" s="179"/>
-      <c r="F2" s="179"/>
-      <c r="G2" s="179"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
+      <c r="F2" s="163"/>
+      <c r="G2" s="163"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="193" t="s">
+      <c r="L2" s="162" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="179"/>
+      <c r="M2" s="163"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="180" t="s">
+      <c r="A3" s="188" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="181"/>
-      <c r="C3" s="181"/>
-      <c r="D3" s="181"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="161"/>
+      <c r="D3" s="161"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="195" t="s">
+      <c r="F3" s="165" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="181"/>
-      <c r="H3" s="181"/>
-      <c r="I3" s="181"/>
+      <c r="G3" s="161"/>
+      <c r="H3" s="161"/>
+      <c r="I3" s="161"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="181" t="str" cm="1">
+      <c r="L3" s="161" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="181"/>
-      <c r="N3" s="181"/>
+      <c r="M3" s="161"/>
+      <c r="N3" s="161"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3250,11 +3313,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="176" t="s">
+      <c r="B4" s="185" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="177"/>
-      <c r="D4" s="177"/>
+      <c r="C4" s="186"/>
+      <c r="D4" s="186"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3286,12 +3349,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="172"/>
-      <c r="C5" s="173"/>
-      <c r="D5" s="173"/>
-      <c r="E5" s="182"/>
-      <c r="F5" s="173"/>
-      <c r="G5" s="173"/>
+      <c r="B5" s="182"/>
+      <c r="C5" s="179"/>
+      <c r="D5" s="179"/>
+      <c r="E5" s="178"/>
+      <c r="F5" s="179"/>
+      <c r="G5" s="179"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3318,22 +3381,22 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="173"/>
-      <c r="C6" s="173"/>
-      <c r="D6" s="173"/>
-      <c r="E6" s="173"/>
-      <c r="F6" s="173"/>
-      <c r="G6" s="173"/>
+      <c r="B6" s="179"/>
+      <c r="C6" s="179"/>
+      <c r="D6" s="179"/>
+      <c r="E6" s="179"/>
+      <c r="F6" s="179"/>
+      <c r="G6" s="179"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
       <c r="I6" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="J6" s="133" t="s">
+      <c r="J6" s="122" t="s">
         <v>21</v>
       </c>
-      <c r="K6" s="134"/>
+      <c r="K6" s="123"/>
       <c r="L6" s="26"/>
       <c r="M6" s="18"/>
       <c r="N6" s="27"/>
@@ -3342,11 +3405,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="28"/>
-      <c r="B7" s="174" t="s">
+      <c r="B7" s="183" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="175"/>
-      <c r="D7" s="175"/>
+      <c r="C7" s="184"/>
+      <c r="D7" s="184"/>
       <c r="E7" s="30"/>
       <c r="F7" s="29" t="s">
         <v>22</v>
@@ -3381,7 +3444,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="37"/>
-      <c r="C8" s="121" t="s">
+      <c r="C8" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D8" s="38"/>
@@ -3397,24 +3460,24 @@
         <v/>
       </c>
       <c r="H8" s="42"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="44" t="str">
+      <c r="I8" s="189"/>
+      <c r="J8" s="190" t="str">
         <f>IF(AND(ISNUMBER(H8),NOT(ISERROR(H8&gt;8)),H8&gt;8),H8-8,"")</f>
         <v/>
       </c>
-      <c r="K8" s="45"/>
-      <c r="L8" s="46"/>
-      <c r="M8" s="47"/>
-      <c r="N8" s="183"/>
-      <c r="O8" s="184"/>
+      <c r="K8" s="191"/>
+      <c r="L8" s="43"/>
+      <c r="M8" s="44"/>
+      <c r="N8" s="166"/>
+      <c r="O8" s="167"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="36">
         <v>2</v>
       </c>
-      <c r="B9" s="132"/>
-      <c r="C9" s="121" t="s">
+      <c r="B9" s="121"/>
+      <c r="C9" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D9" s="38"/>
@@ -3429,17 +3492,17 @@
         <f t="array" ref="G9">IF(ISBLANK(D9),"","12.30")</f>
         <v/>
       </c>
-      <c r="H9" s="47"/>
-      <c r="I9" s="48"/>
-      <c r="J9" s="5" t="str" cm="1">
+      <c r="H9" s="44"/>
+      <c r="I9" s="192"/>
+      <c r="J9" s="193" t="str" cm="1">
         <f t="array" ref="J9">IF(AND(ISNUMBER(H9),NOT(ISERROR(H9&gt;8)),H9&gt;8),H9-8,"")</f>
         <v/>
       </c>
-      <c r="K9" s="49"/>
-      <c r="L9" s="46"/>
-      <c r="M9" s="47"/>
-      <c r="N9" s="183"/>
-      <c r="O9" s="184"/>
+      <c r="K9" s="194"/>
+      <c r="L9" s="43"/>
+      <c r="M9" s="44"/>
+      <c r="N9" s="166"/>
+      <c r="O9" s="167"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3447,7 +3510,7 @@
         <v>3</v>
       </c>
       <c r="B10" s="37"/>
-      <c r="C10" s="121" t="s">
+      <c r="C10" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D10" s="38"/>
@@ -3463,16 +3526,16 @@
         <v/>
       </c>
       <c r="H10" s="42"/>
-      <c r="I10" s="50"/>
-      <c r="J10" s="51" t="str" cm="1">
+      <c r="I10" s="195"/>
+      <c r="J10" s="196" t="str" cm="1">
         <f t="array" ref="J10">IF(AND(ISNUMBER(H10),NOT(ISERROR(H10&gt;8)),H10&gt;8),H10-8,"")</f>
         <v/>
       </c>
-      <c r="K10" s="49"/>
-      <c r="L10" s="46"/>
-      <c r="M10" s="47"/>
-      <c r="N10" s="183"/>
-      <c r="O10" s="184"/>
+      <c r="K10" s="194"/>
+      <c r="L10" s="43"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="166"/>
+      <c r="O10" s="167"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3480,7 +3543,7 @@
         <v>4</v>
       </c>
       <c r="B11" s="37"/>
-      <c r="C11" s="121" t="s">
+      <c r="C11" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D11" s="38"/>
@@ -3496,16 +3559,16 @@
         <v/>
       </c>
       <c r="H11" s="42"/>
-      <c r="I11" s="50"/>
-      <c r="J11" s="5" t="str" cm="1">
+      <c r="I11" s="195"/>
+      <c r="J11" s="193" t="str" cm="1">
         <f t="array" ref="J11">IF(AND(ISNUMBER(H11),NOT(ISERROR(H11&gt;8)),H11&gt;8),H11-8,"")</f>
         <v/>
       </c>
-      <c r="K11" s="49"/>
-      <c r="L11" s="46"/>
-      <c r="M11" s="47"/>
-      <c r="N11" s="183"/>
-      <c r="O11" s="184"/>
+      <c r="K11" s="194"/>
+      <c r="L11" s="43"/>
+      <c r="M11" s="44"/>
+      <c r="N11" s="166"/>
+      <c r="O11" s="167"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3513,7 +3576,7 @@
         <v>5</v>
       </c>
       <c r="B12" s="37"/>
-      <c r="C12" s="121" t="s">
+      <c r="C12" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="38"/>
@@ -3529,16 +3592,16 @@
         <v/>
       </c>
       <c r="H12" s="42"/>
-      <c r="I12" s="50"/>
-      <c r="J12" s="51" t="str" cm="1">
+      <c r="I12" s="195"/>
+      <c r="J12" s="196" t="str" cm="1">
         <f t="array" ref="J12">IF(AND(ISNUMBER(H12),NOT(ISERROR(H12&gt;8)),H12&gt;8),H12-8,"")</f>
         <v/>
       </c>
-      <c r="K12" s="49"/>
-      <c r="L12" s="46"/>
-      <c r="M12" s="128"/>
-      <c r="N12" s="185"/>
-      <c r="O12" s="186"/>
+      <c r="K12" s="194"/>
+      <c r="L12" s="43"/>
+      <c r="M12" s="117"/>
+      <c r="N12" s="180"/>
+      <c r="O12" s="181"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3546,7 +3609,7 @@
         <v>6</v>
       </c>
       <c r="B13" s="37"/>
-      <c r="C13" s="121" t="s">
+      <c r="C13" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D13" s="38"/>
@@ -3561,25 +3624,25 @@
         <f t="array" ref="G13">IF(ISBLANK(D13),"","12.30")</f>
         <v/>
       </c>
-      <c r="H13" s="47"/>
-      <c r="I13" s="50"/>
-      <c r="J13" s="5" t="str" cm="1">
+      <c r="H13" s="44"/>
+      <c r="I13" s="195"/>
+      <c r="J13" s="193" t="str" cm="1">
         <f t="array" ref="J13">IF(AND(ISNUMBER(H13),NOT(ISERROR(H13&gt;8)),H13&gt;8),H13-8,"")</f>
         <v/>
       </c>
-      <c r="K13" s="49"/>
-      <c r="L13" s="130"/>
-      <c r="M13" s="131"/>
-      <c r="N13" s="196"/>
-      <c r="O13" s="197"/>
-      <c r="P13" s="66"/>
+      <c r="K13" s="194"/>
+      <c r="L13" s="119"/>
+      <c r="M13" s="120"/>
+      <c r="N13" s="168"/>
+      <c r="O13" s="169"/>
+      <c r="P13" s="55"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="36">
         <v>7</v>
       </c>
       <c r="B14" s="37"/>
-      <c r="C14" s="121" t="s">
+      <c r="C14" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D14" s="38"/>
@@ -3594,17 +3657,17 @@
         <f t="array" ref="G14">IF(ISBLANK(D14),"","12.30")</f>
         <v/>
       </c>
-      <c r="H14" s="47"/>
-      <c r="I14" s="50"/>
-      <c r="J14" s="5" t="str" cm="1">
+      <c r="H14" s="44"/>
+      <c r="I14" s="195"/>
+      <c r="J14" s="193" t="str" cm="1">
         <f t="array" ref="J14">IF(AND(ISNUMBER(H14),NOT(ISERROR(H14&gt;8)),H14&gt;8),H14-8,"")</f>
         <v/>
       </c>
-      <c r="K14" s="49"/>
-      <c r="L14" s="46"/>
-      <c r="M14" s="129"/>
-      <c r="N14" s="198"/>
-      <c r="O14" s="199"/>
+      <c r="K14" s="194"/>
+      <c r="L14" s="43"/>
+      <c r="M14" s="118"/>
+      <c r="N14" s="170"/>
+      <c r="O14" s="171"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3612,7 +3675,7 @@
         <v>8</v>
       </c>
       <c r="B15" s="37"/>
-      <c r="C15" s="121" t="s">
+      <c r="C15" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D15" s="38"/>
@@ -3628,16 +3691,16 @@
         <v/>
       </c>
       <c r="H15" s="42"/>
-      <c r="I15" s="50"/>
-      <c r="J15" s="51" t="str" cm="1">
+      <c r="I15" s="195"/>
+      <c r="J15" s="196" t="str" cm="1">
         <f t="array" ref="J15">IF(AND(ISNUMBER(H15),NOT(ISERROR(H15&gt;8)),H15&gt;8),H15-8,"")</f>
         <v/>
       </c>
-      <c r="K15" s="49"/>
-      <c r="L15" s="46"/>
-      <c r="M15" s="47"/>
-      <c r="N15" s="183"/>
-      <c r="O15" s="184"/>
+      <c r="K15" s="194"/>
+      <c r="L15" s="43"/>
+      <c r="M15" s="44"/>
+      <c r="N15" s="166"/>
+      <c r="O15" s="167"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3645,7 +3708,7 @@
         <v>9</v>
       </c>
       <c r="B16" s="37"/>
-      <c r="C16" s="121" t="s">
+      <c r="C16" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D16" s="38"/>
@@ -3661,16 +3724,16 @@
         <v/>
       </c>
       <c r="H16" s="42"/>
-      <c r="I16" s="50"/>
-      <c r="J16" s="51" t="str" cm="1">
+      <c r="I16" s="195"/>
+      <c r="J16" s="196" t="str" cm="1">
         <f t="array" ref="J16">IF(AND(ISNUMBER(H16),NOT(ISERROR(H16&gt;8)),H16&gt;8),H16-8,"")</f>
         <v/>
       </c>
-      <c r="K16" s="49"/>
-      <c r="L16" s="46"/>
-      <c r="M16" s="47"/>
-      <c r="N16" s="183"/>
-      <c r="O16" s="184"/>
+      <c r="K16" s="194"/>
+      <c r="L16" s="43"/>
+      <c r="M16" s="44"/>
+      <c r="N16" s="166"/>
+      <c r="O16" s="167"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3678,7 +3741,7 @@
         <v>10</v>
       </c>
       <c r="B17" s="37"/>
-      <c r="C17" s="121" t="s">
+      <c r="C17" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D17" s="38"/>
@@ -3694,16 +3757,16 @@
         <v/>
       </c>
       <c r="H17" s="42"/>
-      <c r="I17" s="50"/>
-      <c r="J17" s="51" t="str" cm="1">
+      <c r="I17" s="195"/>
+      <c r="J17" s="196" t="str" cm="1">
         <f t="array" ref="J17">IF(AND(ISNUMBER(H17),NOT(ISERROR(H17&gt;8)),H17&gt;8),H17-8,"")</f>
         <v/>
       </c>
-      <c r="K17" s="49"/>
-      <c r="L17" s="46"/>
-      <c r="M17" s="47"/>
-      <c r="N17" s="183"/>
-      <c r="O17" s="184"/>
+      <c r="K17" s="194"/>
+      <c r="L17" s="43"/>
+      <c r="M17" s="44"/>
+      <c r="N17" s="166"/>
+      <c r="O17" s="167"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3711,7 +3774,7 @@
         <v>11</v>
       </c>
       <c r="B18" s="37"/>
-      <c r="C18" s="121" t="s">
+      <c r="C18" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D18" s="38"/>
@@ -3727,16 +3790,16 @@
         <v/>
       </c>
       <c r="H18" s="42"/>
-      <c r="I18" s="50"/>
-      <c r="J18" s="5" t="str" cm="1">
+      <c r="I18" s="195"/>
+      <c r="J18" s="193" t="str" cm="1">
         <f t="array" ref="J18">IF(AND(ISNUMBER(H18),NOT(ISERROR(H18&gt;8)),H18&gt;8),H18-8,"")</f>
         <v/>
       </c>
-      <c r="K18" s="49"/>
-      <c r="L18" s="46"/>
-      <c r="M18" s="47"/>
-      <c r="N18" s="183"/>
-      <c r="O18" s="184"/>
+      <c r="K18" s="194"/>
+      <c r="L18" s="43"/>
+      <c r="M18" s="44"/>
+      <c r="N18" s="166"/>
+      <c r="O18" s="167"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3744,7 +3807,7 @@
         <v>12</v>
       </c>
       <c r="B19" s="37"/>
-      <c r="C19" s="121" t="s">
+      <c r="C19" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D19" s="38"/>
@@ -3760,16 +3823,16 @@
         <v/>
       </c>
       <c r="H19" s="42"/>
-      <c r="I19" s="50"/>
-      <c r="J19" s="51" t="str" cm="1">
+      <c r="I19" s="195"/>
+      <c r="J19" s="196" t="str" cm="1">
         <f t="array" ref="J19">IF(AND(ISNUMBER(H19),NOT(ISERROR(H19&gt;8)),H19&gt;8),H19-8,"")</f>
         <v/>
       </c>
-      <c r="K19" s="49"/>
-      <c r="L19" s="46"/>
-      <c r="M19" s="47"/>
-      <c r="N19" s="183"/>
-      <c r="O19" s="184"/>
+      <c r="K19" s="194"/>
+      <c r="L19" s="43"/>
+      <c r="M19" s="44"/>
+      <c r="N19" s="166"/>
+      <c r="O19" s="167"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3777,7 +3840,7 @@
         <v>13</v>
       </c>
       <c r="B20" s="37"/>
-      <c r="C20" s="121" t="s">
+      <c r="C20" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D20" s="38"/>
@@ -3792,17 +3855,17 @@
         <f t="array" ref="G20">IF(ISBLANK(D20),"","12.30")</f>
         <v/>
       </c>
-      <c r="H20" s="47"/>
-      <c r="I20" s="52"/>
-      <c r="J20" s="5" t="str" cm="1">
+      <c r="H20" s="44"/>
+      <c r="I20" s="197"/>
+      <c r="J20" s="193" t="str" cm="1">
         <f t="array" ref="J20">IF(AND(ISNUMBER(H20),NOT(ISERROR(H20&gt;8)),H20&gt;8),H20-8,"")</f>
         <v/>
       </c>
-      <c r="K20" s="49"/>
-      <c r="L20" s="46"/>
-      <c r="M20" s="47"/>
-      <c r="N20" s="183"/>
-      <c r="O20" s="184"/>
+      <c r="K20" s="194"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="44"/>
+      <c r="N20" s="166"/>
+      <c r="O20" s="167"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3810,7 +3873,7 @@
         <v>14</v>
       </c>
       <c r="B21" s="37"/>
-      <c r="C21" s="121" t="s">
+      <c r="C21" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D21" s="38"/>
@@ -3825,17 +3888,17 @@
         <f t="array" ref="G21">IF(ISBLANK(D21),"","12.30")</f>
         <v/>
       </c>
-      <c r="H21" s="47"/>
-      <c r="I21" s="50"/>
-      <c r="J21" s="5" t="str" cm="1">
+      <c r="H21" s="44"/>
+      <c r="I21" s="195"/>
+      <c r="J21" s="193" t="str" cm="1">
         <f t="array" ref="J21">IF(AND(ISNUMBER(H21),NOT(ISERROR(H21&gt;8)),H21&gt;8),H21-8,"")</f>
         <v/>
       </c>
-      <c r="K21" s="49"/>
-      <c r="L21" s="46"/>
-      <c r="M21" s="47"/>
-      <c r="N21" s="183"/>
-      <c r="O21" s="184"/>
+      <c r="K21" s="194"/>
+      <c r="L21" s="43"/>
+      <c r="M21" s="44"/>
+      <c r="N21" s="166"/>
+      <c r="O21" s="167"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3843,7 +3906,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="37"/>
-      <c r="C22" s="121" t="s">
+      <c r="C22" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D22" s="38"/>
@@ -3859,16 +3922,16 @@
         <v/>
       </c>
       <c r="H22" s="42"/>
-      <c r="I22" s="50"/>
-      <c r="J22" s="51" t="str" cm="1">
+      <c r="I22" s="195"/>
+      <c r="J22" s="196" t="str" cm="1">
         <f t="array" ref="J22">IF(AND(ISNUMBER(H22),NOT(ISERROR(H22&gt;8)),H22&gt;8),H22-8,"")</f>
         <v/>
       </c>
-      <c r="K22" s="49"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="47"/>
-      <c r="N22" s="183"/>
-      <c r="O22" s="184"/>
+      <c r="K22" s="194"/>
+      <c r="L22" s="43"/>
+      <c r="M22" s="44"/>
+      <c r="N22" s="166"/>
+      <c r="O22" s="167"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3876,7 +3939,7 @@
         <v>16</v>
       </c>
       <c r="B23" s="37"/>
-      <c r="C23" s="121" t="s">
+      <c r="C23" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D23" s="38"/>
@@ -3892,16 +3955,16 @@
         <v/>
       </c>
       <c r="H23" s="42"/>
-      <c r="I23" s="50"/>
-      <c r="J23" s="5" t="str" cm="1">
+      <c r="I23" s="195"/>
+      <c r="J23" s="193" t="str" cm="1">
         <f t="array" ref="J23">IF(AND(ISNUMBER(H23),NOT(ISERROR(H23&gt;8)),H23&gt;8),H23-8,"")</f>
         <v/>
       </c>
-      <c r="K23" s="49"/>
-      <c r="L23" s="46"/>
-      <c r="M23" s="47"/>
-      <c r="N23" s="183"/>
-      <c r="O23" s="184"/>
+      <c r="K23" s="194"/>
+      <c r="L23" s="43"/>
+      <c r="M23" s="44"/>
+      <c r="N23" s="166"/>
+      <c r="O23" s="167"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3909,7 +3972,7 @@
         <v>17</v>
       </c>
       <c r="B24" s="37"/>
-      <c r="C24" s="121" t="s">
+      <c r="C24" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D24" s="38"/>
@@ -3925,16 +3988,16 @@
         <v/>
       </c>
       <c r="H24" s="42"/>
-      <c r="I24" s="50"/>
-      <c r="J24" s="51" t="str" cm="1">
+      <c r="I24" s="195"/>
+      <c r="J24" s="196" t="str" cm="1">
         <f t="array" ref="J24">IF(AND(ISNUMBER(H24),NOT(ISERROR(H24&gt;8)),H24&gt;8),H24-8,"")</f>
         <v/>
       </c>
-      <c r="K24" s="49"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="183"/>
-      <c r="O24" s="184"/>
+      <c r="K24" s="194"/>
+      <c r="L24" s="43"/>
+      <c r="M24" s="44"/>
+      <c r="N24" s="166"/>
+      <c r="O24" s="167"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3942,7 +4005,7 @@
         <v>18</v>
       </c>
       <c r="B25" s="37"/>
-      <c r="C25" s="121" t="s">
+      <c r="C25" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D25" s="38"/>
@@ -3958,16 +4021,16 @@
         <v/>
       </c>
       <c r="H25" s="42"/>
-      <c r="I25" s="50"/>
-      <c r="J25" s="5" t="str" cm="1">
+      <c r="I25" s="195"/>
+      <c r="J25" s="193" t="str" cm="1">
         <f t="array" ref="J25">IF(AND(ISNUMBER(H25),NOT(ISERROR(H25&gt;8)),H25&gt;8),H25-8,"")</f>
         <v/>
       </c>
-      <c r="K25" s="49"/>
-      <c r="L25" s="46"/>
-      <c r="M25" s="47"/>
-      <c r="N25" s="183"/>
-      <c r="O25" s="184"/>
+      <c r="K25" s="194"/>
+      <c r="L25" s="43"/>
+      <c r="M25" s="44"/>
+      <c r="N25" s="166"/>
+      <c r="O25" s="167"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3975,7 +4038,7 @@
         <v>19</v>
       </c>
       <c r="B26" s="37"/>
-      <c r="C26" s="121" t="s">
+      <c r="C26" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D26" s="38"/>
@@ -3991,16 +4054,16 @@
         <v/>
       </c>
       <c r="H26" s="42"/>
-      <c r="I26" s="50"/>
-      <c r="J26" s="5" t="str" cm="1">
+      <c r="I26" s="195"/>
+      <c r="J26" s="193" t="str" cm="1">
         <f t="array" ref="J26">IF(AND(ISNUMBER(H26),NOT(ISERROR(H26&gt;8)),H26&gt;8),H26-8,"")</f>
         <v/>
       </c>
-      <c r="K26" s="49"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="183"/>
-      <c r="O26" s="184"/>
+      <c r="K26" s="194"/>
+      <c r="L26" s="43"/>
+      <c r="M26" s="44"/>
+      <c r="N26" s="166"/>
+      <c r="O26" s="167"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4008,7 +4071,7 @@
         <v>20</v>
       </c>
       <c r="B27" s="37"/>
-      <c r="C27" s="121" t="s">
+      <c r="C27" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D27" s="38"/>
@@ -4023,17 +4086,17 @@
         <f t="array" ref="G27">IF(ISBLANK(D27),"","12.30")</f>
         <v/>
       </c>
-      <c r="H27" s="47"/>
-      <c r="I27" s="50"/>
-      <c r="J27" s="5" t="str" cm="1">
+      <c r="H27" s="44"/>
+      <c r="I27" s="195"/>
+      <c r="J27" s="193" t="str" cm="1">
         <f t="array" ref="J27">IF(AND(ISNUMBER(H27),NOT(ISERROR(H27&gt;8)),H27&gt;8),H27-8,"")</f>
         <v/>
       </c>
-      <c r="K27" s="49"/>
-      <c r="L27" s="46"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="183"/>
-      <c r="O27" s="184"/>
+      <c r="K27" s="194"/>
+      <c r="L27" s="43"/>
+      <c r="M27" s="44"/>
+      <c r="N27" s="166"/>
+      <c r="O27" s="167"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4041,7 +4104,7 @@
         <v>21</v>
       </c>
       <c r="B28" s="37"/>
-      <c r="C28" s="121" t="s">
+      <c r="C28" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D28" s="38"/>
@@ -4056,25 +4119,25 @@
         <f t="array" ref="G28">IF(ISBLANK(D28),"","12.30")</f>
         <v/>
       </c>
-      <c r="H28" s="47"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="5" t="str" cm="1">
+      <c r="H28" s="44"/>
+      <c r="I28" s="195"/>
+      <c r="J28" s="193" t="str" cm="1">
         <f t="array" ref="J28">IF(AND(ISNUMBER(H28),NOT(ISERROR(H28&gt;8)),H28&gt;8),H28-8,"")</f>
         <v/>
       </c>
-      <c r="K28" s="49"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="47"/>
-      <c r="N28" s="183"/>
-      <c r="O28" s="184"/>
+      <c r="K28" s="194"/>
+      <c r="L28" s="43"/>
+      <c r="M28" s="44"/>
+      <c r="N28" s="166"/>
+      <c r="O28" s="167"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="36">
         <v>22</v>
       </c>
-      <c r="B29" s="132"/>
-      <c r="C29" s="121" t="s">
+      <c r="B29" s="121"/>
+      <c r="C29" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="38"/>
@@ -4089,25 +4152,25 @@
         <f t="array" ref="G29">IF(ISBLANK(D29),"","12.30")</f>
         <v/>
       </c>
-      <c r="H29" s="47"/>
-      <c r="I29" s="48"/>
-      <c r="J29" s="5" t="str" cm="1">
+      <c r="H29" s="44"/>
+      <c r="I29" s="192"/>
+      <c r="J29" s="193" t="str" cm="1">
         <f t="array" ref="J29">IF(AND(ISNUMBER(H29),NOT(ISERROR(H29&gt;8)),H29&gt;8),H29-8,"")</f>
         <v/>
       </c>
-      <c r="K29" s="49"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="183"/>
-      <c r="O29" s="184"/>
+      <c r="K29" s="194"/>
+      <c r="L29" s="43"/>
+      <c r="M29" s="44"/>
+      <c r="N29" s="166"/>
+      <c r="O29" s="167"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="36">
         <v>23</v>
       </c>
-      <c r="B30" s="132"/>
-      <c r="C30" s="121" t="s">
+      <c r="B30" s="121"/>
+      <c r="C30" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D30" s="38"/>
@@ -4122,25 +4185,25 @@
         <f t="array" ref="G30">IF(ISBLANK(D30),"","12.30")</f>
         <v/>
       </c>
-      <c r="H30" s="47"/>
-      <c r="I30" s="48"/>
-      <c r="J30" s="5" t="str" cm="1">
+      <c r="H30" s="44"/>
+      <c r="I30" s="192"/>
+      <c r="J30" s="193" t="str" cm="1">
         <f t="array" ref="J30">IF(AND(ISNUMBER(H30),NOT(ISERROR(H30&gt;8)),H30&gt;8),H30-8,"")</f>
         <v/>
       </c>
-      <c r="K30" s="49"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="47"/>
-      <c r="N30" s="183"/>
-      <c r="O30" s="184"/>
+      <c r="K30" s="194"/>
+      <c r="L30" s="43"/>
+      <c r="M30" s="44"/>
+      <c r="N30" s="166"/>
+      <c r="O30" s="167"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="36">
         <v>24</v>
       </c>
-      <c r="B31" s="163"/>
-      <c r="C31" s="121" t="s">
+      <c r="B31" s="152"/>
+      <c r="C31" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D31" s="38"/>
@@ -4155,25 +4218,25 @@
         <f t="array" ref="G31">IF(ISBLANK(D31),"","12.30")</f>
         <v/>
       </c>
-      <c r="H31" s="47"/>
-      <c r="I31" s="50"/>
-      <c r="J31" s="5" t="str" cm="1">
+      <c r="H31" s="44"/>
+      <c r="I31" s="195"/>
+      <c r="J31" s="193" t="str" cm="1">
         <f t="array" ref="J31">IF(AND(ISNUMBER(H31),NOT(ISERROR(H31&gt;8)),H31&gt;8),H31-8,"")</f>
         <v/>
       </c>
-      <c r="K31" s="49"/>
-      <c r="L31" s="46"/>
-      <c r="M31" s="47"/>
-      <c r="N31" s="183"/>
-      <c r="O31" s="184"/>
+      <c r="K31" s="194"/>
+      <c r="L31" s="43"/>
+      <c r="M31" s="44"/>
+      <c r="N31" s="166"/>
+      <c r="O31" s="167"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="36">
         <v>25</v>
       </c>
-      <c r="B32" s="132"/>
-      <c r="C32" s="121" t="s">
+      <c r="B32" s="121"/>
+      <c r="C32" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D32" s="38"/>
@@ -4188,25 +4251,25 @@
         <f t="array" ref="G32">IF(ISBLANK(D32),"","12.30")</f>
         <v/>
       </c>
-      <c r="H32" s="47"/>
-      <c r="I32" s="50"/>
-      <c r="J32" s="5" t="str" cm="1">
+      <c r="H32" s="44"/>
+      <c r="I32" s="195"/>
+      <c r="J32" s="193" t="str" cm="1">
         <f t="array" ref="J32">IF(AND(ISNUMBER(H32),NOT(ISERROR(H32&gt;8)),H32&gt;8),H32-8,"")</f>
         <v/>
       </c>
-      <c r="K32" s="49"/>
-      <c r="L32" s="46"/>
-      <c r="M32" s="47"/>
-      <c r="N32" s="183"/>
-      <c r="O32" s="184"/>
+      <c r="K32" s="194"/>
+      <c r="L32" s="43"/>
+      <c r="M32" s="44"/>
+      <c r="N32" s="166"/>
+      <c r="O32" s="167"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="36">
         <v>26</v>
       </c>
-      <c r="B33" s="132"/>
-      <c r="C33" s="121" t="s">
+      <c r="B33" s="121"/>
+      <c r="C33" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D33" s="38"/>
@@ -4221,17 +4284,17 @@
         <f t="array" ref="G33">IF(ISBLANK(D33),"","12.30")</f>
         <v/>
       </c>
-      <c r="H33" s="47"/>
-      <c r="I33" s="50"/>
-      <c r="J33" s="5" t="str" cm="1">
+      <c r="H33" s="44"/>
+      <c r="I33" s="195"/>
+      <c r="J33" s="193" t="str" cm="1">
         <f t="array" ref="J33">IF(AND(ISNUMBER(H33),NOT(ISERROR(H33&gt;8)),H33&gt;8),H33-8,"")</f>
         <v/>
       </c>
-      <c r="K33" s="49"/>
-      <c r="L33" s="46"/>
-      <c r="M33" s="47"/>
-      <c r="N33" s="183"/>
-      <c r="O33" s="184"/>
+      <c r="K33" s="194"/>
+      <c r="L33" s="43"/>
+      <c r="M33" s="44"/>
+      <c r="N33" s="166"/>
+      <c r="O33" s="167"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4239,7 +4302,7 @@
         <v>27</v>
       </c>
       <c r="B34" s="37"/>
-      <c r="C34" s="121" t="s">
+      <c r="C34" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D34" s="38"/>
@@ -4254,17 +4317,17 @@
         <f t="array" ref="G34">IF(ISBLANK(D34),"","12.30")</f>
         <v/>
       </c>
-      <c r="H34" s="47"/>
-      <c r="I34" s="50"/>
-      <c r="J34" s="5" t="str" cm="1">
+      <c r="H34" s="44"/>
+      <c r="I34" s="195"/>
+      <c r="J34" s="193" t="str" cm="1">
         <f t="array" ref="J34">IF(AND(ISNUMBER(H34),NOT(ISERROR(H34&gt;8)),H34&gt;8),H34-8,"")</f>
         <v/>
       </c>
-      <c r="K34" s="49"/>
-      <c r="L34" s="46"/>
-      <c r="M34" s="47"/>
-      <c r="N34" s="183"/>
-      <c r="O34" s="184"/>
+      <c r="K34" s="194"/>
+      <c r="L34" s="43"/>
+      <c r="M34" s="44"/>
+      <c r="N34" s="166"/>
+      <c r="O34" s="167"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4272,7 +4335,7 @@
         <v>28</v>
       </c>
       <c r="B35" s="37"/>
-      <c r="C35" s="121" t="s">
+      <c r="C35" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D35" s="38"/>
@@ -4287,25 +4350,25 @@
         <f t="array" ref="G35">IF(ISBLANK(D35),"","12.30")</f>
         <v/>
       </c>
-      <c r="H35" s="47"/>
-      <c r="I35" s="50"/>
-      <c r="J35" s="5" t="str" cm="1">
+      <c r="H35" s="44"/>
+      <c r="I35" s="195"/>
+      <c r="J35" s="193" t="str" cm="1">
         <f t="array" ref="J35">IF(AND(ISNUMBER(H35),NOT(ISERROR(H35&gt;8)),H35&gt;8),H35-8,"")</f>
         <v/>
       </c>
-      <c r="K35" s="49"/>
-      <c r="L35" s="46"/>
-      <c r="M35" s="47"/>
-      <c r="N35" s="183"/>
-      <c r="O35" s="184"/>
+      <c r="K35" s="194"/>
+      <c r="L35" s="43"/>
+      <c r="M35" s="44"/>
+      <c r="N35" s="166"/>
+      <c r="O35" s="167"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="36">
         <v>29</v>
       </c>
-      <c r="B36" s="132"/>
-      <c r="C36" s="121" t="s">
+      <c r="B36" s="121"/>
+      <c r="C36" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D36" s="38"/>
@@ -4320,25 +4383,25 @@
         <f t="array" ref="G36">IF(ISBLANK(D36),"","12.30")</f>
         <v/>
       </c>
-      <c r="H36" s="47"/>
-      <c r="I36" s="48"/>
-      <c r="J36" s="5" t="str" cm="1">
+      <c r="H36" s="44"/>
+      <c r="I36" s="192"/>
+      <c r="J36" s="193" t="str" cm="1">
         <f t="array" ref="J36">IF(AND(ISNUMBER(H36),NOT(ISERROR(H36&gt;8)),H36&gt;8),H36-8,"")</f>
         <v/>
       </c>
-      <c r="K36" s="49"/>
-      <c r="L36" s="46"/>
-      <c r="M36" s="47"/>
-      <c r="N36" s="183"/>
-      <c r="O36" s="184"/>
+      <c r="K36" s="194"/>
+      <c r="L36" s="43"/>
+      <c r="M36" s="44"/>
+      <c r="N36" s="166"/>
+      <c r="O36" s="167"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="36">
         <v>30</v>
       </c>
-      <c r="B37" s="132"/>
-      <c r="C37" s="121" t="s">
+      <c r="B37" s="121"/>
+      <c r="C37" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D37" s="38"/>
@@ -4353,25 +4416,25 @@
         <f t="array" ref="G37">IF(ISBLANK(D37),"","12.30")</f>
         <v/>
       </c>
-      <c r="H37" s="47"/>
-      <c r="I37" s="48"/>
-      <c r="J37" s="5" t="str" cm="1">
+      <c r="H37" s="44"/>
+      <c r="I37" s="192"/>
+      <c r="J37" s="193" t="str" cm="1">
         <f t="array" ref="J37">IF(AND(ISNUMBER(H37),NOT(ISERROR(H37&gt;8)),H37&gt;8),H37-8,"")</f>
         <v/>
       </c>
-      <c r="K37" s="49"/>
-      <c r="L37" s="46"/>
-      <c r="M37" s="47"/>
-      <c r="N37" s="183"/>
-      <c r="O37" s="184"/>
+      <c r="K37" s="194"/>
+      <c r="L37" s="43"/>
+      <c r="M37" s="44"/>
+      <c r="N37" s="166"/>
+      <c r="O37" s="167"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="36">
         <v>31</v>
       </c>
-      <c r="B38" s="132"/>
-      <c r="C38" s="121" t="s">
+      <c r="B38" s="121"/>
+      <c r="C38" s="110" t="s">
         <v>27</v>
       </c>
       <c r="D38" s="41"/>
@@ -4379,39 +4442,39 @@
         <f t="array" ref="E38">IF(ISBLANK(D38),"","12.00")</f>
         <v/>
       </c>
-      <c r="F38" s="123" t="s">
+      <c r="F38" s="112" t="s">
         <v>27</v>
       </c>
       <c r="G38" s="41" t="str" cm="1">
         <f t="array" ref="G38">IF(ISBLANK(D38),"","12.30")</f>
         <v/>
       </c>
-      <c r="H38" s="47"/>
-      <c r="I38" s="53"/>
-      <c r="J38" s="54" t="str" cm="1">
+      <c r="H38" s="44"/>
+      <c r="I38" s="198"/>
+      <c r="J38" s="199" t="str" cm="1">
         <f t="array" ref="J38">IF(AND(ISNUMBER(H38),NOT(ISERROR(H38&gt;8)),H38&gt;8),H38-8,"")</f>
         <v/>
       </c>
-      <c r="K38" s="55"/>
-      <c r="L38" s="46"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="183"/>
-      <c r="O38" s="184"/>
+      <c r="K38" s="200"/>
+      <c r="L38" s="43"/>
+      <c r="M38" s="44"/>
+      <c r="N38" s="166"/>
+      <c r="O38" s="167"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="56" t="s">
+      <c r="A39" s="45" t="s">
         <v>28</v>
       </c>
-      <c r="B39" s="57"/>
-      <c r="C39" s="57"/>
-      <c r="D39" s="57"/>
-      <c r="E39" s="125"/>
-      <c r="F39" s="126" t="s">
+      <c r="B39" s="46"/>
+      <c r="C39" s="46"/>
+      <c r="D39" s="46"/>
+      <c r="E39" s="114"/>
+      <c r="F39" s="115" t="s">
         <v>29</v>
       </c>
-      <c r="G39" s="127"/>
-      <c r="H39" s="122" cm="1">
+      <c r="G39" s="116"/>
+      <c r="H39" s="111" cm="1">
         <f t="array" ref="H39">SUM(H8:H38)</f>
         <v>0</v>
       </c>
@@ -4423,82 +4486,82 @@
         <f t="array" ref="J39">SUM(J8:J38)</f>
         <v>0</v>
       </c>
-      <c r="K39" s="170" cm="1">
+      <c r="K39" s="159" cm="1">
         <f t="array" ref="K39">SUM(K8:K38)</f>
         <v>0</v>
       </c>
-      <c r="L39" s="171" cm="1">
+      <c r="L39" s="160" cm="1">
         <f t="array" ref="L39">SUM(L8:L38)</f>
         <v>0</v>
       </c>
-      <c r="M39" s="58" t="s">
+      <c r="M39" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="N39" s="187" t="s">
+      <c r="N39" s="176" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="184"/>
+      <c r="O39" s="167"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="59"/>
-      <c r="B40" s="60"/>
-      <c r="C40" s="60"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="124"/>
-      <c r="F40" s="124"/>
-      <c r="G40" s="124"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="60"/>
-      <c r="L40" s="61"/>
-      <c r="M40" s="62"/>
-      <c r="N40" s="62"/>
-      <c r="O40" s="62"/>
+      <c r="A40" s="48"/>
+      <c r="B40" s="49"/>
+      <c r="C40" s="49"/>
+      <c r="D40" s="49"/>
+      <c r="E40" s="113"/>
+      <c r="F40" s="113"/>
+      <c r="G40" s="113"/>
+      <c r="H40" s="49"/>
+      <c r="I40" s="49"/>
+      <c r="J40" s="49"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="50"/>
+      <c r="M40" s="51"/>
+      <c r="N40" s="51"/>
+      <c r="O40" s="51"/>
       <c r="P40" s="2"/>
     </row>
     <row r="41" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="63" t="s">
+      <c r="A41" s="52" t="s">
         <v>30</v>
       </c>
-      <c r="B41" s="64"/>
-      <c r="C41" s="64"/>
-      <c r="D41" s="64"/>
-      <c r="E41" s="64"/>
-      <c r="F41" s="64"/>
-      <c r="G41" s="64"/>
-      <c r="H41" s="64"/>
-      <c r="I41" s="64"/>
-      <c r="J41" s="64"/>
-      <c r="K41" s="65" t="s">
+      <c r="B41" s="53"/>
+      <c r="C41" s="53"/>
+      <c r="D41" s="53"/>
+      <c r="E41" s="53"/>
+      <c r="F41" s="53"/>
+      <c r="G41" s="53"/>
+      <c r="H41" s="53"/>
+      <c r="I41" s="53"/>
+      <c r="J41" s="53"/>
+      <c r="K41" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="L41" s="66"/>
+      <c r="L41" s="55"/>
       <c r="M41" s="2"/>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" s="2"/>
     </row>
     <row r="42" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="67" t="s">
+      <c r="A42" s="56" t="s">
         <v>31</v>
       </c>
-      <c r="B42" s="68"/>
-      <c r="C42" s="68"/>
-      <c r="D42" s="68"/>
-      <c r="E42" s="68"/>
-      <c r="F42" s="68"/>
-      <c r="G42" s="68"/>
-      <c r="H42" s="69"/>
-      <c r="I42" s="69"/>
-      <c r="J42" s="70"/>
-      <c r="K42" s="144">
+      <c r="B42" s="57"/>
+      <c r="C42" s="57"/>
+      <c r="D42" s="57"/>
+      <c r="E42" s="57"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="57"/>
+      <c r="H42" s="58"/>
+      <c r="I42" s="58"/>
+      <c r="J42" s="59"/>
+      <c r="K42" s="133">
         <f>H39-J39-K39</f>
         <v>0</v>
       </c>
-      <c r="L42" s="71"/>
-      <c r="M42" s="72" t="s">
+      <c r="L42" s="60"/>
+      <c r="M42" s="61" t="s">
         <v>32</v>
       </c>
       <c r="N42" s="2"/>
@@ -4506,24 +4569,24 @@
       <c r="P42" s="2"/>
     </row>
     <row r="43" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="73" t="s">
+      <c r="A43" s="62" t="s">
         <v>33</v>
       </c>
-      <c r="B43" s="74"/>
-      <c r="C43" s="74"/>
-      <c r="D43" s="74"/>
-      <c r="E43" s="74"/>
-      <c r="F43" s="74"/>
-      <c r="G43" s="74"/>
-      <c r="H43" s="75"/>
-      <c r="I43" s="75"/>
-      <c r="J43" s="76"/>
-      <c r="K43" s="145">
+      <c r="B43" s="63"/>
+      <c r="C43" s="63"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="63"/>
+      <c r="F43" s="63"/>
+      <c r="G43" s="63"/>
+      <c r="H43" s="64"/>
+      <c r="I43" s="64"/>
+      <c r="J43" s="65"/>
+      <c r="K43" s="134">
         <f>J39</f>
         <v>0</v>
       </c>
-      <c r="L43" s="169"/>
-      <c r="M43" s="168" t="s">
+      <c r="L43" s="158"/>
+      <c r="M43" s="157" t="s">
         <v>34</v>
       </c>
       <c r="N43" s="2"/>
@@ -4531,24 +4594,24 @@
       <c r="P43" s="2"/>
     </row>
     <row r="44" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="77" t="s">
+      <c r="A44" s="66" t="s">
         <v>35</v>
       </c>
-      <c r="B44" s="78"/>
-      <c r="C44" s="78"/>
-      <c r="D44" s="78"/>
-      <c r="E44" s="78"/>
-      <c r="F44" s="78"/>
-      <c r="G44" s="78"/>
-      <c r="H44" s="79"/>
-      <c r="I44" s="79"/>
-      <c r="J44" s="80"/>
-      <c r="K44" s="146">
+      <c r="B44" s="67"/>
+      <c r="C44" s="67"/>
+      <c r="D44" s="67"/>
+      <c r="E44" s="67"/>
+      <c r="F44" s="67"/>
+      <c r="G44" s="67"/>
+      <c r="H44" s="68"/>
+      <c r="I44" s="68"/>
+      <c r="J44" s="69"/>
+      <c r="K44" s="135">
         <f>K39</f>
         <v>0</v>
       </c>
-      <c r="L44" s="135"/>
-      <c r="M44" s="72" t="s">
+      <c r="L44" s="124"/>
+      <c r="M44" s="61" t="s">
         <v>36</v>
       </c>
       <c r="N44" s="2"/>
@@ -4556,24 +4619,24 @@
       <c r="P44" s="2"/>
     </row>
     <row r="45" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="81" t="s">
+      <c r="A45" s="70" t="s">
         <v>37</v>
       </c>
-      <c r="B45" s="82"/>
-      <c r="C45" s="82"/>
-      <c r="D45" s="82"/>
-      <c r="E45" s="82"/>
-      <c r="F45" s="82"/>
-      <c r="G45" s="82"/>
-      <c r="H45" s="83"/>
-      <c r="I45" s="83"/>
-      <c r="J45" s="84"/>
-      <c r="K45" s="159">
+      <c r="B45" s="71"/>
+      <c r="C45" s="71"/>
+      <c r="D45" s="71"/>
+      <c r="E45" s="71"/>
+      <c r="F45" s="71"/>
+      <c r="G45" s="71"/>
+      <c r="H45" s="72"/>
+      <c r="I45" s="72"/>
+      <c r="J45" s="73"/>
+      <c r="K45" s="148">
         <f>H39</f>
         <v>0</v>
       </c>
-      <c r="L45" s="71"/>
-      <c r="M45" s="72" t="s">
+      <c r="L45" s="60"/>
+      <c r="M45" s="61" t="s">
         <v>38</v>
       </c>
       <c r="N45" s="2"/>
@@ -4581,19 +4644,19 @@
       <c r="P45" s="2"/>
     </row>
     <row r="46" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="85"/>
-      <c r="B46" s="86"/>
-      <c r="C46" s="86"/>
-      <c r="D46" s="86"/>
-      <c r="E46" s="86"/>
-      <c r="F46" s="86"/>
-      <c r="G46" s="86"/>
-      <c r="H46" s="86"/>
-      <c r="I46" s="86"/>
-      <c r="J46" s="86"/>
-      <c r="K46" s="86"/>
-      <c r="L46" s="66"/>
-      <c r="M46" s="72" t="s">
+      <c r="A46" s="74"/>
+      <c r="B46" s="75"/>
+      <c r="C46" s="75"/>
+      <c r="D46" s="75"/>
+      <c r="E46" s="75"/>
+      <c r="F46" s="75"/>
+      <c r="G46" s="75"/>
+      <c r="H46" s="75"/>
+      <c r="I46" s="75"/>
+      <c r="J46" s="75"/>
+      <c r="K46" s="75"/>
+      <c r="L46" s="55"/>
+      <c r="M46" s="61" t="s">
         <v>39</v>
       </c>
       <c r="N46" s="2"/>
@@ -4601,27 +4664,27 @@
       <c r="P46" s="2"/>
     </row>
     <row r="47" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="87" t="s">
+      <c r="A47" s="76" t="s">
         <v>40</v>
       </c>
-      <c r="B47" s="88"/>
-      <c r="C47" s="88"/>
-      <c r="D47" s="88"/>
-      <c r="E47" s="88"/>
-      <c r="F47" s="88"/>
-      <c r="G47" s="88"/>
-      <c r="H47" s="64"/>
-      <c r="I47" s="65" t="s">
+      <c r="B47" s="77"/>
+      <c r="C47" s="77"/>
+      <c r="D47" s="77"/>
+      <c r="E47" s="77"/>
+      <c r="F47" s="77"/>
+      <c r="G47" s="77"/>
+      <c r="H47" s="53"/>
+      <c r="I47" s="54" t="s">
         <v>41</v>
       </c>
-      <c r="J47" s="65" t="s">
+      <c r="J47" s="54" t="s">
         <v>42</v>
       </c>
-      <c r="K47" s="65" t="s">
+      <c r="K47" s="54" t="s">
         <v>17</v>
       </c>
-      <c r="L47" s="66"/>
-      <c r="M47" s="72" t="s">
+      <c r="L47" s="55"/>
+      <c r="M47" s="61" t="s">
         <v>43</v>
       </c>
       <c r="N47" s="2"/>
@@ -4629,29 +4692,29 @@
       <c r="P47" s="2"/>
     </row>
     <row r="48" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="67" t="s">
+      <c r="A48" s="56" t="s">
         <v>44</v>
       </c>
-      <c r="B48" s="68"/>
-      <c r="C48" s="68"/>
-      <c r="D48" s="68"/>
-      <c r="E48" s="89"/>
-      <c r="F48" s="89"/>
-      <c r="G48" s="89"/>
-      <c r="H48" s="89"/>
-      <c r="I48" s="90" t="s">
+      <c r="B48" s="57"/>
+      <c r="C48" s="57"/>
+      <c r="D48" s="57"/>
+      <c r="E48" s="78"/>
+      <c r="F48" s="78"/>
+      <c r="G48" s="78"/>
+      <c r="H48" s="78"/>
+      <c r="I48" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="J48" s="147">
+      <c r="J48" s="136">
         <f>K48/8</f>
         <v>0</v>
       </c>
-      <c r="K48" s="154">
+      <c r="K48" s="143">
         <f>K42</f>
         <v>0</v>
       </c>
-      <c r="L48" s="71"/>
-      <c r="M48" s="72" t="s">
+      <c r="L48" s="60"/>
+      <c r="M48" s="61" t="s">
         <v>45</v>
       </c>
       <c r="N48" s="2"/>
@@ -4659,29 +4722,29 @@
       <c r="P48" s="2"/>
     </row>
     <row r="49" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="73" t="s">
+      <c r="A49" s="62" t="s">
         <v>46</v>
       </c>
-      <c r="B49" s="74"/>
-      <c r="C49" s="74"/>
-      <c r="D49" s="74"/>
-      <c r="E49" s="92"/>
-      <c r="F49" s="92"/>
-      <c r="G49" s="92"/>
-      <c r="H49" s="92"/>
-      <c r="I49" s="93" t="s">
+      <c r="B49" s="63"/>
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="81"/>
+      <c r="F49" s="81"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="81"/>
+      <c r="I49" s="82" t="s">
         <v>29</v>
       </c>
-      <c r="J49" s="148">
+      <c r="J49" s="137">
         <f>K49/8</f>
         <v>0</v>
       </c>
-      <c r="K49" s="155">
+      <c r="K49" s="144">
         <f>I39</f>
         <v>0</v>
       </c>
-      <c r="L49" s="71"/>
-      <c r="M49" s="72" t="s">
+      <c r="L49" s="60"/>
+      <c r="M49" s="61" t="s">
         <v>47</v>
       </c>
       <c r="N49" s="2"/>
@@ -4689,28 +4752,28 @@
       <c r="P49" s="2"/>
     </row>
     <row r="50" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="77" t="s">
+      <c r="A50" s="66" t="s">
         <v>48</v>
       </c>
-      <c r="B50" s="78"/>
-      <c r="C50" s="78"/>
-      <c r="D50" s="78"/>
-      <c r="E50" s="94"/>
-      <c r="F50" s="94"/>
-      <c r="G50" s="94"/>
-      <c r="H50" s="94"/>
-      <c r="I50" s="95" t="s">
+      <c r="B50" s="67"/>
+      <c r="C50" s="67"/>
+      <c r="D50" s="67"/>
+      <c r="E50" s="83"/>
+      <c r="F50" s="83"/>
+      <c r="G50" s="83"/>
+      <c r="H50" s="83"/>
+      <c r="I50" s="84" t="s">
         <v>29</v>
       </c>
-      <c r="J50" s="149" t="s">
+      <c r="J50" s="138" t="s">
         <v>29</v>
       </c>
-      <c r="K50" s="156">
+      <c r="K50" s="145">
         <f>K39</f>
         <v>0</v>
       </c>
-      <c r="L50" s="71"/>
-      <c r="M50" s="72" t="s">
+      <c r="L50" s="60"/>
+      <c r="M50" s="61" t="s">
         <v>49</v>
       </c>
       <c r="N50" s="2"/>
@@ -4718,29 +4781,29 @@
       <c r="P50" s="2"/>
     </row>
     <row r="51" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="96" t="s">
+      <c r="A51" s="85" t="s">
         <v>50</v>
       </c>
-      <c r="B51" s="82"/>
-      <c r="C51" s="82"/>
-      <c r="D51" s="82"/>
-      <c r="E51" s="97"/>
-      <c r="F51" s="97"/>
-      <c r="G51" s="97"/>
-      <c r="H51" s="97"/>
-      <c r="I51" s="98" t="s">
+      <c r="B51" s="71"/>
+      <c r="C51" s="71"/>
+      <c r="D51" s="71"/>
+      <c r="E51" s="86"/>
+      <c r="F51" s="86"/>
+      <c r="G51" s="86"/>
+      <c r="H51" s="86"/>
+      <c r="I51" s="87" t="s">
         <v>29</v>
       </c>
-      <c r="J51" s="150">
+      <c r="J51" s="139">
         <f>SUM(J48:J49)</f>
         <v>0</v>
       </c>
-      <c r="K51" s="157">
+      <c r="K51" s="146">
         <f>SUM(K48:K50)</f>
         <v>0</v>
       </c>
-      <c r="L51" s="71"/>
-      <c r="M51" s="72" t="s">
+      <c r="L51" s="60"/>
+      <c r="M51" s="61" t="s">
         <v>51</v>
       </c>
       <c r="N51" s="2"/>
@@ -4748,229 +4811,229 @@
       <c r="P51" s="2"/>
     </row>
     <row r="52" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="67" t="s">
+      <c r="A52" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="B52" s="68"/>
-      <c r="C52" s="68"/>
-      <c r="D52" s="68"/>
-      <c r="E52" s="89"/>
-      <c r="F52" s="89"/>
-      <c r="G52" s="89"/>
-      <c r="H52" s="89"/>
-      <c r="I52" s="90" t="s">
+      <c r="B52" s="57"/>
+      <c r="C52" s="57"/>
+      <c r="D52" s="57"/>
+      <c r="E52" s="78"/>
+      <c r="F52" s="78"/>
+      <c r="G52" s="78"/>
+      <c r="H52" s="78"/>
+      <c r="I52" s="79" t="s">
         <v>29</v>
       </c>
-      <c r="J52" s="147">
+      <c r="J52" s="136">
         <f>COUNTIF(L8:L38,"&gt;0")</f>
         <v>0</v>
       </c>
-      <c r="K52" s="158">
+      <c r="K52" s="147">
         <f>L39</f>
         <v>0</v>
       </c>
-      <c r="L52" s="71"/>
-      <c r="M52" s="137"/>
-      <c r="N52" s="137"/>
-      <c r="O52" s="137"/>
+      <c r="L52" s="60"/>
+      <c r="M52" s="126"/>
+      <c r="N52" s="126"/>
+      <c r="O52" s="126"/>
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="188" t="s">
+      <c r="A53" s="172" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="189"/>
-      <c r="C53" s="184"/>
-      <c r="D53" s="184"/>
-      <c r="E53" s="184"/>
-      <c r="F53" s="184"/>
-      <c r="G53" s="100"/>
-      <c r="H53" s="190"/>
-      <c r="I53" s="189"/>
-      <c r="J53" s="151">
+      <c r="B53" s="173"/>
+      <c r="C53" s="167"/>
+      <c r="D53" s="167"/>
+      <c r="E53" s="167"/>
+      <c r="F53" s="167"/>
+      <c r="G53" s="89"/>
+      <c r="H53" s="177"/>
+      <c r="I53" s="173"/>
+      <c r="J53" s="140">
         <f>COUNTIF(C8:C38,"=D")</f>
         <v>0</v>
       </c>
-      <c r="K53" s="155">
+      <c r="K53" s="144">
         <f>J53*8</f>
         <v>0</v>
       </c>
-      <c r="L53" s="138"/>
-      <c r="M53" s="139" t="s">
+      <c r="L53" s="127"/>
+      <c r="M53" s="128" t="s">
         <v>54</v>
       </c>
-      <c r="N53" s="140" t="s">
+      <c r="N53" s="129" t="s">
         <v>55</v>
       </c>
-      <c r="O53" s="141" t="s">
+      <c r="O53" s="130" t="s">
         <v>56</v>
       </c>
-      <c r="P53" s="66"/>
+      <c r="P53" s="55"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="188" t="s">
+      <c r="A54" s="172" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="189"/>
-      <c r="C54" s="184"/>
-      <c r="D54" s="184"/>
-      <c r="E54" s="184"/>
-      <c r="F54" s="184"/>
-      <c r="G54" s="100"/>
-      <c r="H54" s="101"/>
-      <c r="I54" s="102"/>
-      <c r="J54" s="152">
+      <c r="B54" s="173"/>
+      <c r="C54" s="167"/>
+      <c r="D54" s="167"/>
+      <c r="E54" s="167"/>
+      <c r="F54" s="167"/>
+      <c r="G54" s="89"/>
+      <c r="H54" s="90"/>
+      <c r="I54" s="91"/>
+      <c r="J54" s="141">
         <f>COUNTIF(C8:C38,"=Sv")</f>
         <v>0</v>
       </c>
-      <c r="K54" s="155">
+      <c r="K54" s="144">
         <f t="shared" ref="K54:K57" si="0">J54*8</f>
         <v>0</v>
       </c>
-      <c r="L54" s="138"/>
-      <c r="M54" s="142" t="s">
+      <c r="L54" s="127"/>
+      <c r="M54" s="131" t="s">
         <v>58</v>
       </c>
-      <c r="N54" s="161"/>
-      <c r="O54" s="166">
+      <c r="N54" s="150"/>
+      <c r="O54" s="155">
         <f>N54*8</f>
         <v>0</v>
       </c>
-      <c r="P54" s="66"/>
+      <c r="P54" s="55"/>
     </row>
     <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="188" t="s">
+      <c r="A55" s="172" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="189"/>
-      <c r="C55" s="184"/>
-      <c r="D55" s="184"/>
-      <c r="E55" s="184"/>
-      <c r="F55" s="184"/>
-      <c r="G55" s="100"/>
-      <c r="H55" s="101"/>
-      <c r="I55" s="102"/>
-      <c r="J55" s="148">
+      <c r="B55" s="173"/>
+      <c r="C55" s="167"/>
+      <c r="D55" s="167"/>
+      <c r="E55" s="167"/>
+      <c r="F55" s="167"/>
+      <c r="G55" s="89"/>
+      <c r="H55" s="90"/>
+      <c r="I55" s="91"/>
+      <c r="J55" s="137">
         <f>COUNTIF(C8:C38,"=N")</f>
         <v>0</v>
       </c>
-      <c r="K55" s="155">
+      <c r="K55" s="144">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L55" s="138"/>
-      <c r="M55" s="142" t="s">
+      <c r="L55" s="127"/>
+      <c r="M55" s="131" t="s">
         <v>60</v>
       </c>
-      <c r="N55" s="162">
+      <c r="N55" s="151">
         <f>J54</f>
         <v>0</v>
       </c>
-      <c r="O55" s="166">
+      <c r="O55" s="155">
         <f>N55*8</f>
         <v>0</v>
       </c>
-      <c r="P55" s="66"/>
+      <c r="P55" s="55"/>
     </row>
     <row r="56" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="188" t="s">
+      <c r="A56" s="172" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="189"/>
-      <c r="C56" s="184"/>
-      <c r="D56" s="184"/>
-      <c r="E56" s="184"/>
-      <c r="F56" s="184"/>
-      <c r="G56" s="100"/>
-      <c r="H56" s="101"/>
-      <c r="I56" s="102"/>
-      <c r="J56" s="148">
+      <c r="B56" s="173"/>
+      <c r="C56" s="167"/>
+      <c r="D56" s="167"/>
+      <c r="E56" s="167"/>
+      <c r="F56" s="167"/>
+      <c r="G56" s="89"/>
+      <c r="H56" s="90"/>
+      <c r="I56" s="91"/>
+      <c r="J56" s="137">
         <f>COUNTIF(C8:C38,"=Oš")</f>
         <v>0</v>
       </c>
-      <c r="K56" s="155">
+      <c r="K56" s="144">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L56" s="138"/>
-      <c r="M56" s="143" t="s">
+      <c r="L56" s="127"/>
+      <c r="M56" s="132" t="s">
         <v>8</v>
       </c>
-      <c r="N56" s="160">
+      <c r="N56" s="149">
         <f>SUM(N54:N55)</f>
         <v>0</v>
       </c>
-      <c r="O56" s="167">
+      <c r="O56" s="156">
         <f>SUM(O54:O55)</f>
         <v>0</v>
       </c>
-      <c r="P56" s="66"/>
+      <c r="P56" s="55"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="188" t="s">
+      <c r="A57" s="172" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="189"/>
-      <c r="C57" s="184"/>
-      <c r="D57" s="184"/>
-      <c r="E57" s="184"/>
-      <c r="F57" s="184"/>
-      <c r="G57" s="100"/>
-      <c r="H57" s="101"/>
-      <c r="I57" s="102"/>
-      <c r="J57" s="148">
+      <c r="B57" s="173"/>
+      <c r="C57" s="167"/>
+      <c r="D57" s="167"/>
+      <c r="E57" s="167"/>
+      <c r="F57" s="167"/>
+      <c r="G57" s="89"/>
+      <c r="H57" s="90"/>
+      <c r="I57" s="91"/>
+      <c r="J57" s="137">
         <f>COUNTIF(C8:C38,"=NP")</f>
         <v>0</v>
       </c>
-      <c r="K57" s="155">
+      <c r="K57" s="144">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L57" s="71"/>
-      <c r="M57" s="136"/>
-      <c r="O57" s="136"/>
+      <c r="L57" s="60"/>
+      <c r="M57" s="125"/>
+      <c r="O57" s="125"/>
       <c r="P57" s="2"/>
     </row>
     <row r="58" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="191" t="s">
+      <c r="A58" s="174" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="192"/>
-      <c r="C58" s="192"/>
-      <c r="D58" s="192"/>
-      <c r="E58" s="192"/>
-      <c r="F58" s="192"/>
-      <c r="G58" s="104"/>
-      <c r="H58" s="104"/>
-      <c r="I58" s="105" t="s">
+      <c r="B58" s="175"/>
+      <c r="C58" s="175"/>
+      <c r="D58" s="175"/>
+      <c r="E58" s="175"/>
+      <c r="F58" s="175"/>
+      <c r="G58" s="93"/>
+      <c r="H58" s="93"/>
+      <c r="I58" s="94" t="s">
         <v>29</v>
       </c>
-      <c r="J58" s="153">
+      <c r="J58" s="142">
         <f>SUM(J51:J57)</f>
         <v>0</v>
       </c>
-      <c r="K58" s="156">
+      <c r="K58" s="145">
         <f>SUM(K51:K57)</f>
         <v>0</v>
       </c>
-      <c r="L58" s="71"/>
+      <c r="L58" s="60"/>
       <c r="M58" s="2"/>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
       <c r="P58" s="2"/>
     </row>
     <row r="59" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="106"/>
-      <c r="B59" s="106"/>
-      <c r="C59" s="106"/>
-      <c r="D59" s="106"/>
-      <c r="E59" s="106"/>
-      <c r="F59" s="106"/>
-      <c r="G59" s="106"/>
-      <c r="H59" s="106"/>
-      <c r="I59" s="106"/>
-      <c r="J59" s="107"/>
-      <c r="K59" s="107"/>
+      <c r="A59" s="95"/>
+      <c r="B59" s="95"/>
+      <c r="C59" s="95"/>
+      <c r="D59" s="95"/>
+      <c r="E59" s="95"/>
+      <c r="F59" s="95"/>
+      <c r="G59" s="95"/>
+      <c r="H59" s="95"/>
+      <c r="I59" s="95"/>
+      <c r="J59" s="96"/>
+      <c r="K59" s="96"/>
       <c r="L59" s="2"/>
       <c r="M59" s="2"/>
       <c r="N59" s="2"/>
@@ -4978,19 +5041,19 @@
       <c r="P59" s="2"/>
     </row>
     <row r="60" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="108" t="s">
+      <c r="A60" s="97" t="s">
         <v>63</v>
       </c>
-      <c r="B60" s="109"/>
-      <c r="C60" s="109"/>
-      <c r="D60" s="109"/>
-      <c r="E60" s="109"/>
-      <c r="F60" s="109"/>
-      <c r="G60" s="109"/>
-      <c r="H60" s="109"/>
-      <c r="I60" s="109"/>
-      <c r="J60" s="110"/>
-      <c r="K60" s="111" t="s">
+      <c r="B60" s="98"/>
+      <c r="C60" s="98"/>
+      <c r="D60" s="98"/>
+      <c r="E60" s="98"/>
+      <c r="F60" s="98"/>
+      <c r="G60" s="98"/>
+      <c r="H60" s="98"/>
+      <c r="I60" s="98"/>
+      <c r="J60" s="99"/>
+      <c r="K60" s="100" t="s">
         <v>17</v>
       </c>
       <c r="L60" s="2"/>
@@ -5000,118 +5063,151 @@
       <c r="P60" s="2"/>
     </row>
     <row r="61" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="112" t="s">
+      <c r="A61" s="101" t="s">
         <v>64</v>
       </c>
-      <c r="B61" s="113"/>
-      <c r="C61" s="113"/>
-      <c r="D61" s="113"/>
-      <c r="E61" s="114"/>
-      <c r="F61" s="114"/>
-      <c r="G61" s="114"/>
-      <c r="H61" s="114"/>
-      <c r="I61" s="114"/>
-      <c r="J61" s="115"/>
-      <c r="K61" s="91"/>
-      <c r="L61" s="71"/>
+      <c r="B61" s="102"/>
+      <c r="C61" s="102"/>
+      <c r="D61" s="102"/>
+      <c r="E61" s="103"/>
+      <c r="F61" s="103"/>
+      <c r="G61" s="103"/>
+      <c r="H61" s="103"/>
+      <c r="I61" s="103"/>
+      <c r="J61" s="104"/>
+      <c r="K61" s="80"/>
+      <c r="L61" s="60"/>
       <c r="M61" s="2"/>
       <c r="N61" s="2"/>
       <c r="O61" s="2"/>
       <c r="P61" s="2"/>
     </row>
     <row r="62" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="99" t="s">
+      <c r="A62" s="88" t="s">
         <v>65</v>
       </c>
-      <c r="B62" s="116"/>
-      <c r="C62" s="116"/>
-      <c r="D62" s="116"/>
-      <c r="E62" s="101"/>
-      <c r="F62" s="101"/>
-      <c r="G62" s="101"/>
-      <c r="H62" s="101"/>
-      <c r="I62" s="101"/>
-      <c r="J62" s="102"/>
-      <c r="K62" s="164">
+      <c r="B62" s="105"/>
+      <c r="C62" s="105"/>
+      <c r="D62" s="105"/>
+      <c r="E62" s="90"/>
+      <c r="F62" s="90"/>
+      <c r="G62" s="90"/>
+      <c r="H62" s="90"/>
+      <c r="I62" s="90"/>
+      <c r="J62" s="91"/>
+      <c r="K62" s="153">
         <f>I39</f>
         <v>0</v>
       </c>
-      <c r="L62" s="71"/>
+      <c r="L62" s="60"/>
       <c r="M62" s="2"/>
       <c r="N62" s="2"/>
       <c r="O62" s="2"/>
       <c r="P62" s="2"/>
     </row>
     <row r="63" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="99" t="s">
+      <c r="A63" s="88" t="s">
         <v>66</v>
       </c>
-      <c r="B63" s="116"/>
-      <c r="C63" s="116"/>
-      <c r="D63" s="116"/>
-      <c r="E63" s="101"/>
-      <c r="F63" s="101"/>
-      <c r="G63" s="101"/>
-      <c r="H63" s="101"/>
-      <c r="I63" s="101"/>
-      <c r="J63" s="102"/>
-      <c r="K63" s="164">
+      <c r="B63" s="105"/>
+      <c r="C63" s="105"/>
+      <c r="D63" s="105"/>
+      <c r="E63" s="90"/>
+      <c r="F63" s="90"/>
+      <c r="G63" s="90"/>
+      <c r="H63" s="90"/>
+      <c r="I63" s="90"/>
+      <c r="J63" s="91"/>
+      <c r="K63" s="153">
         <f>J39</f>
         <v>0</v>
       </c>
-      <c r="L63" s="71"/>
-      <c r="M63" s="72" t="s">
+      <c r="L63" s="60"/>
+      <c r="M63" s="61" t="s">
         <v>67</v>
       </c>
-      <c r="N63" s="117"/>
-      <c r="O63" s="117"/>
+      <c r="N63" s="106"/>
+      <c r="O63" s="106"/>
       <c r="P63" s="2"/>
     </row>
     <row r="64" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="103" t="s">
+      <c r="A64" s="92" t="s">
         <v>68</v>
       </c>
-      <c r="B64" s="118"/>
-      <c r="C64" s="118"/>
-      <c r="D64" s="118"/>
-      <c r="E64" s="104"/>
-      <c r="F64" s="104"/>
-      <c r="G64" s="104"/>
-      <c r="H64" s="104"/>
-      <c r="I64" s="104"/>
-      <c r="J64" s="119"/>
-      <c r="K64" s="165">
+      <c r="B64" s="107"/>
+      <c r="C64" s="107"/>
+      <c r="D64" s="107"/>
+      <c r="E64" s="93"/>
+      <c r="F64" s="93"/>
+      <c r="G64" s="93"/>
+      <c r="H64" s="93"/>
+      <c r="I64" s="93"/>
+      <c r="J64" s="108"/>
+      <c r="K64" s="154">
         <f>K61+K63-K62</f>
         <v>0</v>
       </c>
-      <c r="L64" s="71"/>
-      <c r="M64" s="72" t="s">
+      <c r="L64" s="60"/>
+      <c r="M64" s="61" t="s">
         <v>69</v>
       </c>
-      <c r="N64" s="117"/>
-      <c r="O64" s="117"/>
+      <c r="N64" s="106"/>
+      <c r="O64" s="106"/>
       <c r="P64" s="2"/>
     </row>
     <row r="65" spans="1:16" ht="12" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="106"/>
-      <c r="B65" s="106"/>
-      <c r="C65" s="106"/>
-      <c r="D65" s="106"/>
-      <c r="E65" s="106"/>
-      <c r="F65" s="106"/>
-      <c r="G65" s="106"/>
-      <c r="H65" s="106"/>
-      <c r="I65" s="120"/>
-      <c r="J65" s="120"/>
-      <c r="K65" s="120"/>
-      <c r="L65" s="117"/>
+      <c r="A65" s="95"/>
+      <c r="B65" s="95"/>
+      <c r="C65" s="95"/>
+      <c r="D65" s="95"/>
+      <c r="E65" s="95"/>
+      <c r="F65" s="95"/>
+      <c r="G65" s="95"/>
+      <c r="H65" s="95"/>
+      <c r="I65" s="109"/>
+      <c r="J65" s="109"/>
+      <c r="K65" s="109"/>
+      <c r="L65" s="106"/>
       <c r="M65" s="2"/>
       <c r="N65" s="2"/>
       <c r="O65" s="2"/>
-      <c r="P65" s="117"/>
+      <c r="P65" s="106"/>
     </row>
   </sheetData>
   <mergeCells count="49">
+    <mergeCell ref="B5:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="L3:N3"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="A2:G2"/>
@@ -5128,39 +5224,6 @@
     <mergeCell ref="N35:O35"/>
     <mergeCell ref="N30:O30"/>
     <mergeCell ref="N31:O31"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A58:F58"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="E5:G6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="B5:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.59055100000000005" right="0.19685" top="0.59055100000000005" bottom="0" header="0.11811000000000001" footer="0.11811000000000001"/>
   <pageSetup scale="85" orientation="portrait"/>

</xml_diff>

<commit_message>
Updated XLSX template to not include lunch break when work time is less than 6 hours
</commit_message>
<xml_diff>
--- a/public/template.xlsx
+++ b/public/template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/david/Git/work/vykaz-util/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C0C7D16-FC37-4948-ADC5-B8EA08727873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{649D121F-DDFE-3349-AE32-8C88B030F964}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="17280" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1705,7 +1705,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="201">
+  <cellXfs count="203">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -2009,85 +2009,91 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="87" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="68" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="69" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="67" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="54" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="66" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="88" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="89" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="90" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="93" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="91" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="92" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="91" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="94" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="95" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="96" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3244,9 +3250,9 @@
   <sheetData>
     <row r="1" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="2"/>
-      <c r="B1" s="187"/>
-      <c r="C1" s="163"/>
-      <c r="D1" s="163"/>
+      <c r="B1" s="179"/>
+      <c r="C1" s="180"/>
+      <c r="D1" s="180"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
@@ -3263,49 +3269,49 @@
       <c r="P1" s="4"/>
     </row>
     <row r="2" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="164" t="s">
+      <c r="A2" s="195" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="163"/>
-      <c r="C2" s="163"/>
-      <c r="D2" s="163"/>
-      <c r="E2" s="163"/>
-      <c r="F2" s="163"/>
-      <c r="G2" s="163"/>
+      <c r="B2" s="180"/>
+      <c r="C2" s="180"/>
+      <c r="D2" s="180"/>
+      <c r="E2" s="180"/>
+      <c r="F2" s="180"/>
+      <c r="G2" s="180"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="162" t="s">
+      <c r="L2" s="194" t="s">
         <v>2</v>
       </c>
-      <c r="M2" s="163"/>
+      <c r="M2" s="180"/>
       <c r="N2" s="5"/>
       <c r="O2" s="5"/>
       <c r="P2" s="6"/>
     </row>
     <row r="3" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="188" t="s">
+      <c r="A3" s="181" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="161"/>
-      <c r="C3" s="161"/>
-      <c r="D3" s="161"/>
+      <c r="B3" s="182"/>
+      <c r="C3" s="182"/>
+      <c r="D3" s="182"/>
       <c r="E3" s="8"/>
-      <c r="F3" s="165" t="s">
+      <c r="F3" s="196" t="s">
         <v>4</v>
       </c>
-      <c r="G3" s="161"/>
-      <c r="H3" s="161"/>
-      <c r="I3" s="161"/>
+      <c r="G3" s="182"/>
+      <c r="H3" s="182"/>
+      <c r="I3" s="182"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="161" t="str" cm="1">
+      <c r="L3" s="182" t="str" cm="1">
         <f t="array" ref="L3">_xlfn.CONCAT("Období(měsíc/rok) ",12,"/",2025)</f>
         <v>Období(měsíc/rok) 12/2025</v>
       </c>
-      <c r="M3" s="161"/>
-      <c r="N3" s="161"/>
+      <c r="M3" s="182"/>
+      <c r="N3" s="182"/>
       <c r="O3" s="7"/>
       <c r="P3" s="6"/>
     </row>
@@ -3313,11 +3319,11 @@
       <c r="A4" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="185" t="s">
+      <c r="B4" s="177" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="186"/>
-      <c r="D4" s="186"/>
+      <c r="C4" s="178"/>
+      <c r="D4" s="178"/>
       <c r="E4" s="11"/>
       <c r="F4" s="10" t="s">
         <v>7</v>
@@ -3349,12 +3355,12 @@
     </row>
     <row r="5" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="18"/>
-      <c r="B5" s="182"/>
-      <c r="C5" s="179"/>
-      <c r="D5" s="179"/>
-      <c r="E5" s="178"/>
-      <c r="F5" s="179"/>
-      <c r="G5" s="179"/>
+      <c r="B5" s="173"/>
+      <c r="C5" s="174"/>
+      <c r="D5" s="174"/>
+      <c r="E5" s="183"/>
+      <c r="F5" s="174"/>
+      <c r="G5" s="174"/>
       <c r="H5" s="19" t="s">
         <v>14</v>
       </c>
@@ -3381,12 +3387,12 @@
     </row>
     <row r="6" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="18"/>
-      <c r="B6" s="179"/>
-      <c r="C6" s="179"/>
-      <c r="D6" s="179"/>
-      <c r="E6" s="179"/>
-      <c r="F6" s="179"/>
-      <c r="G6" s="179"/>
+      <c r="B6" s="174"/>
+      <c r="C6" s="174"/>
+      <c r="D6" s="174"/>
+      <c r="E6" s="174"/>
+      <c r="F6" s="174"/>
+      <c r="G6" s="174"/>
       <c r="H6" s="19" t="s">
         <v>19</v>
       </c>
@@ -3405,11 +3411,11 @@
     </row>
     <row r="7" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="28"/>
-      <c r="B7" s="183" t="s">
+      <c r="B7" s="175" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="184"/>
-      <c r="D7" s="184"/>
+      <c r="C7" s="176"/>
+      <c r="D7" s="176"/>
       <c r="E7" s="30"/>
       <c r="F7" s="29" t="s">
         <v>22</v>
@@ -3443,33 +3449,33 @@
       <c r="A8" s="36">
         <v>1</v>
       </c>
-      <c r="B8" s="37"/>
+      <c r="B8" s="201"/>
       <c r="C8" s="110" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="38"/>
-      <c r="E8" s="39" t="str" cm="1">
-        <f t="array" ref="E8">IF(ISBLANK(D8),"","12.00")</f>
+      <c r="D8" s="202"/>
+      <c r="E8" s="39" t="str">
+        <f>IF(ISBLANK(D8),"",IF(H8&gt;6,"12.00",""))</f>
         <v/>
       </c>
       <c r="F8" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="41" t="str" cm="1">
-        <f t="array" ref="G8">IF(ISBLANK(D8),"","12.30")</f>
+      <c r="G8" s="41" t="str">
+        <f>IF(ISBLANK(D8),"",IF(H8&gt;6,"12.30",""))</f>
         <v/>
       </c>
       <c r="H8" s="42"/>
-      <c r="I8" s="189"/>
-      <c r="J8" s="190" t="str">
+      <c r="I8" s="161"/>
+      <c r="J8" s="162" t="str">
         <f>IF(AND(ISNUMBER(H8),NOT(ISERROR(H8&gt;8)),H8&gt;8),H8-8,"")</f>
         <v/>
       </c>
-      <c r="K8" s="191"/>
+      <c r="K8" s="163"/>
       <c r="L8" s="43"/>
       <c r="M8" s="44"/>
-      <c r="N8" s="166"/>
-      <c r="O8" s="167"/>
+      <c r="N8" s="184"/>
+      <c r="O8" s="185"/>
       <c r="P8" s="17"/>
     </row>
     <row r="9" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3481,28 +3487,28 @@
         <v>27</v>
       </c>
       <c r="D9" s="38"/>
-      <c r="E9" s="39" t="str" cm="1">
-        <f t="array" ref="E9">IF(ISBLANK(D9),"","12.00")</f>
+      <c r="E9" s="39" t="str">
+        <f t="shared" ref="E9:E38" si="0">IF(ISBLANK(D9),"",IF(H9&gt;6,"12.00",""))</f>
         <v/>
       </c>
       <c r="F9" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="41" t="str" cm="1">
-        <f t="array" ref="G9">IF(ISBLANK(D9),"","12.30")</f>
+      <c r="G9" s="41" t="str">
+        <f t="shared" ref="G9:G38" si="1">IF(ISBLANK(D9),"",IF(H9&gt;6,"12.30",""))</f>
         <v/>
       </c>
       <c r="H9" s="44"/>
-      <c r="I9" s="192"/>
-      <c r="J9" s="193" t="str" cm="1">
+      <c r="I9" s="164"/>
+      <c r="J9" s="165" t="str" cm="1">
         <f t="array" ref="J9">IF(AND(ISNUMBER(H9),NOT(ISERROR(H9&gt;8)),H9&gt;8),H9-8,"")</f>
         <v/>
       </c>
-      <c r="K9" s="194"/>
+      <c r="K9" s="166"/>
       <c r="L9" s="43"/>
       <c r="M9" s="44"/>
-      <c r="N9" s="166"/>
-      <c r="O9" s="167"/>
+      <c r="N9" s="184"/>
+      <c r="O9" s="185"/>
       <c r="P9" s="17"/>
     </row>
     <row r="10" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3514,28 +3520,28 @@
         <v>27</v>
       </c>
       <c r="D10" s="38"/>
-      <c r="E10" s="39" t="str" cm="1">
-        <f t="array" ref="E10">IF(ISBLANK(D10),"","12.00")</f>
+      <c r="E10" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F10" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="41" t="str" cm="1">
-        <f t="array" ref="G10">IF(ISBLANK(D10),"","12.30")</f>
+      <c r="G10" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H10" s="42"/>
-      <c r="I10" s="195"/>
-      <c r="J10" s="196" t="str" cm="1">
+      <c r="I10" s="167"/>
+      <c r="J10" s="168" t="str" cm="1">
         <f t="array" ref="J10">IF(AND(ISNUMBER(H10),NOT(ISERROR(H10&gt;8)),H10&gt;8),H10-8,"")</f>
         <v/>
       </c>
-      <c r="K10" s="194"/>
+      <c r="K10" s="166"/>
       <c r="L10" s="43"/>
       <c r="M10" s="44"/>
-      <c r="N10" s="166"/>
-      <c r="O10" s="167"/>
+      <c r="N10" s="184"/>
+      <c r="O10" s="185"/>
       <c r="P10" s="17"/>
     </row>
     <row r="11" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3547,28 +3553,28 @@
         <v>27</v>
       </c>
       <c r="D11" s="38"/>
-      <c r="E11" s="39" t="str" cm="1">
-        <f t="array" ref="E11">IF(ISBLANK(D11),"","12.00")</f>
+      <c r="E11" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F11" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="41" t="str" cm="1">
-        <f t="array" ref="G11">IF(ISBLANK(D11),"","12.30")</f>
+      <c r="G11" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H11" s="42"/>
-      <c r="I11" s="195"/>
-      <c r="J11" s="193" t="str" cm="1">
+      <c r="I11" s="167"/>
+      <c r="J11" s="165" t="str" cm="1">
         <f t="array" ref="J11">IF(AND(ISNUMBER(H11),NOT(ISERROR(H11&gt;8)),H11&gt;8),H11-8,"")</f>
         <v/>
       </c>
-      <c r="K11" s="194"/>
+      <c r="K11" s="166"/>
       <c r="L11" s="43"/>
       <c r="M11" s="44"/>
-      <c r="N11" s="166"/>
-      <c r="O11" s="167"/>
+      <c r="N11" s="184"/>
+      <c r="O11" s="185"/>
       <c r="P11" s="17"/>
     </row>
     <row r="12" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3580,28 +3586,28 @@
         <v>27</v>
       </c>
       <c r="D12" s="38"/>
-      <c r="E12" s="39" t="str" cm="1">
-        <f t="array" ref="E12">IF(ISBLANK(D12),"","12.00")</f>
+      <c r="E12" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F12" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="41" t="str" cm="1">
-        <f t="array" ref="G12">IF(ISBLANK(D12),"","12.30")</f>
+      <c r="G12" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H12" s="42"/>
-      <c r="I12" s="195"/>
-      <c r="J12" s="196" t="str" cm="1">
+      <c r="I12" s="167"/>
+      <c r="J12" s="168" t="str" cm="1">
         <f t="array" ref="J12">IF(AND(ISNUMBER(H12),NOT(ISERROR(H12&gt;8)),H12&gt;8),H12-8,"")</f>
         <v/>
       </c>
-      <c r="K12" s="194"/>
+      <c r="K12" s="166"/>
       <c r="L12" s="43"/>
       <c r="M12" s="117"/>
-      <c r="N12" s="180"/>
-      <c r="O12" s="181"/>
+      <c r="N12" s="186"/>
+      <c r="O12" s="187"/>
       <c r="P12" s="17"/>
     </row>
     <row r="13" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3613,28 +3619,28 @@
         <v>27</v>
       </c>
       <c r="D13" s="38"/>
-      <c r="E13" s="39" t="str" cm="1">
-        <f t="array" ref="E13">IF(ISBLANK(D13),"","12.00")</f>
+      <c r="E13" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F13" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G13" s="41" t="str" cm="1">
-        <f t="array" ref="G13">IF(ISBLANK(D13),"","12.30")</f>
+      <c r="G13" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H13" s="44"/>
-      <c r="I13" s="195"/>
-      <c r="J13" s="193" t="str" cm="1">
+      <c r="I13" s="167"/>
+      <c r="J13" s="165" t="str" cm="1">
         <f t="array" ref="J13">IF(AND(ISNUMBER(H13),NOT(ISERROR(H13&gt;8)),H13&gt;8),H13-8,"")</f>
         <v/>
       </c>
-      <c r="K13" s="194"/>
+      <c r="K13" s="166"/>
       <c r="L13" s="119"/>
       <c r="M13" s="120"/>
-      <c r="N13" s="168"/>
-      <c r="O13" s="169"/>
+      <c r="N13" s="197"/>
+      <c r="O13" s="198"/>
       <c r="P13" s="55"/>
     </row>
     <row r="14" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3646,28 +3652,28 @@
         <v>27</v>
       </c>
       <c r="D14" s="38"/>
-      <c r="E14" s="39" t="str" cm="1">
-        <f t="array" ref="E14">IF(ISBLANK(D14),"","12.00")</f>
+      <c r="E14" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F14" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G14" s="41" t="str" cm="1">
-        <f t="array" ref="G14">IF(ISBLANK(D14),"","12.30")</f>
+      <c r="G14" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H14" s="44"/>
-      <c r="I14" s="195"/>
-      <c r="J14" s="193" t="str" cm="1">
+      <c r="I14" s="167"/>
+      <c r="J14" s="165" t="str" cm="1">
         <f t="array" ref="J14">IF(AND(ISNUMBER(H14),NOT(ISERROR(H14&gt;8)),H14&gt;8),H14-8,"")</f>
         <v/>
       </c>
-      <c r="K14" s="194"/>
+      <c r="K14" s="166"/>
       <c r="L14" s="43"/>
       <c r="M14" s="118"/>
-      <c r="N14" s="170"/>
-      <c r="O14" s="171"/>
+      <c r="N14" s="199"/>
+      <c r="O14" s="200"/>
       <c r="P14" s="17"/>
     </row>
     <row r="15" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3679,28 +3685,28 @@
         <v>27</v>
       </c>
       <c r="D15" s="38"/>
-      <c r="E15" s="39" t="str" cm="1">
-        <f t="array" ref="E15">IF(ISBLANK(D15),"","12.00")</f>
+      <c r="E15" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F15" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G15" s="41" t="str" cm="1">
-        <f t="array" ref="G15">IF(ISBLANK(D15),"","12.30")</f>
+      <c r="G15" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H15" s="42"/>
-      <c r="I15" s="195"/>
-      <c r="J15" s="196" t="str" cm="1">
+      <c r="I15" s="167"/>
+      <c r="J15" s="168" t="str" cm="1">
         <f t="array" ref="J15">IF(AND(ISNUMBER(H15),NOT(ISERROR(H15&gt;8)),H15&gt;8),H15-8,"")</f>
         <v/>
       </c>
-      <c r="K15" s="194"/>
+      <c r="K15" s="166"/>
       <c r="L15" s="43"/>
       <c r="M15" s="44"/>
-      <c r="N15" s="166"/>
-      <c r="O15" s="167"/>
+      <c r="N15" s="184"/>
+      <c r="O15" s="185"/>
       <c r="P15" s="17"/>
     </row>
     <row r="16" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3712,28 +3718,28 @@
         <v>27</v>
       </c>
       <c r="D16" s="38"/>
-      <c r="E16" s="39" t="str" cm="1">
-        <f t="array" ref="E16">IF(ISBLANK(D16),"","12.00")</f>
+      <c r="E16" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F16" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G16" s="41" t="str" cm="1">
-        <f t="array" ref="G16">IF(ISBLANK(D16),"","12.30")</f>
+      <c r="G16" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H16" s="42"/>
-      <c r="I16" s="195"/>
-      <c r="J16" s="196" t="str" cm="1">
+      <c r="I16" s="167"/>
+      <c r="J16" s="168" t="str" cm="1">
         <f t="array" ref="J16">IF(AND(ISNUMBER(H16),NOT(ISERROR(H16&gt;8)),H16&gt;8),H16-8,"")</f>
         <v/>
       </c>
-      <c r="K16" s="194"/>
+      <c r="K16" s="166"/>
       <c r="L16" s="43"/>
       <c r="M16" s="44"/>
-      <c r="N16" s="166"/>
-      <c r="O16" s="167"/>
+      <c r="N16" s="184"/>
+      <c r="O16" s="185"/>
       <c r="P16" s="17"/>
     </row>
     <row r="17" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3745,28 +3751,28 @@
         <v>27</v>
       </c>
       <c r="D17" s="38"/>
-      <c r="E17" s="39" t="str" cm="1">
-        <f t="array" ref="E17">IF(ISBLANK(D17),"","12.00")</f>
+      <c r="E17" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F17" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="41" t="str" cm="1">
-        <f t="array" ref="G17">IF(ISBLANK(D17),"","12.30")</f>
+      <c r="G17" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H17" s="42"/>
-      <c r="I17" s="195"/>
-      <c r="J17" s="196" t="str" cm="1">
+      <c r="I17" s="167"/>
+      <c r="J17" s="168" t="str" cm="1">
         <f t="array" ref="J17">IF(AND(ISNUMBER(H17),NOT(ISERROR(H17&gt;8)),H17&gt;8),H17-8,"")</f>
         <v/>
       </c>
-      <c r="K17" s="194"/>
+      <c r="K17" s="166"/>
       <c r="L17" s="43"/>
       <c r="M17" s="44"/>
-      <c r="N17" s="166"/>
-      <c r="O17" s="167"/>
+      <c r="N17" s="184"/>
+      <c r="O17" s="185"/>
       <c r="P17" s="17"/>
     </row>
     <row r="18" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3778,28 +3784,28 @@
         <v>27</v>
       </c>
       <c r="D18" s="38"/>
-      <c r="E18" s="39" t="str" cm="1">
-        <f t="array" ref="E18">IF(ISBLANK(D18),"","12.00")</f>
+      <c r="E18" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F18" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G18" s="41" t="str" cm="1">
-        <f t="array" ref="G18">IF(ISBLANK(D18),"","12.30")</f>
+      <c r="G18" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H18" s="42"/>
-      <c r="I18" s="195"/>
-      <c r="J18" s="193" t="str" cm="1">
+      <c r="I18" s="167"/>
+      <c r="J18" s="165" t="str" cm="1">
         <f t="array" ref="J18">IF(AND(ISNUMBER(H18),NOT(ISERROR(H18&gt;8)),H18&gt;8),H18-8,"")</f>
         <v/>
       </c>
-      <c r="K18" s="194"/>
+      <c r="K18" s="166"/>
       <c r="L18" s="43"/>
       <c r="M18" s="44"/>
-      <c r="N18" s="166"/>
-      <c r="O18" s="167"/>
+      <c r="N18" s="184"/>
+      <c r="O18" s="185"/>
       <c r="P18" s="17"/>
     </row>
     <row r="19" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3811,28 +3817,28 @@
         <v>27</v>
       </c>
       <c r="D19" s="38"/>
-      <c r="E19" s="39" t="str" cm="1">
-        <f t="array" ref="E19">IF(ISBLANK(D19),"","12.00")</f>
+      <c r="E19" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F19" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G19" s="41" t="str" cm="1">
-        <f t="array" ref="G19">IF(ISBLANK(D19),"","12.30")</f>
+      <c r="G19" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H19" s="42"/>
-      <c r="I19" s="195"/>
-      <c r="J19" s="196" t="str" cm="1">
+      <c r="I19" s="167"/>
+      <c r="J19" s="168" t="str" cm="1">
         <f t="array" ref="J19">IF(AND(ISNUMBER(H19),NOT(ISERROR(H19&gt;8)),H19&gt;8),H19-8,"")</f>
         <v/>
       </c>
-      <c r="K19" s="194"/>
+      <c r="K19" s="166"/>
       <c r="L19" s="43"/>
       <c r="M19" s="44"/>
-      <c r="N19" s="166"/>
-      <c r="O19" s="167"/>
+      <c r="N19" s="184"/>
+      <c r="O19" s="185"/>
       <c r="P19" s="17"/>
     </row>
     <row r="20" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3844,28 +3850,28 @@
         <v>27</v>
       </c>
       <c r="D20" s="38"/>
-      <c r="E20" s="39" t="str" cm="1">
-        <f t="array" ref="E20">IF(ISBLANK(D20),"","12.00")</f>
+      <c r="E20" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F20" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G20" s="41" t="str" cm="1">
-        <f t="array" ref="G20">IF(ISBLANK(D20),"","12.30")</f>
+      <c r="G20" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H20" s="44"/>
-      <c r="I20" s="197"/>
-      <c r="J20" s="193" t="str" cm="1">
+      <c r="I20" s="169"/>
+      <c r="J20" s="165" t="str" cm="1">
         <f t="array" ref="J20">IF(AND(ISNUMBER(H20),NOT(ISERROR(H20&gt;8)),H20&gt;8),H20-8,"")</f>
         <v/>
       </c>
-      <c r="K20" s="194"/>
+      <c r="K20" s="166"/>
       <c r="L20" s="43"/>
       <c r="M20" s="44"/>
-      <c r="N20" s="166"/>
-      <c r="O20" s="167"/>
+      <c r="N20" s="184"/>
+      <c r="O20" s="185"/>
       <c r="P20" s="17"/>
     </row>
     <row r="21" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3877,28 +3883,28 @@
         <v>27</v>
       </c>
       <c r="D21" s="38"/>
-      <c r="E21" s="39" t="str" cm="1">
-        <f t="array" ref="E21">IF(ISBLANK(D21),"","12.00")</f>
+      <c r="E21" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F21" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G21" s="41" t="str" cm="1">
-        <f t="array" ref="G21">IF(ISBLANK(D21),"","12.30")</f>
+      <c r="G21" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H21" s="44"/>
-      <c r="I21" s="195"/>
-      <c r="J21" s="193" t="str" cm="1">
+      <c r="I21" s="167"/>
+      <c r="J21" s="165" t="str" cm="1">
         <f t="array" ref="J21">IF(AND(ISNUMBER(H21),NOT(ISERROR(H21&gt;8)),H21&gt;8),H21-8,"")</f>
         <v/>
       </c>
-      <c r="K21" s="194"/>
+      <c r="K21" s="166"/>
       <c r="L21" s="43"/>
       <c r="M21" s="44"/>
-      <c r="N21" s="166"/>
-      <c r="O21" s="167"/>
+      <c r="N21" s="184"/>
+      <c r="O21" s="185"/>
       <c r="P21" s="17"/>
     </row>
     <row r="22" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3910,28 +3916,28 @@
         <v>27</v>
       </c>
       <c r="D22" s="38"/>
-      <c r="E22" s="39" t="str" cm="1">
-        <f t="array" ref="E22">IF(ISBLANK(D22),"","12.00")</f>
+      <c r="E22" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F22" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="41" t="str" cm="1">
-        <f t="array" ref="G22">IF(ISBLANK(D22),"","12.30")</f>
+      <c r="G22" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H22" s="42"/>
-      <c r="I22" s="195"/>
-      <c r="J22" s="196" t="str" cm="1">
+      <c r="I22" s="167"/>
+      <c r="J22" s="168" t="str" cm="1">
         <f t="array" ref="J22">IF(AND(ISNUMBER(H22),NOT(ISERROR(H22&gt;8)),H22&gt;8),H22-8,"")</f>
         <v/>
       </c>
-      <c r="K22" s="194"/>
+      <c r="K22" s="166"/>
       <c r="L22" s="43"/>
       <c r="M22" s="44"/>
-      <c r="N22" s="166"/>
-      <c r="O22" s="167"/>
+      <c r="N22" s="184"/>
+      <c r="O22" s="185"/>
       <c r="P22" s="17"/>
     </row>
     <row r="23" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3943,28 +3949,28 @@
         <v>27</v>
       </c>
       <c r="D23" s="38"/>
-      <c r="E23" s="39" t="str" cm="1">
-        <f t="array" ref="E23">IF(ISBLANK(D23),"","12.00")</f>
+      <c r="E23" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F23" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G23" s="41" t="str" cm="1">
-        <f t="array" ref="G23">IF(ISBLANK(D23),"","12.30")</f>
+      <c r="G23" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H23" s="42"/>
-      <c r="I23" s="195"/>
-      <c r="J23" s="193" t="str" cm="1">
+      <c r="I23" s="167"/>
+      <c r="J23" s="165" t="str" cm="1">
         <f t="array" ref="J23">IF(AND(ISNUMBER(H23),NOT(ISERROR(H23&gt;8)),H23&gt;8),H23-8,"")</f>
         <v/>
       </c>
-      <c r="K23" s="194"/>
+      <c r="K23" s="166"/>
       <c r="L23" s="43"/>
       <c r="M23" s="44"/>
-      <c r="N23" s="166"/>
-      <c r="O23" s="167"/>
+      <c r="N23" s="184"/>
+      <c r="O23" s="185"/>
       <c r="P23" s="17"/>
     </row>
     <row r="24" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3976,28 +3982,28 @@
         <v>27</v>
       </c>
       <c r="D24" s="38"/>
-      <c r="E24" s="39" t="str" cm="1">
-        <f t="array" ref="E24">IF(ISBLANK(D24),"","12.00")</f>
+      <c r="E24" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F24" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G24" s="41" t="str" cm="1">
-        <f t="array" ref="G24">IF(ISBLANK(D24),"","12.30")</f>
+      <c r="G24" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H24" s="42"/>
-      <c r="I24" s="195"/>
-      <c r="J24" s="196" t="str" cm="1">
+      <c r="I24" s="167"/>
+      <c r="J24" s="168" t="str" cm="1">
         <f t="array" ref="J24">IF(AND(ISNUMBER(H24),NOT(ISERROR(H24&gt;8)),H24&gt;8),H24-8,"")</f>
         <v/>
       </c>
-      <c r="K24" s="194"/>
+      <c r="K24" s="166"/>
       <c r="L24" s="43"/>
       <c r="M24" s="44"/>
-      <c r="N24" s="166"/>
-      <c r="O24" s="167"/>
+      <c r="N24" s="184"/>
+      <c r="O24" s="185"/>
       <c r="P24" s="17"/>
     </row>
     <row r="25" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4009,28 +4015,28 @@
         <v>27</v>
       </c>
       <c r="D25" s="38"/>
-      <c r="E25" s="39" t="str" cm="1">
-        <f t="array" ref="E25">IF(ISBLANK(D25),"","12.00")</f>
+      <c r="E25" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F25" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G25" s="41" t="str" cm="1">
-        <f t="array" ref="G25">IF(ISBLANK(D25),"","12.30")</f>
+      <c r="G25" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H25" s="42"/>
-      <c r="I25" s="195"/>
-      <c r="J25" s="193" t="str" cm="1">
+      <c r="I25" s="167"/>
+      <c r="J25" s="165" t="str" cm="1">
         <f t="array" ref="J25">IF(AND(ISNUMBER(H25),NOT(ISERROR(H25&gt;8)),H25&gt;8),H25-8,"")</f>
         <v/>
       </c>
-      <c r="K25" s="194"/>
+      <c r="K25" s="166"/>
       <c r="L25" s="43"/>
       <c r="M25" s="44"/>
-      <c r="N25" s="166"/>
-      <c r="O25" s="167"/>
+      <c r="N25" s="184"/>
+      <c r="O25" s="185"/>
       <c r="P25" s="17"/>
     </row>
     <row r="26" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4042,28 +4048,28 @@
         <v>27</v>
       </c>
       <c r="D26" s="38"/>
-      <c r="E26" s="39" t="str" cm="1">
-        <f t="array" ref="E26">IF(ISBLANK(D26),"","12.00")</f>
+      <c r="E26" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F26" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G26" s="41" t="str" cm="1">
-        <f t="array" ref="G26">IF(ISBLANK(D26),"","12.30")</f>
+      <c r="G26" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H26" s="42"/>
-      <c r="I26" s="195"/>
-      <c r="J26" s="193" t="str" cm="1">
+      <c r="I26" s="167"/>
+      <c r="J26" s="165" t="str" cm="1">
         <f t="array" ref="J26">IF(AND(ISNUMBER(H26),NOT(ISERROR(H26&gt;8)),H26&gt;8),H26-8,"")</f>
         <v/>
       </c>
-      <c r="K26" s="194"/>
+      <c r="K26" s="166"/>
       <c r="L26" s="43"/>
       <c r="M26" s="44"/>
-      <c r="N26" s="166"/>
-      <c r="O26" s="167"/>
+      <c r="N26" s="184"/>
+      <c r="O26" s="185"/>
       <c r="P26" s="17"/>
     </row>
     <row r="27" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4075,28 +4081,28 @@
         <v>27</v>
       </c>
       <c r="D27" s="38"/>
-      <c r="E27" s="39" t="str" cm="1">
-        <f t="array" ref="E27">IF(ISBLANK(D27),"","12.00")</f>
+      <c r="E27" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F27" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G27" s="41" t="str" cm="1">
-        <f t="array" ref="G27">IF(ISBLANK(D27),"","12.30")</f>
+      <c r="G27" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H27" s="44"/>
-      <c r="I27" s="195"/>
-      <c r="J27" s="193" t="str" cm="1">
+      <c r="I27" s="167"/>
+      <c r="J27" s="165" t="str" cm="1">
         <f t="array" ref="J27">IF(AND(ISNUMBER(H27),NOT(ISERROR(H27&gt;8)),H27&gt;8),H27-8,"")</f>
         <v/>
       </c>
-      <c r="K27" s="194"/>
+      <c r="K27" s="166"/>
       <c r="L27" s="43"/>
       <c r="M27" s="44"/>
-      <c r="N27" s="166"/>
-      <c r="O27" s="167"/>
+      <c r="N27" s="184"/>
+      <c r="O27" s="185"/>
       <c r="P27" s="17"/>
     </row>
     <row r="28" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4108,28 +4114,28 @@
         <v>27</v>
       </c>
       <c r="D28" s="38"/>
-      <c r="E28" s="39" t="str" cm="1">
-        <f t="array" ref="E28">IF(ISBLANK(D28),"","12.00")</f>
+      <c r="E28" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F28" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="41" t="str" cm="1">
-        <f t="array" ref="G28">IF(ISBLANK(D28),"","12.30")</f>
+      <c r="G28" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H28" s="44"/>
-      <c r="I28" s="195"/>
-      <c r="J28" s="193" t="str" cm="1">
+      <c r="I28" s="167"/>
+      <c r="J28" s="165" t="str" cm="1">
         <f t="array" ref="J28">IF(AND(ISNUMBER(H28),NOT(ISERROR(H28&gt;8)),H28&gt;8),H28-8,"")</f>
         <v/>
       </c>
-      <c r="K28" s="194"/>
+      <c r="K28" s="166"/>
       <c r="L28" s="43"/>
       <c r="M28" s="44"/>
-      <c r="N28" s="166"/>
-      <c r="O28" s="167"/>
+      <c r="N28" s="184"/>
+      <c r="O28" s="185"/>
       <c r="P28" s="17"/>
     </row>
     <row r="29" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4141,28 +4147,28 @@
         <v>27</v>
       </c>
       <c r="D29" s="38"/>
-      <c r="E29" s="39" t="str" cm="1">
-        <f t="array" ref="E29">IF(ISBLANK(D29),"","12.00")</f>
+      <c r="E29" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F29" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G29" s="41" t="str" cm="1">
-        <f t="array" ref="G29">IF(ISBLANK(D29),"","12.30")</f>
+      <c r="G29" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H29" s="44"/>
-      <c r="I29" s="192"/>
-      <c r="J29" s="193" t="str" cm="1">
+      <c r="I29" s="164"/>
+      <c r="J29" s="165" t="str" cm="1">
         <f t="array" ref="J29">IF(AND(ISNUMBER(H29),NOT(ISERROR(H29&gt;8)),H29&gt;8),H29-8,"")</f>
         <v/>
       </c>
-      <c r="K29" s="194"/>
+      <c r="K29" s="166"/>
       <c r="L29" s="43"/>
       <c r="M29" s="44"/>
-      <c r="N29" s="166"/>
-      <c r="O29" s="167"/>
+      <c r="N29" s="184"/>
+      <c r="O29" s="185"/>
       <c r="P29" s="17"/>
     </row>
     <row r="30" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4174,28 +4180,28 @@
         <v>27</v>
       </c>
       <c r="D30" s="38"/>
-      <c r="E30" s="39" t="str" cm="1">
-        <f t="array" ref="E30">IF(ISBLANK(D30),"","12.00")</f>
+      <c r="E30" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F30" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G30" s="41" t="str" cm="1">
-        <f t="array" ref="G30">IF(ISBLANK(D30),"","12.30")</f>
+      <c r="G30" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H30" s="44"/>
-      <c r="I30" s="192"/>
-      <c r="J30" s="193" t="str" cm="1">
+      <c r="I30" s="164"/>
+      <c r="J30" s="165" t="str" cm="1">
         <f t="array" ref="J30">IF(AND(ISNUMBER(H30),NOT(ISERROR(H30&gt;8)),H30&gt;8),H30-8,"")</f>
         <v/>
       </c>
-      <c r="K30" s="194"/>
+      <c r="K30" s="166"/>
       <c r="L30" s="43"/>
       <c r="M30" s="44"/>
-      <c r="N30" s="166"/>
-      <c r="O30" s="167"/>
+      <c r="N30" s="184"/>
+      <c r="O30" s="185"/>
       <c r="P30" s="17"/>
     </row>
     <row r="31" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4207,28 +4213,28 @@
         <v>27</v>
       </c>
       <c r="D31" s="38"/>
-      <c r="E31" s="39" t="str" cm="1">
-        <f t="array" ref="E31">IF(ISBLANK(D31),"","12.00")</f>
+      <c r="E31" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F31" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G31" s="41" t="str" cm="1">
-        <f t="array" ref="G31">IF(ISBLANK(D31),"","12.30")</f>
+      <c r="G31" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H31" s="44"/>
-      <c r="I31" s="195"/>
-      <c r="J31" s="193" t="str" cm="1">
+      <c r="I31" s="167"/>
+      <c r="J31" s="165" t="str" cm="1">
         <f t="array" ref="J31">IF(AND(ISNUMBER(H31),NOT(ISERROR(H31&gt;8)),H31&gt;8),H31-8,"")</f>
         <v/>
       </c>
-      <c r="K31" s="194"/>
+      <c r="K31" s="166"/>
       <c r="L31" s="43"/>
       <c r="M31" s="44"/>
-      <c r="N31" s="166"/>
-      <c r="O31" s="167"/>
+      <c r="N31" s="184"/>
+      <c r="O31" s="185"/>
       <c r="P31" s="17"/>
     </row>
     <row r="32" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4240,28 +4246,28 @@
         <v>27</v>
       </c>
       <c r="D32" s="38"/>
-      <c r="E32" s="39" t="str" cm="1">
-        <f t="array" ref="E32">IF(ISBLANK(D32),"","12.00")</f>
+      <c r="E32" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F32" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G32" s="41" t="str" cm="1">
-        <f t="array" ref="G32">IF(ISBLANK(D32),"","12.30")</f>
+      <c r="G32" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H32" s="44"/>
-      <c r="I32" s="195"/>
-      <c r="J32" s="193" t="str" cm="1">
+      <c r="I32" s="167"/>
+      <c r="J32" s="165" t="str" cm="1">
         <f t="array" ref="J32">IF(AND(ISNUMBER(H32),NOT(ISERROR(H32&gt;8)),H32&gt;8),H32-8,"")</f>
         <v/>
       </c>
-      <c r="K32" s="194"/>
+      <c r="K32" s="166"/>
       <c r="L32" s="43"/>
       <c r="M32" s="44"/>
-      <c r="N32" s="166"/>
-      <c r="O32" s="167"/>
+      <c r="N32" s="184"/>
+      <c r="O32" s="185"/>
       <c r="P32" s="17"/>
     </row>
     <row r="33" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4273,28 +4279,28 @@
         <v>27</v>
       </c>
       <c r="D33" s="38"/>
-      <c r="E33" s="39" t="str" cm="1">
-        <f t="array" ref="E33">IF(ISBLANK(D33),"","12.00")</f>
+      <c r="E33" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F33" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G33" s="41" t="str" cm="1">
-        <f t="array" ref="G33">IF(ISBLANK(D33),"","12.30")</f>
+      <c r="G33" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H33" s="44"/>
-      <c r="I33" s="195"/>
-      <c r="J33" s="193" t="str" cm="1">
+      <c r="I33" s="167"/>
+      <c r="J33" s="165" t="str" cm="1">
         <f t="array" ref="J33">IF(AND(ISNUMBER(H33),NOT(ISERROR(H33&gt;8)),H33&gt;8),H33-8,"")</f>
         <v/>
       </c>
-      <c r="K33" s="194"/>
+      <c r="K33" s="166"/>
       <c r="L33" s="43"/>
       <c r="M33" s="44"/>
-      <c r="N33" s="166"/>
-      <c r="O33" s="167"/>
+      <c r="N33" s="184"/>
+      <c r="O33" s="185"/>
       <c r="P33" s="17"/>
     </row>
     <row r="34" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4306,28 +4312,28 @@
         <v>27</v>
       </c>
       <c r="D34" s="38"/>
-      <c r="E34" s="39" t="str" cm="1">
-        <f t="array" ref="E34">IF(ISBLANK(D34),"","12.00")</f>
+      <c r="E34" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F34" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G34" s="41" t="str" cm="1">
-        <f t="array" ref="G34">IF(ISBLANK(D34),"","12.30")</f>
+      <c r="G34" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H34" s="44"/>
-      <c r="I34" s="195"/>
-      <c r="J34" s="193" t="str" cm="1">
+      <c r="I34" s="167"/>
+      <c r="J34" s="165" t="str" cm="1">
         <f t="array" ref="J34">IF(AND(ISNUMBER(H34),NOT(ISERROR(H34&gt;8)),H34&gt;8),H34-8,"")</f>
         <v/>
       </c>
-      <c r="K34" s="194"/>
+      <c r="K34" s="166"/>
       <c r="L34" s="43"/>
       <c r="M34" s="44"/>
-      <c r="N34" s="166"/>
-      <c r="O34" s="167"/>
+      <c r="N34" s="184"/>
+      <c r="O34" s="185"/>
       <c r="P34" s="17"/>
     </row>
     <row r="35" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4339,28 +4345,28 @@
         <v>27</v>
       </c>
       <c r="D35" s="38"/>
-      <c r="E35" s="39" t="str" cm="1">
-        <f t="array" ref="E35">IF(ISBLANK(D35),"","12.00")</f>
+      <c r="E35" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F35" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="41" t="str" cm="1">
-        <f t="array" ref="G35">IF(ISBLANK(D35),"","12.30")</f>
+      <c r="G35" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H35" s="44"/>
-      <c r="I35" s="195"/>
-      <c r="J35" s="193" t="str" cm="1">
+      <c r="I35" s="167"/>
+      <c r="J35" s="165" t="str" cm="1">
         <f t="array" ref="J35">IF(AND(ISNUMBER(H35),NOT(ISERROR(H35&gt;8)),H35&gt;8),H35-8,"")</f>
         <v/>
       </c>
-      <c r="K35" s="194"/>
+      <c r="K35" s="166"/>
       <c r="L35" s="43"/>
       <c r="M35" s="44"/>
-      <c r="N35" s="166"/>
-      <c r="O35" s="167"/>
+      <c r="N35" s="184"/>
+      <c r="O35" s="185"/>
       <c r="P35" s="17"/>
     </row>
     <row r="36" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4372,28 +4378,28 @@
         <v>27</v>
       </c>
       <c r="D36" s="38"/>
-      <c r="E36" s="39" t="str" cm="1">
-        <f t="array" ref="E36">IF(ISBLANK(D36),"","12.00")</f>
+      <c r="E36" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F36" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G36" s="41" t="str" cm="1">
-        <f t="array" ref="G36">IF(ISBLANK(D36),"","12.30")</f>
+      <c r="G36" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H36" s="44"/>
-      <c r="I36" s="192"/>
-      <c r="J36" s="193" t="str" cm="1">
+      <c r="I36" s="164"/>
+      <c r="J36" s="165" t="str" cm="1">
         <f t="array" ref="J36">IF(AND(ISNUMBER(H36),NOT(ISERROR(H36&gt;8)),H36&gt;8),H36-8,"")</f>
         <v/>
       </c>
-      <c r="K36" s="194"/>
+      <c r="K36" s="166"/>
       <c r="L36" s="43"/>
       <c r="M36" s="44"/>
-      <c r="N36" s="166"/>
-      <c r="O36" s="167"/>
+      <c r="N36" s="184"/>
+      <c r="O36" s="185"/>
       <c r="P36" s="17"/>
     </row>
     <row r="37" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4405,28 +4411,28 @@
         <v>27</v>
       </c>
       <c r="D37" s="38"/>
-      <c r="E37" s="39" t="str" cm="1">
-        <f t="array" ref="E37">IF(ISBLANK(D37),"","12.00")</f>
+      <c r="E37" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F37" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="G37" s="41" t="str" cm="1">
-        <f t="array" ref="G37">IF(ISBLANK(D37),"","12.30")</f>
+      <c r="G37" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H37" s="44"/>
-      <c r="I37" s="192"/>
-      <c r="J37" s="193" t="str" cm="1">
+      <c r="I37" s="164"/>
+      <c r="J37" s="165" t="str" cm="1">
         <f t="array" ref="J37">IF(AND(ISNUMBER(H37),NOT(ISERROR(H37&gt;8)),H37&gt;8),H37-8,"")</f>
         <v/>
       </c>
-      <c r="K37" s="194"/>
+      <c r="K37" s="166"/>
       <c r="L37" s="43"/>
       <c r="M37" s="44"/>
-      <c r="N37" s="166"/>
-      <c r="O37" s="167"/>
+      <c r="N37" s="184"/>
+      <c r="O37" s="185"/>
       <c r="P37" s="17"/>
     </row>
     <row r="38" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4438,28 +4444,28 @@
         <v>27</v>
       </c>
       <c r="D38" s="41"/>
-      <c r="E38" s="39" t="str" cm="1">
-        <f t="array" ref="E38">IF(ISBLANK(D38),"","12.00")</f>
+      <c r="E38" s="39" t="str">
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="F38" s="112" t="s">
         <v>27</v>
       </c>
-      <c r="G38" s="41" t="str" cm="1">
-        <f t="array" ref="G38">IF(ISBLANK(D38),"","12.30")</f>
+      <c r="G38" s="41" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="H38" s="44"/>
-      <c r="I38" s="198"/>
-      <c r="J38" s="199" t="str" cm="1">
+      <c r="I38" s="170"/>
+      <c r="J38" s="171" t="str" cm="1">
         <f t="array" ref="J38">IF(AND(ISNUMBER(H38),NOT(ISERROR(H38&gt;8)),H38&gt;8),H38-8,"")</f>
         <v/>
       </c>
-      <c r="K38" s="200"/>
+      <c r="K38" s="172"/>
       <c r="L38" s="43"/>
       <c r="M38" s="44"/>
-      <c r="N38" s="166"/>
-      <c r="O38" s="167"/>
+      <c r="N38" s="184"/>
+      <c r="O38" s="185"/>
       <c r="P38" s="17"/>
     </row>
     <row r="39" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4497,10 +4503,10 @@
       <c r="M39" s="47" t="s">
         <v>29</v>
       </c>
-      <c r="N39" s="176" t="s">
+      <c r="N39" s="188" t="s">
         <v>29</v>
       </c>
-      <c r="O39" s="167"/>
+      <c r="O39" s="185"/>
       <c r="P39" s="17"/>
     </row>
     <row r="40" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -4839,17 +4845,17 @@
       <c r="P52" s="2"/>
     </row>
     <row r="53" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="172" t="s">
+      <c r="A53" s="189" t="s">
         <v>53</v>
       </c>
-      <c r="B53" s="173"/>
-      <c r="C53" s="167"/>
-      <c r="D53" s="167"/>
-      <c r="E53" s="167"/>
-      <c r="F53" s="167"/>
+      <c r="B53" s="190"/>
+      <c r="C53" s="185"/>
+      <c r="D53" s="185"/>
+      <c r="E53" s="185"/>
+      <c r="F53" s="185"/>
       <c r="G53" s="89"/>
-      <c r="H53" s="177"/>
-      <c r="I53" s="173"/>
+      <c r="H53" s="191"/>
+      <c r="I53" s="190"/>
       <c r="J53" s="140">
         <f>COUNTIF(C8:C38,"=D")</f>
         <v>0</v>
@@ -4871,14 +4877,14 @@
       <c r="P53" s="55"/>
     </row>
     <row r="54" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="172" t="s">
+      <c r="A54" s="189" t="s">
         <v>57</v>
       </c>
-      <c r="B54" s="173"/>
-      <c r="C54" s="167"/>
-      <c r="D54" s="167"/>
-      <c r="E54" s="167"/>
-      <c r="F54" s="167"/>
+      <c r="B54" s="190"/>
+      <c r="C54" s="185"/>
+      <c r="D54" s="185"/>
+      <c r="E54" s="185"/>
+      <c r="F54" s="185"/>
       <c r="G54" s="89"/>
       <c r="H54" s="90"/>
       <c r="I54" s="91"/>
@@ -4887,7 +4893,7 @@
         <v>0</v>
       </c>
       <c r="K54" s="144">
-        <f t="shared" ref="K54:K57" si="0">J54*8</f>
+        <f t="shared" ref="K54:K57" si="2">J54*8</f>
         <v>0</v>
       </c>
       <c r="L54" s="127"/>
@@ -4902,14 +4908,14 @@
       <c r="P54" s="55"/>
     </row>
     <row r="55" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="172" t="s">
+      <c r="A55" s="189" t="s">
         <v>59</v>
       </c>
-      <c r="B55" s="173"/>
-      <c r="C55" s="167"/>
-      <c r="D55" s="167"/>
-      <c r="E55" s="167"/>
-      <c r="F55" s="167"/>
+      <c r="B55" s="190"/>
+      <c r="C55" s="185"/>
+      <c r="D55" s="185"/>
+      <c r="E55" s="185"/>
+      <c r="F55" s="185"/>
       <c r="G55" s="89"/>
       <c r="H55" s="90"/>
       <c r="I55" s="91"/>
@@ -4918,7 +4924,7 @@
         <v>0</v>
       </c>
       <c r="K55" s="144">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L55" s="127"/>
@@ -4936,14 +4942,14 @@
       <c r="P55" s="55"/>
     </row>
     <row r="56" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="172" t="s">
+      <c r="A56" s="189" t="s">
         <v>61</v>
       </c>
-      <c r="B56" s="173"/>
-      <c r="C56" s="167"/>
-      <c r="D56" s="167"/>
-      <c r="E56" s="167"/>
-      <c r="F56" s="167"/>
+      <c r="B56" s="190"/>
+      <c r="C56" s="185"/>
+      <c r="D56" s="185"/>
+      <c r="E56" s="185"/>
+      <c r="F56" s="185"/>
       <c r="G56" s="89"/>
       <c r="H56" s="90"/>
       <c r="I56" s="91"/>
@@ -4952,7 +4958,7 @@
         <v>0</v>
       </c>
       <c r="K56" s="144">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L56" s="127"/>
@@ -4970,14 +4976,14 @@
       <c r="P56" s="55"/>
     </row>
     <row r="57" spans="1:16" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="172" t="s">
+      <c r="A57" s="189" t="s">
         <v>62</v>
       </c>
-      <c r="B57" s="173"/>
-      <c r="C57" s="167"/>
-      <c r="D57" s="167"/>
-      <c r="E57" s="167"/>
-      <c r="F57" s="167"/>
+      <c r="B57" s="190"/>
+      <c r="C57" s="185"/>
+      <c r="D57" s="185"/>
+      <c r="E57" s="185"/>
+      <c r="F57" s="185"/>
       <c r="G57" s="89"/>
       <c r="H57" s="90"/>
       <c r="I57" s="91"/>
@@ -4986,7 +4992,7 @@
         <v>0</v>
       </c>
       <c r="K57" s="144">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="L57" s="60"/>
@@ -4995,14 +5001,14 @@
       <c r="P57" s="2"/>
     </row>
     <row r="58" spans="1:16" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="174" t="s">
+      <c r="A58" s="192" t="s">
         <v>8</v>
       </c>
-      <c r="B58" s="175"/>
-      <c r="C58" s="175"/>
-      <c r="D58" s="175"/>
-      <c r="E58" s="175"/>
-      <c r="F58" s="175"/>
+      <c r="B58" s="193"/>
+      <c r="C58" s="193"/>
+      <c r="D58" s="193"/>
+      <c r="E58" s="193"/>
+      <c r="F58" s="193"/>
       <c r="G58" s="93"/>
       <c r="H58" s="93"/>
       <c r="I58" s="94" t="s">
@@ -5175,39 +5181,6 @@
     </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="B5:D6"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E5:G6"/>
-    <mergeCell ref="N9:O9"/>
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="N28:O28"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="A53:F53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="A54:F54"/>
-    <mergeCell ref="A55:F55"/>
-    <mergeCell ref="A56:F56"/>
-    <mergeCell ref="A57:F57"/>
-    <mergeCell ref="A58:F58"/>
     <mergeCell ref="L3:N3"/>
     <mergeCell ref="L2:M2"/>
     <mergeCell ref="A2:G2"/>
@@ -5224,6 +5197,39 @@
     <mergeCell ref="N35:O35"/>
     <mergeCell ref="N30:O30"/>
     <mergeCell ref="N31:O31"/>
+    <mergeCell ref="A54:F54"/>
+    <mergeCell ref="A55:F55"/>
+    <mergeCell ref="A56:F56"/>
+    <mergeCell ref="A57:F57"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="N38:O38"/>
+    <mergeCell ref="N39:O39"/>
+    <mergeCell ref="A53:F53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="N32:O32"/>
+    <mergeCell ref="N33:O33"/>
+    <mergeCell ref="N34:O34"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="N28:O28"/>
+    <mergeCell ref="N29:O29"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="E5:G6"/>
+    <mergeCell ref="N9:O9"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="B5:D6"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A3:D3"/>
   </mergeCells>
   <pageMargins left="0.59055100000000005" right="0.19685" top="0.59055100000000005" bottom="0" header="0.11811000000000001" footer="0.11811000000000001"/>
   <pageSetup scale="85" orientation="portrait"/>

</xml_diff>